<commit_message>
Add reviewed Richard product images 013-024
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Ra5391bf9ac9f4f31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R999c29b608144915"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -12610,9 +12610,11 @@
       <x:c r="K240" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L240" t="str"/>
+      <x:c r="L240" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000254-sp1-sash-painter.png</x:v>
+      </x:c>
       <x:c r="M240" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N240" t="str"/>
       <x:c r="O240" t="str"/>
@@ -12655,9 +12657,11 @@
       <x:c r="K241" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L241" t="str"/>
+      <x:c r="L241" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000255-rubber-sanding-block.png</x:v>
+      </x:c>
       <x:c r="M241" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N241" t="str"/>
       <x:c r="O241" t="str"/>
@@ -12700,9 +12704,11 @@
       <x:c r="K242" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L242" t="str"/>
+      <x:c r="L242" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000256-richard-wallpaper-smoother-605.png</x:v>
+      </x:c>
       <x:c r="M242" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N242" t="str"/>
       <x:c r="O242" t="str"/>
@@ -12745,9 +12751,11 @@
       <x:c r="K243" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L243" t="str"/>
+      <x:c r="L243" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000257-richard-utility-blades-u-1-b.png</x:v>
+      </x:c>
       <x:c r="M243" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N243" t="str"/>
       <x:c r="O243" t="str"/>
@@ -12790,9 +12798,11 @@
       <x:c r="K244" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L244" t="str"/>
+      <x:c r="L244" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000258-richard-18-stirwhip-mixer.png</x:v>
+      </x:c>
       <x:c r="M244" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N244" t="str"/>
       <x:c r="O244" t="str"/>
@@ -12835,9 +12845,11 @@
       <x:c r="K245" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L245" t="str"/>
+      <x:c r="L245" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000259-richard-hd-plastic-tray-liner-92068.png</x:v>
+      </x:c>
       <x:c r="M245" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N245" t="str"/>
       <x:c r="O245" t="str"/>
@@ -12880,9 +12892,11 @@
       <x:c r="K246" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L246" t="str"/>
+      <x:c r="L246" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000260-richard-hd-jumbo-plastic-tray.png</x:v>
+      </x:c>
       <x:c r="M246" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N246" t="str"/>
       <x:c r="O246" t="str"/>
@@ -12925,9 +12939,11 @@
       <x:c r="K247" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L247" t="str"/>
+      <x:c r="L247" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000261-richard-fat-boy-2-5-oval-angle-brush.png</x:v>
+      </x:c>
       <x:c r="M247" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N247" t="str"/>
       <x:c r="O247" t="str"/>
@@ -12970,9 +12986,11 @@
       <x:c r="K248" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L248" t="str"/>
+      <x:c r="L248" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000262-richard-ergo-grip-hand-sander-rub-18350.png</x:v>
+      </x:c>
       <x:c r="M248" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N248" t="str"/>
       <x:c r="O248" t="str"/>
@@ -13015,9 +13033,11 @@
       <x:c r="K249" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L249" t="str"/>
+      <x:c r="L249" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000263-richard-drywall-saw-ergo-grip-18828.png</x:v>
+      </x:c>
       <x:c r="M249" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N249" t="str"/>
       <x:c r="O249" t="str"/>
@@ -13060,9 +13080,11 @@
       <x:c r="K250" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L250" t="str"/>
+      <x:c r="L250" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000264-richard-drywall-patch-18204.png</x:v>
+      </x:c>
       <x:c r="M250" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N250" t="str"/>
       <x:c r="O250" t="str"/>
@@ -13105,9 +13127,11 @@
       <x:c r="K251" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L251" t="str"/>
+      <x:c r="L251" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000265-richard-aluminum-pole-sander-18393.png</x:v>
+      </x:c>
       <x:c r="M251" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N251" t="str"/>
       <x:c r="O251" t="str"/>

</xml_diff>

<commit_message>
Add reviewed Richard product images 025-036
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R999c29b608144915"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R0c6b81ace7ed4a6e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13221,9 +13221,11 @@
       <x:c r="K253" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L253" t="str"/>
+      <x:c r="L253" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000267-richard-ergo-grip-taping-knife.png</x:v>
+      </x:c>
       <x:c r="M253" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N253" t="str"/>
       <x:c r="O253" t="str"/>
@@ -13313,9 +13315,11 @@
       <x:c r="K255" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L255" t="str"/>
+      <x:c r="L255" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000269-richard-floor-scraper-blade-13304.png</x:v>
+      </x:c>
       <x:c r="M255" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N255" t="str"/>
       <x:c r="O255" t="str"/>
@@ -13358,9 +13362,11 @@
       <x:c r="K256" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L256" t="str"/>
+      <x:c r="L256" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000270-richard-rub-114-taping-knife.png</x:v>
+      </x:c>
       <x:c r="M256" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N256" t="str"/>
       <x:c r="O256" t="str"/>
@@ -13403,9 +13409,11 @@
       <x:c r="K257" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L257" t="str"/>
+      <x:c r="L257" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000271-richard-stainless-steel-putty-knife.png</x:v>
+      </x:c>
       <x:c r="M257" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N257" t="str"/>
       <x:c r="O257" t="str"/>
@@ -13448,9 +13456,11 @@
       <x:c r="K258" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L258" t="str"/>
+      <x:c r="L258" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000272-richard-goose-neck-brush-80833.png</x:v>
+      </x:c>
       <x:c r="M258" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N258" t="str"/>
       <x:c r="O258" t="str"/>
@@ -13493,9 +13503,11 @@
       <x:c r="K259" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L259" t="str"/>
+      <x:c r="L259" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000273-richard-ergo-grip-razor-scraper.png</x:v>
+      </x:c>
       <x:c r="M259" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N259" t="str"/>
       <x:c r="O259" t="str"/>
@@ -13538,9 +13550,11 @@
       <x:c r="K260" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L260" t="str"/>
+      <x:c r="L260" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000274-richard-plastic-pole-sander-18300.png</x:v>
+      </x:c>
       <x:c r="M260" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N260" t="str"/>
       <x:c r="O260" t="str"/>
@@ -13583,9 +13597,11 @@
       <x:c r="K261" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L261" t="str"/>
+      <x:c r="L261" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000275-richard-mini-wire-brush-03281.png</x:v>
+      </x:c>
       <x:c r="M261" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N261" t="str"/>
       <x:c r="O261" t="str"/>
@@ -13628,9 +13644,11 @@
       <x:c r="K262" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L262" t="str"/>
+      <x:c r="L262" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000276-richard-paint-pad-sp2.png</x:v>
+      </x:c>
       <x:c r="M262" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N262" t="str"/>
       <x:c r="O262" t="str"/>
@@ -13673,9 +13691,11 @@
       <x:c r="K263" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L263" t="str"/>
+      <x:c r="L263" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000277-richard-window-scraper-blades.png</x:v>
+      </x:c>
       <x:c r="M263" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N263" t="str"/>
       <x:c r="O263" t="str"/>
@@ -13718,9 +13738,11 @@
       <x:c r="K264" t="str">
         <x:v>ARICHAR</x:v>
       </x:c>
-      <x:c r="L264" t="str"/>
+      <x:c r="L264" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000278-richard-rw-10-ab-drywall-knife.png</x:v>
+      </x:c>
       <x:c r="M264" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N264" t="str"/>
       <x:c r="O264" t="str"/>
@@ -13763,9 +13785,11 @@
       <x:c r="K265" t="str">
         <x:v>ADV01-S</x:v>
       </x:c>
-      <x:c r="L265" t="str"/>
+      <x:c r="L265" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AE-000000279-advance-seam-buster-51101.png</x:v>
+      </x:c>
       <x:c r="M265" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N265" t="str"/>
       <x:c r="O265" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 037-048
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R0c6b81ace7ed4a6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R6d5fc5497252491a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13832,9 +13832,11 @@
       <x:c r="K266" t="str">
         <x:v>ADV01-S</x:v>
       </x:c>
-      <x:c r="L266" t="str"/>
+      <x:c r="L266" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AE-000000280-advance-quicktruss-q300-door-painting-stands.png</x:v>
+      </x:c>
       <x:c r="M266" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N266" t="str"/>
       <x:c r="O266" t="str"/>
@@ -13877,9 +13879,11 @@
       <x:c r="K267" t="str">
         <x:v>ADV01-S</x:v>
       </x:c>
-      <x:c r="L267" t="str"/>
+      <x:c r="L267" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AE-000000281-advance-684-stainless-steel-seam-roller.png</x:v>
+      </x:c>
       <x:c r="M267" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N267" t="str"/>
       <x:c r="O267" t="str"/>
@@ -13922,9 +13926,11 @@
       <x:c r="K268" t="str">
         <x:v>ADV01-S</x:v>
       </x:c>
-      <x:c r="L268" t="str"/>
+      <x:c r="L268" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AE-000000282-advance-695-plastic-oval-seam-roller.png</x:v>
+      </x:c>
       <x:c r="M268" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N268" t="str"/>
       <x:c r="O268" t="str"/>
@@ -13967,9 +13973,11 @@
       <x:c r="K269" t="str">
         <x:v>ADV01-S</x:v>
       </x:c>
-      <x:c r="L269" t="str"/>
+      <x:c r="L269" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AE-000000283-advance-694-plastic-flat-seam-roller.png</x:v>
+      </x:c>
       <x:c r="M269" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N269" t="str"/>
       <x:c r="O269" t="str"/>
@@ -14020,9 +14028,11 @@
       <x:c r="K270" t="str">
         <x:v>ANC01</x:v>
       </x:c>
-      <x:c r="L270" t="str"/>
+      <x:c r="L270" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ANC-000000284-floor-guard-400-sq-ft.png</x:v>
+      </x:c>
       <x:c r="M270" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N270" t="str"/>
       <x:c r="O270" t="str"/>
@@ -14065,9 +14075,11 @@
       <x:c r="K271" t="str">
         <x:v>ANC01</x:v>
       </x:c>
-      <x:c r="L271" t="str"/>
+      <x:c r="L271" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ANC-000000285-anchored-rubberized-floor-paper.png</x:v>
+      </x:c>
       <x:c r="M271" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N271" t="str"/>
       <x:c r="O271" t="str"/>
@@ -14110,9 +14122,11 @@
       <x:c r="K272" t="str">
         <x:v>ANC01</x:v>
       </x:c>
-      <x:c r="L272" t="str"/>
+      <x:c r="L272" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ANC-000000286-anchored-coated-paper-700-sq-ft.png</x:v>
+      </x:c>
       <x:c r="M272" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N272" t="str"/>
       <x:c r="O272" t="str"/>
@@ -14155,9 +14169,11 @@
       <x:c r="K273" t="str">
         <x:v>ATRIUM</x:v>
       </x:c>
-      <x:c r="L273" t="str"/>
+      <x:c r="L273" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ATR-000000287-everbuild-wonder-wipes-100.png</x:v>
+      </x:c>
       <x:c r="M273" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N273" t="str"/>
       <x:c r="O273" t="str"/>
@@ -14200,9 +14216,11 @@
       <x:c r="K274" t="str">
         <x:v>ATRIUM</x:v>
       </x:c>
-      <x:c r="L274" t="str"/>
+      <x:c r="L274" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ATR-000000288-everbuild-mitre-fast-bonding-kit.png</x:v>
+      </x:c>
       <x:c r="M274" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N274" t="str"/>
       <x:c r="O274" t="str"/>
@@ -14245,9 +14263,11 @@
       <x:c r="K275" t="str">
         <x:v>ATRIUM</x:v>
       </x:c>
-      <x:c r="L275" t="str"/>
+      <x:c r="L275" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ATR-000000289-everbuild-mammoth-double-sided-tape-25mm-x-2-5m.png</x:v>
+      </x:c>
       <x:c r="M275" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N275" t="str"/>
       <x:c r="O275" t="str"/>
@@ -14290,9 +14310,11 @@
       <x:c r="K276" t="str">
         <x:v>MOO01</x:v>
       </x:c>
-      <x:c r="L276" t="str"/>
+      <x:c r="L276" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/I-000000290-insl-x-fire-retardant-flat-white.png</x:v>
+      </x:c>
       <x:c r="M276" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N276" t="str"/>
       <x:c r="O276" t="str"/>
@@ -14335,9 +14357,11 @@
       <x:c r="K277" t="str">
         <x:v>MOO01</x:v>
       </x:c>
-      <x:c r="L277" t="str"/>
+      <x:c r="L277" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BM-000000291-benjamin-moore-hp1560-epoxy-floor-sealer.png</x:v>
+      </x:c>
       <x:c r="M277" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N277" t="str"/>
       <x:c r="O277" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 049-060
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R6d5fc5497252491a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R49f7e416a4c54234"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14404,9 +14404,11 @@
       <x:c r="K278" t="str">
         <x:v>MOO01</x:v>
       </x:c>
-      <x:c r="L278" t="str"/>
+      <x:c r="L278" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BM-000000292-benjamin-moore-hp2210-alkyd-urethane.png</x:v>
+      </x:c>
       <x:c r="M278" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N278" t="str">
         <x:v>Finishes</x:v>
@@ -14457,9 +14459,11 @@
       <x:c r="K279" t="str">
         <x:v>MOO01</x:v>
       </x:c>
-      <x:c r="L279" t="str"/>
+      <x:c r="L279" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BM-000000293-benjamin-moore-hp2300-quick-dry-alkyd-enamel.png</x:v>
+      </x:c>
       <x:c r="M279" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N279" t="str"/>
       <x:c r="O279" t="str"/>
@@ -14502,9 +14506,11 @@
       <x:c r="K280" t="str">
         <x:v>MOO01</x:v>
       </x:c>
-      <x:c r="L280" t="str"/>
+      <x:c r="L280" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BM-000000294-benjamin-moore-hp2400-rapid-dry-alkyd-enamel.png</x:v>
+      </x:c>
       <x:c r="M280" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N280" t="str"/>
       <x:c r="O280" t="str"/>
@@ -14547,9 +14553,11 @@
       <x:c r="K281" t="str">
         <x:v>MOO01</x:v>
       </x:c>
-      <x:c r="L281" t="str"/>
+      <x:c r="L281" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BM-000000295-benjamin-moore-hp4400-waterborne-epoxy.png</x:v>
+      </x:c>
       <x:c r="M281" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N281" t="str"/>
       <x:c r="O281" t="str"/>
@@ -14827,9 +14835,11 @@
       <x:c r="K287" t="str">
         <x:v>MOO01</x:v>
       </x:c>
-      <x:c r="L287" t="str"/>
+      <x:c r="L287" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BM-000000301-benjamin-moore-latex-dry-fall-flat.png</x:v>
+      </x:c>
       <x:c r="M287" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N287" t="str"/>
       <x:c r="O287" t="str"/>
@@ -14872,9 +14882,11 @@
       <x:c r="K288" t="str">
         <x:v>MOO01</x:v>
       </x:c>
-      <x:c r="L288" t="str"/>
+      <x:c r="L288" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BM-000000302-benjamin-moore-paint-extender-518.png</x:v>
+      </x:c>
       <x:c r="M288" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N288" t="str"/>
       <x:c r="O288" t="str"/>
@@ -14917,9 +14929,11 @@
       <x:c r="K289" t="str">
         <x:v>MOO01</x:v>
       </x:c>
-      <x:c r="L289" t="str"/>
+      <x:c r="L289" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/I-000000303-insl-x-sure-step-anti-slip-knight-gray.png</x:v>
+      </x:c>
       <x:c r="M289" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N289" t="str"/>
       <x:c r="O289" t="str"/>
@@ -15009,9 +15023,11 @@
       <x:c r="K291" t="str">
         <x:v>MOO01</x:v>
       </x:c>
-      <x:c r="L291" t="str"/>
+      <x:c r="L291" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/I-000000305-insl-x-latex-traffic-marking-paint-white.png</x:v>
+      </x:c>
       <x:c r="M291" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N291" t="str"/>
       <x:c r="O291" t="str"/>
@@ -15101,9 +15117,11 @@
       <x:c r="K293" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L293" t="str"/>
+      <x:c r="L293" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000307-bennett-white-taklon-short-flat-3-4.png</x:v>
+      </x:c>
       <x:c r="M293" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N293" t="str"/>
       <x:c r="O293" t="str"/>
@@ -15146,9 +15164,11 @@
       <x:c r="K294" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L294" t="str"/>
+      <x:c r="L294" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000308-bennett-white-taklon-round-3-pack.png</x:v>
+      </x:c>
       <x:c r="M294" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N294" t="str"/>
       <x:c r="O294" t="str"/>
@@ -15191,9 +15211,11 @@
       <x:c r="K295" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L295" t="str"/>
+      <x:c r="L295" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000309-bennett-tray-liner-tpl-4.png</x:v>
+      </x:c>
       <x:c r="M295" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N295" t="str"/>
       <x:c r="O295" t="str"/>
@@ -15236,9 +15258,11 @@
       <x:c r="K296" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L296" t="str"/>
+      <x:c r="L296" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000310-bennett-flat-professional-artist-brushes-3-pack.png</x:v>
+      </x:c>
       <x:c r="M296" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N296" t="str"/>
       <x:c r="O296" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 061-072
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R49f7e416a4c54234"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rc31bad770c5243fe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15305,9 +15305,11 @@
       <x:c r="K297" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L297" t="str"/>
+      <x:c r="L297" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000311-bennett-perfection-2-5-soft-latex-brush.png</x:v>
+      </x:c>
       <x:c r="M297" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N297" t="str"/>
       <x:c r="O297" t="str"/>
@@ -15350,9 +15352,11 @@
       <x:c r="K298" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L298" t="str"/>
+      <x:c r="L298" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000312-bennett-7-inch-replacement-pad.png</x:v>
+      </x:c>
       <x:c r="M298" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N298" t="str"/>
       <x:c r="O298" t="str"/>
@@ -15395,9 +15399,11 @@
       <x:c r="K299" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L299" t="str"/>
+      <x:c r="L299" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000313-bennett-aluminum-pole-sander-head.png</x:v>
+      </x:c>
       <x:c r="M299" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N299" t="str"/>
       <x:c r="O299" t="str"/>
@@ -15440,9 +15446,11 @@
       <x:c r="K300" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L300" t="str"/>
+      <x:c r="L300" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000314-bennett-foam-corner-roller.png</x:v>
+      </x:c>
       <x:c r="M300" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N300" t="str"/>
       <x:c r="O300" t="str"/>
@@ -15485,9 +15493,11 @@
       <x:c r="K301" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L301" t="str"/>
+      <x:c r="L301" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000310-bennett-flat-professional-artist-brushes-3-pack.png</x:v>
+      </x:c>
       <x:c r="M301" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N301" t="str"/>
       <x:c r="O301" t="str"/>
@@ -15530,9 +15540,11 @@
       <x:c r="K302" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L302" t="str"/>
+      <x:c r="L302" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000316-bennett-dualon-blue-stripe-10-inch-roller.png</x:v>
+      </x:c>
       <x:c r="M302" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N302" t="str"/>
       <x:c r="O302" t="str"/>
@@ -15575,9 +15587,11 @@
       <x:c r="K303" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L303" t="str"/>
+      <x:c r="L303" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000317-bennett-lint-free-cheese-cloth.png</x:v>
+      </x:c>
       <x:c r="M303" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N303" t="str"/>
       <x:c r="O303" t="str"/>
@@ -15620,9 +15634,11 @@
       <x:c r="K304" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L304" t="str"/>
+      <x:c r="L304" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CAN-000000318-allpro-canvas-drop-cloth.png</x:v>
+      </x:c>
       <x:c r="M304" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N304" t="str"/>
       <x:c r="O304" t="str"/>
@@ -15673,9 +15689,11 @@
       <x:c r="K305" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L305" t="str"/>
+      <x:c r="L305" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000319-linzer-a555-artist-brush-set.png</x:v>
+      </x:c>
       <x:c r="M305" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N305" t="str"/>
       <x:c r="O305" t="str"/>
@@ -15718,9 +15736,11 @@
       <x:c r="K306" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L306" t="str"/>
+      <x:c r="L306" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000320-bennett-small-paint-tray-liner.png</x:v>
+      </x:c>
       <x:c r="M306" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N306" t="str"/>
       <x:c r="O306" t="str"/>
@@ -15763,9 +15783,11 @@
       <x:c r="K307" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L307" t="str"/>
+      <x:c r="L307" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000321-bennett-small-paint-tray.png</x:v>
+      </x:c>
       <x:c r="M307" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N307" t="str"/>
       <x:c r="O307" t="str"/>
@@ -15808,9 +15830,11 @@
       <x:c r="K308" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L308" t="str"/>
+      <x:c r="L308" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000322-bennett-xxl-plastic-tray-liner.png</x:v>
+      </x:c>
       <x:c r="M308" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N308" t="str"/>
       <x:c r="O308" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 073-084
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rc31bad770c5243fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rc4a3a86d19cb4f9d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11937,7 +11937,7 @@
         <x:v>3MC01</x:v>
       </x:c>
       <x:c r="L226" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/3M-000000240-3m-super77-spray-adhesive.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/3M-000000240-3m-super77-spray-adhesive.png?raw=true</x:v>
       </x:c>
       <x:c r="M226" t="str">
         <x:v>Image Added</x:v>
@@ -12031,7 +12031,7 @@
         <x:v>3MC01</x:v>
       </x:c>
       <x:c r="L228" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/3M-000000242-3m-scotch-brite-general-purpose-hand-pad-7447.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/3M-000000242-3m-scotch-brite-general-purpose-hand-pad-7447.png?raw=true</x:v>
       </x:c>
       <x:c r="M228" t="str">
         <x:v>Image Added</x:v>
@@ -12086,7 +12086,7 @@
         <x:v>3MC01</x:v>
       </x:c>
       <x:c r="L229" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/3M-000000243-3m-replacement-lens-covers-v2.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/3M-000000243-3m-replacement-lens-covers-v2.png?raw=true</x:v>
       </x:c>
       <x:c r="M229" t="str">
         <x:v>Image Added</x:v>
@@ -12133,7 +12133,7 @@
         <x:v>3MC01</x:v>
       </x:c>
       <x:c r="L230" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/3M-000000244-3m-new-safe-release-blue-3m-canad.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/3M-000000244-3m-new-safe-release-blue-3m-canad.png?raw=true</x:v>
       </x:c>
       <x:c r="M230" t="str">
         <x:v>Images for Review</x:v>
@@ -12235,7 +12235,7 @@
         <x:v>3MC01</x:v>
       </x:c>
       <x:c r="L232" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/3M-000000246-3m-filter-p100-v2.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/3M-000000246-3m-filter-p100-v2.png?raw=true</x:v>
       </x:c>
       <x:c r="M232" t="str">
         <x:v>Images for Review</x:v>
@@ -12282,7 +12282,7 @@
         <x:v>3MC01</x:v>
       </x:c>
       <x:c r="L233" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/3M-000000247-3m-blue-long-mask-v2.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/3M-000000247-3m-blue-long-mask-v2.png?raw=true</x:v>
       </x:c>
       <x:c r="M233" t="str">
         <x:v>Images for Review</x:v>
@@ -12329,7 +12329,7 @@
         <x:v>3MC01</x:v>
       </x:c>
       <x:c r="L234" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/3M-000000248-3m-hand-masker-12-film-blade.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/3M-000000248-3m-hand-masker-12-film-blade.png?raw=true</x:v>
       </x:c>
       <x:c r="M234" t="str">
         <x:v>Image Added</x:v>
@@ -12376,7 +12376,7 @@
         <x:v>3MC01</x:v>
       </x:c>
       <x:c r="L235" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/3M-000000249-3m-cutoff-blade.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/3M-000000249-3m-cutoff-blade.png?raw=true</x:v>
       </x:c>
       <x:c r="M235" t="str">
         <x:v>Images for Review</x:v>
@@ -12423,7 +12423,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L236" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000250-w-10-wood-scraper.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000250-w-10-wood-scraper.png?raw=true</x:v>
       </x:c>
       <x:c r="M236" t="str">
         <x:v>Image Added</x:v>
@@ -12470,7 +12470,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L237" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000251-w-1-3-4-blade.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000251-w-1-3-4-blade.png?raw=true</x:v>
       </x:c>
       <x:c r="M237" t="str">
         <x:v>Images for Review</x:v>
@@ -12517,7 +12517,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L238" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000252-u-s-10-richard-lever-bar.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000252-u-s-10-richard-lever-bar.png?raw=true</x:v>
       </x:c>
       <x:c r="M238" t="str">
         <x:v>Image Added</x:v>
@@ -12564,7 +12564,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L239" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000253-sp2-sash-painter.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000253-sp2-sash-painter.png?raw=true</x:v>
       </x:c>
       <x:c r="M239" t="str">
         <x:v>Images for Review</x:v>
@@ -12611,7 +12611,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L240" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000254-sp1-sash-painter.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000254-sp1-sash-painter.png?raw=true</x:v>
       </x:c>
       <x:c r="M240" t="str">
         <x:v>Image Added</x:v>
@@ -12658,7 +12658,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L241" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000255-rubber-sanding-block.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000255-rubber-sanding-block.png?raw=true</x:v>
       </x:c>
       <x:c r="M241" t="str">
         <x:v>Image Added</x:v>
@@ -12705,7 +12705,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L242" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000256-richard-wallpaper-smoother-605.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000256-richard-wallpaper-smoother-605.png?raw=true</x:v>
       </x:c>
       <x:c r="M242" t="str">
         <x:v>Images for Review</x:v>
@@ -12752,7 +12752,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L243" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000257-richard-utility-blades-u-1-b.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000257-richard-utility-blades-u-1-b.png?raw=true</x:v>
       </x:c>
       <x:c r="M243" t="str">
         <x:v>Image Added</x:v>
@@ -12799,7 +12799,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L244" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000258-richard-18-stirwhip-mixer.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000258-richard-18-stirwhip-mixer.png?raw=true</x:v>
       </x:c>
       <x:c r="M244" t="str">
         <x:v>Image Added</x:v>
@@ -12846,7 +12846,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L245" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000259-richard-hd-plastic-tray-liner-92068.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000259-richard-hd-plastic-tray-liner-92068.png?raw=true</x:v>
       </x:c>
       <x:c r="M245" t="str">
         <x:v>Image Added</x:v>
@@ -12893,7 +12893,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L246" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000260-richard-hd-jumbo-plastic-tray.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000260-richard-hd-jumbo-plastic-tray.png?raw=true</x:v>
       </x:c>
       <x:c r="M246" t="str">
         <x:v>Image Added</x:v>
@@ -12940,7 +12940,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L247" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000261-richard-fat-boy-2-5-oval-angle-brush.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000261-richard-fat-boy-2-5-oval-angle-brush.png?raw=true</x:v>
       </x:c>
       <x:c r="M247" t="str">
         <x:v>Image Added</x:v>
@@ -12987,7 +12987,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L248" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000262-richard-ergo-grip-hand-sander-rub-18350.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000262-richard-ergo-grip-hand-sander-rub-18350.png?raw=true</x:v>
       </x:c>
       <x:c r="M248" t="str">
         <x:v>Image Added</x:v>
@@ -13034,7 +13034,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L249" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000263-richard-drywall-saw-ergo-grip-18828.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000263-richard-drywall-saw-ergo-grip-18828.png?raw=true</x:v>
       </x:c>
       <x:c r="M249" t="str">
         <x:v>Image Added</x:v>
@@ -13081,7 +13081,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L250" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000264-richard-drywall-patch-18204.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000264-richard-drywall-patch-18204.png?raw=true</x:v>
       </x:c>
       <x:c r="M250" t="str">
         <x:v>Image Added</x:v>
@@ -13128,7 +13128,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L251" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000265-richard-aluminum-pole-sander-18393.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000265-richard-aluminum-pole-sander-18393.png?raw=true</x:v>
       </x:c>
       <x:c r="M251" t="str">
         <x:v>Images for Review</x:v>
@@ -13222,7 +13222,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L253" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000267-richard-ergo-grip-taping-knife.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000267-richard-ergo-grip-taping-knife.png?raw=true</x:v>
       </x:c>
       <x:c r="M253" t="str">
         <x:v>Images for Review</x:v>
@@ -13316,7 +13316,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L255" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000269-richard-floor-scraper-blade-13304.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000269-richard-floor-scraper-blade-13304.png?raw=true</x:v>
       </x:c>
       <x:c r="M255" t="str">
         <x:v>Images for Review</x:v>
@@ -13363,7 +13363,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L256" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000270-richard-rub-114-taping-knife.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000270-richard-rub-114-taping-knife.png?raw=true</x:v>
       </x:c>
       <x:c r="M256" t="str">
         <x:v>Image Added</x:v>
@@ -13410,7 +13410,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L257" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000271-richard-stainless-steel-putty-knife.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000271-richard-stainless-steel-putty-knife.png?raw=true</x:v>
       </x:c>
       <x:c r="M257" t="str">
         <x:v>Images for Review</x:v>
@@ -13457,7 +13457,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L258" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000272-richard-goose-neck-brush-80833.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000272-richard-goose-neck-brush-80833.png?raw=true</x:v>
       </x:c>
       <x:c r="M258" t="str">
         <x:v>Image Added</x:v>
@@ -13504,7 +13504,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L259" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000273-richard-ergo-grip-razor-scraper.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000273-richard-ergo-grip-razor-scraper.png?raw=true</x:v>
       </x:c>
       <x:c r="M259" t="str">
         <x:v>Images for Review</x:v>
@@ -13551,7 +13551,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L260" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000274-richard-plastic-pole-sander-18300.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000274-richard-plastic-pole-sander-18300.png?raw=true</x:v>
       </x:c>
       <x:c r="M260" t="str">
         <x:v>Image Added</x:v>
@@ -13598,7 +13598,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L261" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000275-richard-mini-wire-brush-03281.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000275-richard-mini-wire-brush-03281.png?raw=true</x:v>
       </x:c>
       <x:c r="M261" t="str">
         <x:v>Images for Review</x:v>
@@ -13645,7 +13645,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L262" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000276-richard-paint-pad-sp2.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000276-richard-paint-pad-sp2.png?raw=true</x:v>
       </x:c>
       <x:c r="M262" t="str">
         <x:v>Image Added</x:v>
@@ -13692,7 +13692,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L263" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000277-richard-window-scraper-blades.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000277-richard-window-scraper-blades.png?raw=true</x:v>
       </x:c>
       <x:c r="M263" t="str">
         <x:v>Images for Review</x:v>
@@ -13739,7 +13739,7 @@
         <x:v>ARICHAR</x:v>
       </x:c>
       <x:c r="L264" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000278-richard-rw-10-ab-drywall-knife.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RIC-000000278-richard-rw-10-ab-drywall-knife.png?raw=true</x:v>
       </x:c>
       <x:c r="M264" t="str">
         <x:v>Image Added</x:v>
@@ -13786,7 +13786,7 @@
         <x:v>ADV01-S</x:v>
       </x:c>
       <x:c r="L265" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AE-000000279-advance-seam-buster-51101.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AE-000000279-advance-seam-buster-51101.png?raw=true</x:v>
       </x:c>
       <x:c r="M265" t="str">
         <x:v>Image Added</x:v>
@@ -13833,7 +13833,7 @@
         <x:v>ADV01-S</x:v>
       </x:c>
       <x:c r="L266" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AE-000000280-advance-quicktruss-q300-door-painting-stands.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AE-000000280-advance-quicktruss-q300-door-painting-stands.png?raw=true</x:v>
       </x:c>
       <x:c r="M266" t="str">
         <x:v>Image Added</x:v>
@@ -13880,7 +13880,7 @@
         <x:v>ADV01-S</x:v>
       </x:c>
       <x:c r="L267" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AE-000000281-advance-684-stainless-steel-seam-roller.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AE-000000281-advance-684-stainless-steel-seam-roller.png?raw=true</x:v>
       </x:c>
       <x:c r="M267" t="str">
         <x:v>Image Added</x:v>
@@ -13927,7 +13927,7 @@
         <x:v>ADV01-S</x:v>
       </x:c>
       <x:c r="L268" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AE-000000282-advance-695-plastic-oval-seam-roller.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AE-000000282-advance-695-plastic-oval-seam-roller.png?raw=true</x:v>
       </x:c>
       <x:c r="M268" t="str">
         <x:v>Image Added</x:v>
@@ -13974,7 +13974,7 @@
         <x:v>ADV01-S</x:v>
       </x:c>
       <x:c r="L269" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AE-000000283-advance-694-plastic-flat-seam-roller.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AE-000000283-advance-694-plastic-flat-seam-roller.png?raw=true</x:v>
       </x:c>
       <x:c r="M269" t="str">
         <x:v>Image Added</x:v>
@@ -14029,7 +14029,7 @@
         <x:v>ANC01</x:v>
       </x:c>
       <x:c r="L270" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ANC-000000284-floor-guard-400-sq-ft.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ANC-000000284-floor-guard-400-sq-ft.png?raw=true</x:v>
       </x:c>
       <x:c r="M270" t="str">
         <x:v>Image Added</x:v>
@@ -14076,7 +14076,7 @@
         <x:v>ANC01</x:v>
       </x:c>
       <x:c r="L271" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ANC-000000285-anchored-rubberized-floor-paper.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ANC-000000285-anchored-rubberized-floor-paper.png?raw=true</x:v>
       </x:c>
       <x:c r="M271" t="str">
         <x:v>Images for Review</x:v>
@@ -14123,7 +14123,7 @@
         <x:v>ANC01</x:v>
       </x:c>
       <x:c r="L272" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ANC-000000286-anchored-coated-paper-700-sq-ft.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ANC-000000286-anchored-coated-paper-700-sq-ft.png?raw=true</x:v>
       </x:c>
       <x:c r="M272" t="str">
         <x:v>Images for Review</x:v>
@@ -14170,7 +14170,7 @@
         <x:v>ATRIUM</x:v>
       </x:c>
       <x:c r="L273" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ATR-000000287-everbuild-wonder-wipes-100.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ATR-000000287-everbuild-wonder-wipes-100.png?raw=true</x:v>
       </x:c>
       <x:c r="M273" t="str">
         <x:v>Image Added</x:v>
@@ -14217,7 +14217,7 @@
         <x:v>ATRIUM</x:v>
       </x:c>
       <x:c r="L274" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ATR-000000288-everbuild-mitre-fast-bonding-kit.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ATR-000000288-everbuild-mitre-fast-bonding-kit.png?raw=true</x:v>
       </x:c>
       <x:c r="M274" t="str">
         <x:v>Images for Review</x:v>
@@ -14264,7 +14264,7 @@
         <x:v>ATRIUM</x:v>
       </x:c>
       <x:c r="L275" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ATR-000000289-everbuild-mammoth-double-sided-tape-25mm-x-2-5m.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ATR-000000289-everbuild-mammoth-double-sided-tape-25mm-x-2-5m.png?raw=true</x:v>
       </x:c>
       <x:c r="M275" t="str">
         <x:v>Images for Review</x:v>
@@ -14311,7 +14311,7 @@
         <x:v>MOO01</x:v>
       </x:c>
       <x:c r="L276" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/I-000000290-insl-x-fire-retardant-flat-white.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/I-000000290-insl-x-fire-retardant-flat-white.png?raw=true</x:v>
       </x:c>
       <x:c r="M276" t="str">
         <x:v>Image Added</x:v>
@@ -14358,7 +14358,7 @@
         <x:v>MOO01</x:v>
       </x:c>
       <x:c r="L277" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BM-000000291-benjamin-moore-hp1560-epoxy-floor-sealer.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BM-000000291-benjamin-moore-hp1560-epoxy-floor-sealer.png?raw=true</x:v>
       </x:c>
       <x:c r="M277" t="str">
         <x:v>Image Added</x:v>
@@ -14405,7 +14405,7 @@
         <x:v>MOO01</x:v>
       </x:c>
       <x:c r="L278" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BM-000000292-benjamin-moore-hp2210-alkyd-urethane.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BM-000000292-benjamin-moore-hp2210-alkyd-urethane.png?raw=true</x:v>
       </x:c>
       <x:c r="M278" t="str">
         <x:v>Images for Review</x:v>
@@ -14460,7 +14460,7 @@
         <x:v>MOO01</x:v>
       </x:c>
       <x:c r="L279" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BM-000000293-benjamin-moore-hp2300-quick-dry-alkyd-enamel.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BM-000000293-benjamin-moore-hp2300-quick-dry-alkyd-enamel.png?raw=true</x:v>
       </x:c>
       <x:c r="M279" t="str">
         <x:v>Image Added</x:v>
@@ -14507,7 +14507,7 @@
         <x:v>MOO01</x:v>
       </x:c>
       <x:c r="L280" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BM-000000294-benjamin-moore-hp2400-rapid-dry-alkyd-enamel.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BM-000000294-benjamin-moore-hp2400-rapid-dry-alkyd-enamel.png?raw=true</x:v>
       </x:c>
       <x:c r="M280" t="str">
         <x:v>Image Added</x:v>
@@ -14554,7 +14554,7 @@
         <x:v>MOO01</x:v>
       </x:c>
       <x:c r="L281" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BM-000000295-benjamin-moore-hp4400-waterborne-epoxy.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BM-000000295-benjamin-moore-hp4400-waterborne-epoxy.png?raw=true</x:v>
       </x:c>
       <x:c r="M281" t="str">
         <x:v>Images for Review</x:v>
@@ -14836,7 +14836,7 @@
         <x:v>MOO01</x:v>
       </x:c>
       <x:c r="L287" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BM-000000301-benjamin-moore-latex-dry-fall-flat.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BM-000000301-benjamin-moore-latex-dry-fall-flat.png?raw=true</x:v>
       </x:c>
       <x:c r="M287" t="str">
         <x:v>Images for Review</x:v>
@@ -14883,7 +14883,7 @@
         <x:v>MOO01</x:v>
       </x:c>
       <x:c r="L288" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BM-000000302-benjamin-moore-paint-extender-518.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BM-000000302-benjamin-moore-paint-extender-518.png?raw=true</x:v>
       </x:c>
       <x:c r="M288" t="str">
         <x:v>Image Added</x:v>
@@ -14930,7 +14930,7 @@
         <x:v>MOO01</x:v>
       </x:c>
       <x:c r="L289" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/I-000000303-insl-x-sure-step-anti-slip-knight-gray.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/I-000000303-insl-x-sure-step-anti-slip-knight-gray.png?raw=true</x:v>
       </x:c>
       <x:c r="M289" t="str">
         <x:v>Images for Review</x:v>
@@ -15024,7 +15024,7 @@
         <x:v>MOO01</x:v>
       </x:c>
       <x:c r="L291" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/I-000000305-insl-x-latex-traffic-marking-paint-white.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/I-000000305-insl-x-latex-traffic-marking-paint-white.png?raw=true</x:v>
       </x:c>
       <x:c r="M291" t="str">
         <x:v>Images for Review</x:v>
@@ -15118,7 +15118,7 @@
         <x:v>BEN01-S</x:v>
       </x:c>
       <x:c r="L293" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000307-bennett-white-taklon-short-flat-3-4.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000307-bennett-white-taklon-short-flat-3-4.png?raw=true</x:v>
       </x:c>
       <x:c r="M293" t="str">
         <x:v>Images for Review</x:v>
@@ -15165,7 +15165,7 @@
         <x:v>BEN01-S</x:v>
       </x:c>
       <x:c r="L294" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000308-bennett-white-taklon-round-3-pack.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000308-bennett-white-taklon-round-3-pack.png?raw=true</x:v>
       </x:c>
       <x:c r="M294" t="str">
         <x:v>Images for Review</x:v>
@@ -15212,7 +15212,7 @@
         <x:v>BEN01-S</x:v>
       </x:c>
       <x:c r="L295" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000309-bennett-tray-liner-tpl-4.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000309-bennett-tray-liner-tpl-4.png?raw=true</x:v>
       </x:c>
       <x:c r="M295" t="str">
         <x:v>Images for Review</x:v>
@@ -15259,7 +15259,7 @@
         <x:v>BEN01-S</x:v>
       </x:c>
       <x:c r="L296" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000310-bennett-flat-professional-artist-brushes-3-pack.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000310-bennett-flat-professional-artist-brushes-3-pack.png?raw=true</x:v>
       </x:c>
       <x:c r="M296" t="str">
         <x:v>Images for Review</x:v>
@@ -15306,7 +15306,7 @@
         <x:v>BEN01-S</x:v>
       </x:c>
       <x:c r="L297" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000311-bennett-perfection-2-5-soft-latex-brush.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000311-bennett-perfection-2-5-soft-latex-brush.png?raw=true</x:v>
       </x:c>
       <x:c r="M297" t="str">
         <x:v>Image Added</x:v>
@@ -15353,7 +15353,7 @@
         <x:v>BEN01-S</x:v>
       </x:c>
       <x:c r="L298" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000312-bennett-7-inch-replacement-pad.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000312-bennett-7-inch-replacement-pad.png?raw=true</x:v>
       </x:c>
       <x:c r="M298" t="str">
         <x:v>Images for Review</x:v>
@@ -15400,7 +15400,7 @@
         <x:v>BEN01-S</x:v>
       </x:c>
       <x:c r="L299" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000313-bennett-aluminum-pole-sander-head.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000313-bennett-aluminum-pole-sander-head.png?raw=true</x:v>
       </x:c>
       <x:c r="M299" t="str">
         <x:v>Image Added</x:v>
@@ -15447,7 +15447,7 @@
         <x:v>BEN01-S</x:v>
       </x:c>
       <x:c r="L300" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000314-bennett-foam-corner-roller.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000314-bennett-foam-corner-roller.png?raw=true</x:v>
       </x:c>
       <x:c r="M300" t="str">
         <x:v>Image Added</x:v>
@@ -15494,7 +15494,7 @@
         <x:v>BEN01-S</x:v>
       </x:c>
       <x:c r="L301" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000310-bennett-flat-professional-artist-brushes-3-pack.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000310-bennett-flat-professional-artist-brushes-3-pack.png?raw=true</x:v>
       </x:c>
       <x:c r="M301" t="str">
         <x:v>Images for Review</x:v>
@@ -15541,7 +15541,7 @@
         <x:v>BEN01-S</x:v>
       </x:c>
       <x:c r="L302" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000316-bennett-dualon-blue-stripe-10-inch-roller.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000316-bennett-dualon-blue-stripe-10-inch-roller.png?raw=true</x:v>
       </x:c>
       <x:c r="M302" t="str">
         <x:v>Images for Review</x:v>
@@ -15588,7 +15588,7 @@
         <x:v>BEN01-S</x:v>
       </x:c>
       <x:c r="L303" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000317-bennett-lint-free-cheese-cloth.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000317-bennett-lint-free-cheese-cloth.png?raw=true</x:v>
       </x:c>
       <x:c r="M303" t="str">
         <x:v>Images for Review</x:v>
@@ -15635,7 +15635,7 @@
         <x:v>BEN01-S</x:v>
       </x:c>
       <x:c r="L304" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CAN-000000318-allpro-canvas-drop-cloth.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CAN-000000318-allpro-canvas-drop-cloth.png?raw=true</x:v>
       </x:c>
       <x:c r="M304" t="str">
         <x:v>Images for Review</x:v>
@@ -15690,7 +15690,7 @@
         <x:v>BEN01-S</x:v>
       </x:c>
       <x:c r="L305" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000319-linzer-a555-artist-brush-set.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000319-linzer-a555-artist-brush-set.png?raw=true</x:v>
       </x:c>
       <x:c r="M305" t="str">
         <x:v>Images for Review</x:v>
@@ -15737,7 +15737,7 @@
         <x:v>BEN01-S</x:v>
       </x:c>
       <x:c r="L306" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000320-bennett-small-paint-tray-liner.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000320-bennett-small-paint-tray-liner.png?raw=true</x:v>
       </x:c>
       <x:c r="M306" t="str">
         <x:v>Images for Review</x:v>
@@ -15784,7 +15784,7 @@
         <x:v>BEN01-S</x:v>
       </x:c>
       <x:c r="L307" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000321-bennett-small-paint-tray.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000321-bennett-small-paint-tray.png?raw=true</x:v>
       </x:c>
       <x:c r="M307" t="str">
         <x:v>Images for Review</x:v>
@@ -15831,7 +15831,7 @@
         <x:v>BEN01-S</x:v>
       </x:c>
       <x:c r="L308" t="str">
-        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000322-bennett-xxl-plastic-tray-liner.png</x:v>
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000322-bennett-xxl-plastic-tray-liner.png?raw=true</x:v>
       </x:c>
       <x:c r="M308" t="str">
         <x:v>Image Added</x:v>
@@ -15877,9 +15877,11 @@
       <x:c r="K309" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L309" t="str"/>
+      <x:c r="L309" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000310-bennett-flat-professional-artist-brushes-3-pack.png?raw=true</x:v>
+      </x:c>
       <x:c r="M309" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N309" t="str"/>
       <x:c r="O309" t="str"/>
@@ -15922,9 +15924,11 @@
       <x:c r="K310" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L310" t="str"/>
+      <x:c r="L310" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000324-bennett-micropro-15mm-10-pack.png?raw=true</x:v>
+      </x:c>
       <x:c r="M310" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N310" t="str"/>
       <x:c r="O310" t="str"/>
@@ -15975,9 +15979,11 @@
       <x:c r="K311" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L311" t="str"/>
+      <x:c r="L311" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000325-bennett-tpl-8-tray-liner.png?raw=true</x:v>
+      </x:c>
       <x:c r="M311" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N311" t="str"/>
       <x:c r="O311" t="str"/>
@@ -16020,9 +16026,11 @@
       <x:c r="K312" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L312" t="str"/>
+      <x:c r="L312" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000326-bennett-large-natural-sea-sponge.png?raw=true</x:v>
+      </x:c>
       <x:c r="M312" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N312" t="str"/>
       <x:c r="O312" t="str"/>
@@ -16065,9 +16073,11 @@
       <x:c r="K313" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L313" t="str"/>
+      <x:c r="L313" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000327-bennett-jumbo-xl-plastic-tray.png?raw=true</x:v>
+      </x:c>
       <x:c r="M313" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N313" t="str"/>
       <x:c r="O313" t="str"/>
@@ -16110,9 +16120,11 @@
       <x:c r="K314" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L314" t="str"/>
+      <x:c r="L314" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000328-bennett-one-gallon-metal-paint-grid.png?raw=true</x:v>
+      </x:c>
       <x:c r="M314" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N314" t="str"/>
       <x:c r="O314" t="str"/>
@@ -16155,9 +16167,11 @@
       <x:c r="K315" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L315" t="str"/>
+      <x:c r="L315" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000329-bennett-coveralls-large.png?raw=true</x:v>
+      </x:c>
       <x:c r="M315" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N315" t="str"/>
       <x:c r="O315" t="str"/>
@@ -16200,9 +16214,11 @@
       <x:c r="K316" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L316" t="str"/>
+      <x:c r="L316" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000330-bennett-mini-brass-wire-brush.png?raw=true</x:v>
+      </x:c>
       <x:c r="M316" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N316" t="str"/>
       <x:c r="O316" t="str"/>
@@ -16245,9 +16261,11 @@
       <x:c r="K317" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L317" t="str"/>
+      <x:c r="L317" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000331-bennett-mini-red-tray.png?raw=true</x:v>
+      </x:c>
       <x:c r="M317" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N317" t="str"/>
       <x:c r="O317" t="str"/>
@@ -16290,9 +16308,11 @@
       <x:c r="K318" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L318" t="str"/>
+      <x:c r="L318" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000332-bennett-pro-glas-fiberglass-pole.png?raw=true</x:v>
+      </x:c>
       <x:c r="M318" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N318" t="str"/>
       <x:c r="O318" t="str"/>
@@ -16343,9 +16363,11 @@
       <x:c r="K319" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L319" t="str"/>
+      <x:c r="L319" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000333-bennett-7-inch-pad-painter.png?raw=true</x:v>
+      </x:c>
       <x:c r="M319" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N319" t="str"/>
       <x:c r="O319" t="str"/>
@@ -16388,9 +16410,11 @@
       <x:c r="K320" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L320" t="str"/>
+      <x:c r="L320" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000334-bennett-twist-fiberglass-pole-6-12.png?raw=true</x:v>
+      </x:c>
       <x:c r="M320" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N320" t="str"/>
       <x:c r="O320" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 085-096
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rc4a3a86d19cb4f9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rc79e830997ba454b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16465,9 +16465,11 @@
       <x:c r="K321" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L321" t="str"/>
+      <x:c r="L321" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000335-bennett-t8-red-paint-tray-v2.png?raw=true</x:v>
+      </x:c>
       <x:c r="M321" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N321" t="str"/>
       <x:c r="O321" t="str"/>
@@ -16510,9 +16512,11 @@
       <x:c r="K322" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L322" t="str"/>
+      <x:c r="L322" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000336-bennett-c60-3-pure-bristle-brush.png?raw=true</x:v>
+      </x:c>
       <x:c r="M322" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N322" t="str"/>
       <x:c r="O322" t="str"/>
@@ -16555,9 +16559,11 @@
       <x:c r="K323" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L323" t="str"/>
+      <x:c r="L323" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000337-bennett-micropro-5-piece-tray-set.png?raw=true</x:v>
+      </x:c>
       <x:c r="M323" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N323" t="str"/>
       <x:c r="O323" t="str"/>
@@ -16600,9 +16606,11 @@
       <x:c r="K324" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L324" t="str"/>
+      <x:c r="L324" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000338-bennett-micropro-13mm-roller-3-pack.png?raw=true</x:v>
+      </x:c>
       <x:c r="M324" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N324" t="str"/>
       <x:c r="O324" t="str"/>
@@ -16645,9 +16653,11 @@
       <x:c r="K325" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L325" t="str"/>
+      <x:c r="L325" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000339-bennett-high-density-foam-refills-10-pack.png?raw=true</x:v>
+      </x:c>
       <x:c r="M325" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N325" t="str"/>
       <x:c r="O325" t="str"/>
@@ -16690,9 +16700,11 @@
       <x:c r="K326" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L326" t="str"/>
+      <x:c r="L326" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000340-bennett-foam-brushes-10-pack.png?raw=true</x:v>
+      </x:c>
       <x:c r="M326" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N326" t="str"/>
       <x:c r="O326" t="str"/>
@@ -16735,9 +16747,11 @@
       <x:c r="K327" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L327" t="str"/>
+      <x:c r="L327" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000341-bennett-4x12-cotton-drop-cloth.png?raw=true</x:v>
+      </x:c>
       <x:c r="M327" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N327" t="str"/>
       <x:c r="O327" t="str"/>
@@ -16780,9 +16794,11 @@
       <x:c r="K328" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L328" t="str"/>
+      <x:c r="L328" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000342-bennett-mix60-drill-mixer.png?raw=true</x:v>
+      </x:c>
       <x:c r="M328" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N328" t="str"/>
       <x:c r="O328" t="str"/>
@@ -16833,9 +16849,11 @@
       <x:c r="K329" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L329" t="str"/>
+      <x:c r="L329" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000343-bennett-mini-roller-frame.png?raw=true</x:v>
+      </x:c>
       <x:c r="M329" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N329" t="str"/>
       <x:c r="O329" t="str"/>
@@ -16925,9 +16943,11 @@
       <x:c r="K331" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L331" t="str"/>
+      <x:c r="L331" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000345-bennett-five-wire-roller-cage.png?raw=true</x:v>
+      </x:c>
       <x:c r="M331" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N331" t="str"/>
       <x:c r="O331" t="str"/>
@@ -16970,9 +16990,11 @@
       <x:c r="K332" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L332" t="str"/>
+      <x:c r="L332" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000346-bennett-8x12-medium-plastic-drop-sheet.png?raw=true</x:v>
+      </x:c>
       <x:c r="M332" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N332" t="str"/>
       <x:c r="O332" t="str"/>
@@ -17015,9 +17037,11 @@
       <x:c r="K333" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L333" t="str"/>
+      <x:c r="L333" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000336-bennett-c60-3-pure-bristle-brush.png?raw=true</x:v>
+      </x:c>
       <x:c r="M333" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N333" t="str"/>
       <x:c r="O333" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 097-108
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rc79e830997ba454b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R52dfc2bcb14c44d3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17131,9 +17131,11 @@
       <x:c r="K335" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L335" t="str"/>
+      <x:c r="L335" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000349-bennett-red-bee-3-inch-brush.png?raw=true</x:v>
+      </x:c>
       <x:c r="M335" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N335" t="str"/>
       <x:c r="O335" t="str"/>
@@ -17176,9 +17178,11 @@
       <x:c r="K336" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L336" t="str"/>
+      <x:c r="L336" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000339-bennett-high-density-foam-refills-10-pack.png?raw=true</x:v>
+      </x:c>
       <x:c r="M336" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N336" t="str"/>
       <x:c r="O336" t="str"/>
@@ -17221,9 +17225,11 @@
       <x:c r="K337" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L337" t="str"/>
+      <x:c r="L337" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000351-bennett-lf-240hp-lint-free-tray-set.png?raw=true</x:v>
+      </x:c>
       <x:c r="M337" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N337" t="str"/>
       <x:c r="O337" t="str"/>
@@ -17266,9 +17272,11 @@
       <x:c r="K338" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L338" t="str"/>
+      <x:c r="L338" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000352-bennett-lint-free-10mm-roller-cover.png?raw=true</x:v>
+      </x:c>
       <x:c r="M338" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N338" t="str"/>
       <x:c r="O338" t="str"/>
@@ -17311,9 +17319,11 @@
       <x:c r="K339" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L339" t="str"/>
+      <x:c r="L339" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000353-bennett-angular-white-taklon-brush-set.png?raw=true</x:v>
+      </x:c>
       <x:c r="M339" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N339" t="str"/>
       <x:c r="O339" t="str"/>
@@ -17356,9 +17366,11 @@
       <x:c r="K340" t="str">
         <x:v>BEN01-S</x:v>
       </x:c>
-      <x:c r="L340" t="str"/>
+      <x:c r="L340" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/BEN-000000354-bennett-high-density-foam-brush.png?raw=true</x:v>
+      </x:c>
       <x:c r="M340" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N340" t="str"/>
       <x:c r="O340" t="str"/>
@@ -17401,9 +17413,11 @@
       <x:c r="K341" t="str">
         <x:v>CANLAK</x:v>
       </x:c>
-      <x:c r="L341" t="str"/>
+      <x:c r="L341" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CAN-000000355-absco-red-x-pro-red-blocker.png?raw=true</x:v>
+      </x:c>
       <x:c r="M341" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N341" t="str"/>
       <x:c r="O341" t="str"/>
@@ -17446,9 +17460,11 @@
       <x:c r="K342" t="str">
         <x:v>CANLAK</x:v>
       </x:c>
-      <x:c r="L342" t="str"/>
+      <x:c r="L342" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CAN-000000358-canlak-industrial-pail.png?raw=true</x:v>
+      </x:c>
       <x:c r="M342" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N342" t="str"/>
       <x:c r="O342" t="str"/>
@@ -17491,9 +17507,11 @@
       <x:c r="K343" t="str">
         <x:v>CANLAK</x:v>
       </x:c>
-      <x:c r="L343" t="str"/>
+      <x:c r="L343" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CAN-000000358-canlak-industrial-pail.png?raw=true</x:v>
+      </x:c>
       <x:c r="M343" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N343" t="str"/>
       <x:c r="O343" t="str"/>
@@ -17536,9 +17554,11 @@
       <x:c r="K344" t="str">
         <x:v>CANLAK</x:v>
       </x:c>
-      <x:c r="L344" t="str"/>
+      <x:c r="L344" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CAN-000000358-canlak-industrial-pail.png?raw=true</x:v>
+      </x:c>
       <x:c r="M344" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N344" t="str"/>
       <x:c r="O344" t="str"/>
@@ -17581,9 +17601,11 @@
       <x:c r="K345" t="str">
         <x:v>CANLAK</x:v>
       </x:c>
-      <x:c r="L345" t="str"/>
+      <x:c r="L345" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CAN-000000358-canlak-industrial-pail.png?raw=true</x:v>
+      </x:c>
       <x:c r="M345" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N345" t="str"/>
       <x:c r="O345" t="str"/>
@@ -17626,9 +17648,11 @@
       <x:c r="K346" t="str">
         <x:v>CANLAK</x:v>
       </x:c>
-      <x:c r="L346" t="str"/>
+      <x:c r="L346" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CAN-000000358-canlak-industrial-pail.png?raw=true</x:v>
+      </x:c>
       <x:c r="M346" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N346" t="str"/>
       <x:c r="O346" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 109-120
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R52dfc2bcb14c44d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rbf5679cd85ce4608"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17695,9 +17695,11 @@
       <x:c r="K347" t="str">
         <x:v>CANLAK</x:v>
       </x:c>
-      <x:c r="L347" t="str"/>
+      <x:c r="L347" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CAN-000000358-canlak-industrial-pail.png?raw=true</x:v>
+      </x:c>
       <x:c r="M347" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N347" t="str"/>
       <x:c r="O347" t="str"/>
@@ -17740,9 +17742,11 @@
       <x:c r="K348" t="str">
         <x:v>CANLAK</x:v>
       </x:c>
-      <x:c r="L348" t="str"/>
+      <x:c r="L348" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CAN-000000358-canlak-industrial-pail.png?raw=true</x:v>
+      </x:c>
       <x:c r="M348" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N348" t="str"/>
       <x:c r="O348" t="str"/>
@@ -17785,9 +17789,11 @@
       <x:c r="K349" t="str">
         <x:v>CANLAK</x:v>
       </x:c>
-      <x:c r="L349" t="str"/>
+      <x:c r="L349" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CAN-000000358-canlak-industrial-pail.png?raw=true</x:v>
+      </x:c>
       <x:c r="M349" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N349" t="str"/>
       <x:c r="O349" t="str"/>
@@ -17830,9 +17836,11 @@
       <x:c r="K350" t="str">
         <x:v>CHAPIN</x:v>
       </x:c>
-      <x:c r="L350" t="str"/>
+      <x:c r="L350" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CHA-000000364-chapin-19049-xtreme-concrete-sprayer.png?raw=true</x:v>
+      </x:c>
       <x:c r="M350" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N350" t="str"/>
       <x:c r="O350" t="str"/>
@@ -17875,9 +17883,11 @@
       <x:c r="K351" t="str">
         <x:v>CHAPIN</x:v>
       </x:c>
-      <x:c r="L351" t="str"/>
+      <x:c r="L351" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AP-000000365-allpro-48oz-wallpaper-sprayer.png?raw=true</x:v>
+      </x:c>
       <x:c r="M351" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N351" t="str"/>
       <x:c r="O351" t="str"/>
@@ -17920,9 +17930,11 @@
       <x:c r="K352" t="str">
         <x:v>COR02-S</x:v>
       </x:c>
-      <x:c r="L352" t="str"/>
+      <x:c r="L352" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/COR-000000366-corona-ultraweave-9-inch-half-inch-nap.png?raw=true</x:v>
+      </x:c>
       <x:c r="M352" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N352" t="str"/>
       <x:c r="O352" t="str"/>
@@ -17973,9 +17985,11 @@
       <x:c r="K353" t="str">
         <x:v>COR02-S</x:v>
       </x:c>
-      <x:c r="L353" t="str"/>
+      <x:c r="L353" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/COR-000000367-corona-ultrafast-9-inch-half-inch-nap.png?raw=true</x:v>
+      </x:c>
       <x:c r="M353" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N353" t="str"/>
       <x:c r="O353" t="str"/>
@@ -18018,9 +18032,11 @@
       <x:c r="K354" t="str">
         <x:v>COR02-S</x:v>
       </x:c>
-      <x:c r="L354" t="str"/>
+      <x:c r="L354" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/COR-000000368-corona-glasskoter-mohair-roller-cover.png?raw=true</x:v>
+      </x:c>
       <x:c r="M354" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N354" t="str"/>
       <x:c r="O354" t="str"/>
@@ -18063,9 +18079,11 @@
       <x:c r="K355" t="str">
         <x:v>COR02-S</x:v>
       </x:c>
-      <x:c r="L355" t="str"/>
+      <x:c r="L355" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/COR-000000369-corona-cortez-2-5-inch-angle-brush.png?raw=true</x:v>
+      </x:c>
       <x:c r="M355" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N355" t="str"/>
       <x:c r="O355" t="str"/>
@@ -18108,9 +18126,11 @@
       <x:c r="K356" t="str">
         <x:v>COR02-S</x:v>
       </x:c>
-      <x:c r="L356" t="str"/>
+      <x:c r="L356" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/COR-000000370-corona-shelby-2-5-inch-angle-brush.png?raw=true</x:v>
+      </x:c>
       <x:c r="M356" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N356" t="str"/>
       <x:c r="O356" t="str"/>
@@ -18153,9 +18173,11 @@
       <x:c r="K357" t="str">
         <x:v>COR02-S</x:v>
       </x:c>
-      <x:c r="L357" t="str"/>
+      <x:c r="L357" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/COR-000000371-corona-excalibur-3-inch-chinex-brush.png?raw=true</x:v>
+      </x:c>
       <x:c r="M357" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N357" t="str"/>
       <x:c r="O357" t="str"/>
@@ -18198,9 +18220,11 @@
       <x:c r="K358" t="str">
         <x:v>COR02-S</x:v>
       </x:c>
-      <x:c r="L358" t="str"/>
+      <x:c r="L358" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/COR-000000372-corona-ryan-2-5-inch-chinex-brush.png?raw=true</x:v>
+      </x:c>
       <x:c r="M358" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N358" t="str"/>
       <x:c r="O358" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 121-132
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rbf5679cd85ce4608"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R5ee3f593e99f41da"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18267,9 +18267,11 @@
       <x:c r="K359" t="str">
         <x:v>COR02-S</x:v>
       </x:c>
-      <x:c r="L359" t="str"/>
+      <x:c r="L359" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/COR-000000373-corona-vegas-2-5-inch-brush.png?raw=true</x:v>
+      </x:c>
       <x:c r="M359" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N359" t="str"/>
       <x:c r="O359" t="str"/>
@@ -18312,9 +18314,11 @@
       <x:c r="K360" t="str">
         <x:v>COR02-S</x:v>
       </x:c>
-      <x:c r="L360" t="str"/>
+      <x:c r="L360" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/COR-000000374-corona-sabre-2-5-inch-angle-brush.png?raw=true</x:v>
+      </x:c>
       <x:c r="M360" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N360" t="str"/>
       <x:c r="O360" t="str"/>
@@ -18357,9 +18361,11 @@
       <x:c r="K361" t="str">
         <x:v>COR02-S</x:v>
       </x:c>
-      <x:c r="L361" t="str"/>
+      <x:c r="L361" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/COR-000000375-corona-classic-smoother-12-inch.png?raw=true</x:v>
+      </x:c>
       <x:c r="M361" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N361" t="str"/>
       <x:c r="O361" t="str"/>
@@ -18402,9 +18408,11 @@
       <x:c r="K362" t="str">
         <x:v>CUTEK</x:v>
       </x:c>
-      <x:c r="L362" t="str"/>
+      <x:c r="L362" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CUT-000000376-cutek-extreme-3-6l.png?raw=true</x:v>
+      </x:c>
       <x:c r="M362" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N362" t="str"/>
       <x:c r="O362" t="str"/>
@@ -18447,9 +18455,11 @@
       <x:c r="K363" t="str">
         <x:v>DAP</x:v>
       </x:c>
-      <x:c r="L363" t="str"/>
+      <x:c r="L363" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DAP-000000377-dynaflex-230-50-year-white-caulk.png?raw=true</x:v>
+      </x:c>
       <x:c r="M363" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N363" t="str"/>
       <x:c r="O363" t="str"/>
@@ -18539,9 +18549,11 @@
       <x:c r="K365" t="str">
         <x:v>DAP</x:v>
       </x:c>
-      <x:c r="L365" t="str"/>
+      <x:c r="L365" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DAP-000000379-100-percent-silicone-white-caulk.png?raw=true</x:v>
+      </x:c>
       <x:c r="M365" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N365" t="str"/>
       <x:c r="O365" t="str"/>
@@ -18584,9 +18596,11 @@
       <x:c r="K366" t="str">
         <x:v>DAP</x:v>
       </x:c>
-      <x:c r="L366" t="str"/>
+      <x:c r="L366" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DAP-000000380-premium-wood-filler-16oz.png?raw=true</x:v>
+      </x:c>
       <x:c r="M366" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N366" t="str"/>
       <x:c r="O366" t="str"/>
@@ -18629,9 +18643,11 @@
       <x:c r="K367" t="str">
         <x:v>DAP</x:v>
       </x:c>
-      <x:c r="L367" t="str"/>
+      <x:c r="L367" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DAP-000000381-platinum-patch-946ml.png?raw=true</x:v>
+      </x:c>
       <x:c r="M367" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N367" t="str"/>
       <x:c r="O367" t="str"/>
@@ -18682,9 +18698,11 @@
       <x:c r="K368" t="str">
         <x:v>DAP</x:v>
       </x:c>
-      <x:c r="L368" t="str"/>
+      <x:c r="L368" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DAP-000000382-natural-woodpro-wood-filler-85g.png?raw=true</x:v>
+      </x:c>
       <x:c r="M368" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N368" t="str"/>
       <x:c r="O368" t="str"/>
@@ -18774,9 +18792,11 @@
       <x:c r="K370" t="str">
         <x:v>DAP</x:v>
       </x:c>
-      <x:c r="L370" t="str"/>
+      <x:c r="L370" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DAP-000000384-kwik-seal-white-5-5oz.png?raw=true</x:v>
+      </x:c>
       <x:c r="M370" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N370" t="str"/>
       <x:c r="O370" t="str"/>
@@ -18819,9 +18839,11 @@
       <x:c r="K371" t="str">
         <x:v>DAP</x:v>
       </x:c>
-      <x:c r="L371" t="str"/>
+      <x:c r="L371" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DAP-000000385-fast-n-final-16oz.png?raw=true</x:v>
+      </x:c>
       <x:c r="M371" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N371" t="str"/>
       <x:c r="O371" t="str"/>
@@ -18864,9 +18886,11 @@
       <x:c r="K372" t="str">
         <x:v>DAP</x:v>
       </x:c>
-      <x:c r="L372" t="str"/>
+      <x:c r="L372" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DAP-000000386-fast-dry-premium-spackling-32oz.png?raw=true</x:v>
+      </x:c>
       <x:c r="M372" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N372" t="str"/>
       <x:c r="O372" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 133-144
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R5ee3f593e99f41da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R6b9e0b9005a74861"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18933,9 +18933,11 @@
       <x:c r="K373" t="str">
         <x:v>DAP</x:v>
       </x:c>
-      <x:c r="L373" t="str"/>
+      <x:c r="L373" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DAP-000000387-alex-flex-spackling-473ml.png?raw=true</x:v>
+      </x:c>
       <x:c r="M373" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N373" t="str"/>
       <x:c r="O373" t="str"/>
@@ -19025,9 +19027,11 @@
       <x:c r="K375" t="str">
         <x:v>DAP</x:v>
       </x:c>
-      <x:c r="L375" t="str"/>
+      <x:c r="L375" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DAP-000000389-alex-fast-dry-white-162ml-squeeze-tube.png?raw=true</x:v>
+      </x:c>
       <x:c r="M375" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N375" t="str"/>
       <x:c r="O375" t="str"/>
@@ -19164,9 +19168,11 @@
       <x:c r="K378" t="str">
         <x:v>DAP</x:v>
       </x:c>
-      <x:c r="L378" t="str"/>
+      <x:c r="L378" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DAP-000000392-dap-33-glazing-half-pint.png?raw=true</x:v>
+      </x:c>
       <x:c r="M378" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N378" t="str"/>
       <x:c r="O378" t="str"/>
@@ -19217,9 +19223,11 @@
       <x:c r="K379" t="str">
         <x:v>DAP</x:v>
       </x:c>
-      <x:c r="L379" t="str"/>
+      <x:c r="L379" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DAP-000000393-plaster-of-paris-25lb-bag.png?raw=true</x:v>
+      </x:c>
       <x:c r="M379" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N379" t="str"/>
       <x:c r="O379" t="str"/>
@@ -19262,9 +19270,11 @@
       <x:c r="K380" t="str">
         <x:v>DECOZI</x:v>
       </x:c>
-      <x:c r="L380" t="str"/>
+      <x:c r="L380" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DEC-000000394-decozi-window-film-dso-02.png?raw=true</x:v>
+      </x:c>
       <x:c r="M380" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N380" t="str"/>
       <x:c r="O380" t="str"/>
@@ -19315,9 +19325,11 @@
       <x:c r="K381" t="str">
         <x:v>DEG01</x:v>
       </x:c>
-      <x:c r="L381" t="str"/>
+      <x:c r="L381" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DEG-000000395-degil-full-body-harness-lanyard-kit.png?raw=true</x:v>
+      </x:c>
       <x:c r="M381" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N381" t="str"/>
       <x:c r="O381" t="str"/>
@@ -19360,9 +19372,11 @@
       <x:c r="K382" t="str">
         <x:v>DEG01</x:v>
       </x:c>
-      <x:c r="L382" t="str"/>
+      <x:c r="L382" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DEG-000000396-degil-type-1-white-hard-hat.png?raw=true</x:v>
+      </x:c>
       <x:c r="M382" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N382" t="str"/>
       <x:c r="O382" t="str"/>
@@ -19405,9 +19419,11 @@
       <x:c r="K383" t="str">
         <x:v>DENTEC</x:v>
       </x:c>
-      <x:c r="L383" t="str"/>
+      <x:c r="L383" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DEN-000000397-dentec-citation-932-gray-safety-glasses.png?raw=true</x:v>
+      </x:c>
       <x:c r="M383" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N383" t="str"/>
       <x:c r="O383" t="str"/>
@@ -19450,9 +19466,11 @@
       <x:c r="K384" t="str">
         <x:v>DICKIES</x:v>
       </x:c>
-      <x:c r="L384" t="str"/>
+      <x:c r="L384" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DIC-000000398-dickies-white-painters-bib-overalls.png?raw=true</x:v>
+      </x:c>
       <x:c r="M384" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N384" t="str"/>
       <x:c r="O384" t="str"/>
@@ -19495,9 +19513,11 @@
       <x:c r="K385" t="str">
         <x:v>DICKIES</x:v>
       </x:c>
-      <x:c r="L385" t="str"/>
+      <x:c r="L385" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DIC-000000399-dickies-white-painter-shorts.png?raw=true</x:v>
+      </x:c>
       <x:c r="M385" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N385" t="str"/>
       <x:c r="O385" t="str"/>
@@ -19540,9 +19560,11 @@
       <x:c r="K386" t="str">
         <x:v>DICKIES</x:v>
       </x:c>
-      <x:c r="L386" t="str"/>
+      <x:c r="L386" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DIC-000000400-dickies-white-painter-pants-32x30.png?raw=true</x:v>
+      </x:c>
       <x:c r="M386" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N386" t="str"/>
       <x:c r="O386" t="str"/>
@@ -19585,9 +19607,11 @@
       <x:c r="K387" t="str">
         <x:v>DOVER</x:v>
       </x:c>
-      <x:c r="L387" t="str"/>
+      <x:c r="L387" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TS-000000401-trade-secret-furniture-polish-cleaner-236ml.png?raw=true</x:v>
+      </x:c>
       <x:c r="M387" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N387" t="str"/>
       <x:c r="O387" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 145-156
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R6b9e0b9005a74861"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R91986e47d6f14504"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19654,9 +19654,11 @@
       <x:c r="K388" t="str">
         <x:v>DOVER</x:v>
       </x:c>
-      <x:c r="L388" t="str"/>
+      <x:c r="L388" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TRA-000000402-tracsafe-anti-slip-sealer-3-78l.png?raw=true</x:v>
+      </x:c>
       <x:c r="M388" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N388" t="str"/>
       <x:c r="O388" t="str"/>
@@ -19699,9 +19701,11 @@
       <x:c r="K389" t="str">
         <x:v>DOVER</x:v>
       </x:c>
-      <x:c r="L389" t="str"/>
+      <x:c r="L389" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DOV-000000403-dover-pump-touch-up-marker-set.png?raw=true</x:v>
+      </x:c>
       <x:c r="M389" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N389" t="str"/>
       <x:c r="O389" t="str"/>
@@ -19744,9 +19748,11 @@
       <x:c r="K390" t="str">
         <x:v>DOVER</x:v>
       </x:c>
-      <x:c r="L390" t="str"/>
+      <x:c r="L390" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TER-000000404-terrazzo-silverado-3-gallon.png?raw=true</x:v>
+      </x:c>
       <x:c r="M390" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N390" t="str"/>
       <x:c r="O390" t="str"/>
@@ -19789,9 +19795,11 @@
       <x:c r="K391" t="str">
         <x:v>DOVER</x:v>
       </x:c>
-      <x:c r="L391" t="str"/>
+      <x:c r="L391" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TS-000000405-trade-secret-scratch-remover-dark-236ml.png?raw=true</x:v>
+      </x:c>
       <x:c r="M391" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N391" t="str">
         <x:v>Finishes</x:v>
@@ -19842,9 +19850,11 @@
       <x:c r="K392" t="str">
         <x:v>DOVER</x:v>
       </x:c>
-      <x:c r="L392" t="str"/>
+      <x:c r="L392" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/HOW-000000406-howard-wax-it-all-9oz.png?raw=true</x:v>
+      </x:c>
       <x:c r="M392" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N392" t="str"/>
       <x:c r="O392" t="str"/>
@@ -19887,9 +19897,11 @@
       <x:c r="K393" t="str">
         <x:v>DOVER</x:v>
       </x:c>
-      <x:c r="L393" t="str"/>
+      <x:c r="L393" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PC-000000407-dover-classic-fill-sticks.png?raw=true</x:v>
+      </x:c>
       <x:c r="M393" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N393" t="str"/>
       <x:c r="O393" t="str"/>
@@ -19932,9 +19944,11 @@
       <x:c r="K394" t="str">
         <x:v>DOVER</x:v>
       </x:c>
-      <x:c r="L394" t="str"/>
+      <x:c r="L394" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DOV-000000408-the-caulking-finger-front.png?raw=true</x:v>
+      </x:c>
       <x:c r="M394" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N394" t="str"/>
       <x:c r="O394" t="str"/>
@@ -19977,9 +19991,11 @@
       <x:c r="K395" t="str">
         <x:v>DOVER</x:v>
       </x:c>
-      <x:c r="L395" t="str"/>
+      <x:c r="L395" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DOV-000000409-dover-pump-touch-up-marker-white-review.png?raw=true</x:v>
+      </x:c>
       <x:c r="M395" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N395" t="str"/>
       <x:c r="O395" t="str"/>
@@ -20022,9 +20038,11 @@
       <x:c r="K396" t="str">
         <x:v>DOVER</x:v>
       </x:c>
-      <x:c r="L396" t="str"/>
+      <x:c r="L396" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DOV-000000410-dover-fill-your-own-empty-marker.png?raw=true</x:v>
+      </x:c>
       <x:c r="M396" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N396" t="str"/>
       <x:c r="O396" t="str"/>
@@ -20067,9 +20085,11 @@
       <x:c r="K397" t="str">
         <x:v>DOVER</x:v>
       </x:c>
-      <x:c r="L397" t="str"/>
+      <x:c r="L397" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DOV-000000411-dover-pro-finish-toner-walnut-family.png?raw=true</x:v>
+      </x:c>
       <x:c r="M397" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N397" t="str"/>
       <x:c r="O397" t="str"/>
@@ -20112,9 +20132,11 @@
       <x:c r="K398" t="str">
         <x:v>DOVER</x:v>
       </x:c>
-      <x:c r="L398" t="str"/>
+      <x:c r="L398" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DOV-000000412-dover-pro-finish-opaque-white-family.png?raw=true</x:v>
+      </x:c>
       <x:c r="M398" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N398" t="str"/>
       <x:c r="O398" t="str"/>
@@ -20157,9 +20179,11 @@
       <x:c r="K399" t="str">
         <x:v>DOVER</x:v>
       </x:c>
-      <x:c r="L399" t="str"/>
+      <x:c r="L399" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DOV-000000413-dover-pro-finish-clear-satin-family.png?raw=true</x:v>
+      </x:c>
       <x:c r="M399" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N399" t="str"/>
       <x:c r="O399" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 157-168
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R91986e47d6f14504"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rd2d1bbccd6534f2e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20226,9 +20226,11 @@
       <x:c r="K400" t="str">
         <x:v>DOVER</x:v>
       </x:c>
-      <x:c r="L400" t="str"/>
+      <x:c r="L400" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DOV-000000414-dover-pro-finish-blush-stopper-family.png?raw=true</x:v>
+      </x:c>
       <x:c r="M400" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N400" t="str"/>
       <x:c r="O400" t="str"/>
@@ -20271,9 +20273,11 @@
       <x:c r="K401" t="str">
         <x:v>DOVER</x:v>
       </x:c>
-      <x:c r="L401" t="str"/>
+      <x:c r="L401" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SKR-000000415-skrapr-and-skrapr-jr.png?raw=true</x:v>
+      </x:c>
       <x:c r="M401" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N401" t="str"/>
       <x:c r="O401" t="str"/>
@@ -20316,9 +20320,11 @@
       <x:c r="K402" t="str">
         <x:v>CANPRO</x:v>
       </x:c>
-      <x:c r="L402" t="str"/>
+      <x:c r="L402" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AP-000000416-allpro-gold-pro-3000-caulk-gun.png?raw=true</x:v>
+      </x:c>
       <x:c r="M402" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N402" t="str"/>
       <x:c r="O402" t="str"/>
@@ -20361,9 +20367,11 @@
       <x:c r="K403" t="str">
         <x:v>CANPRO</x:v>
       </x:c>
-      <x:c r="L403" t="str"/>
+      <x:c r="L403" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AP-000000417-allpro-gold-pro-2000-caulk-gun.png?raw=true</x:v>
+      </x:c>
       <x:c r="M403" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N403" t="str"/>
       <x:c r="O403" t="str"/>
@@ -20406,9 +20414,11 @@
       <x:c r="K404" t="str">
         <x:v>CANPRO</x:v>
       </x:c>
-      <x:c r="L404" t="str"/>
+      <x:c r="L404" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AP-000000418-allpro-100c-consumer-caulk-gun.png?raw=true</x:v>
+      </x:c>
       <x:c r="M404" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N404" t="str"/>
       <x:c r="O404" t="str"/>
@@ -20451,9 +20461,11 @@
       <x:c r="K405" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L405" t="str"/>
+      <x:c r="L405" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DU-000000419-dumond-watch-dog-wipe-out-8402.png?raw=true</x:v>
+      </x:c>
       <x:c r="M405" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N405" t="str"/>
       <x:c r="O405" t="str"/>
@@ -20496,9 +20508,11 @@
       <x:c r="K406" t="str">
         <x:v>BHF01</x:v>
       </x:c>
-      <x:c r="L406" t="str"/>
+      <x:c r="L406" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DUR-000000420-duraseal-quick-coat-rosewood-quart.png?raw=true</x:v>
+      </x:c>
       <x:c r="M406" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N406" t="str"/>
       <x:c r="O406" t="str"/>
@@ -20541,9 +20555,11 @@
       <x:c r="K407" t="str">
         <x:v>ECLECTI</x:v>
       </x:c>
-      <x:c r="L407" t="str"/>
+      <x:c r="L407" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FAM-000000421-famowood-water-based-natural-24oz.png?raw=true</x:v>
+      </x:c>
       <x:c r="M407" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N407" t="str"/>
       <x:c r="O407" t="str"/>
@@ -20594,9 +20610,11 @@
       <x:c r="K408" t="str">
         <x:v>ENN01</x:v>
       </x:c>
-      <x:c r="L408" t="str"/>
+      <x:c r="L408" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/EF-000000422-ennis-flint-traffic-paint-family.png?raw=true</x:v>
+      </x:c>
       <x:c r="M408" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N408" t="str"/>
       <x:c r="O408" t="str"/>
@@ -20639,9 +20657,11 @@
       <x:c r="K409" t="str">
         <x:v>ENN01</x:v>
       </x:c>
-      <x:c r="L409" t="str"/>
+      <x:c r="L409" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/EF-000000422-ennis-flint-traffic-paint-family.png?raw=true</x:v>
+      </x:c>
       <x:c r="M409" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N409" t="str"/>
       <x:c r="O409" t="str"/>
@@ -20684,9 +20704,11 @@
       <x:c r="K410" t="str">
         <x:v>ENN01</x:v>
       </x:c>
-      <x:c r="L410" t="str"/>
+      <x:c r="L410" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/EF-000000422-ennis-flint-traffic-paint-family.png?raw=true</x:v>
+      </x:c>
       <x:c r="M410" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N410" t="str"/>
       <x:c r="O410" t="str"/>
@@ -20729,9 +20751,11 @@
       <x:c r="K411" t="str">
         <x:v>ENN01</x:v>
       </x:c>
-      <x:c r="L411" t="str"/>
+      <x:c r="L411" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/EF-000000422-ennis-flint-traffic-paint-family.png?raw=true</x:v>
+      </x:c>
       <x:c r="M411" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N411" t="str"/>
       <x:c r="O411" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 169-180
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rd2d1bbccd6534f2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R904a35e177304531"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20798,9 +20798,11 @@
       <x:c r="K412" t="str">
         <x:v>ENN01</x:v>
       </x:c>
-      <x:c r="L412" t="str"/>
+      <x:c r="L412" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/EF-000000422-ennis-flint-traffic-paint-family.png?raw=true</x:v>
+      </x:c>
       <x:c r="M412" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N412" t="str"/>
       <x:c r="O412" t="str"/>
@@ -20843,9 +20845,11 @@
       <x:c r="K413" t="str">
         <x:v>ENN01</x:v>
       </x:c>
-      <x:c r="L413" t="str"/>
+      <x:c r="L413" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/EF-000000422-ennis-flint-traffic-paint-family.png?raw=true</x:v>
+      </x:c>
       <x:c r="M413" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N413" t="str"/>
       <x:c r="O413" t="str"/>
@@ -20888,9 +20892,11 @@
       <x:c r="K414" t="str">
         <x:v>FEA01</x:v>
       </x:c>
-      <x:c r="L414" t="str"/>
+      <x:c r="L414" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FEA-000000428-featherlite-fl-3110-04-fiberglass-step-ladder.png?raw=true</x:v>
+      </x:c>
       <x:c r="M414" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N414" t="str"/>
       <x:c r="O414" t="str"/>
@@ -20933,9 +20939,11 @@
       <x:c r="K415" t="str">
         <x:v>TOO01</x:v>
       </x:c>
-      <x:c r="L415" t="str"/>
+      <x:c r="L415" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FEA-000000429-lite-five-foot-aluminum-step-ladder.png?raw=true</x:v>
+      </x:c>
       <x:c r="M415" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N415" t="str"/>
       <x:c r="O415" t="str"/>
@@ -20978,9 +20986,11 @@
       <x:c r="K416" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L416" t="str"/>
+      <x:c r="L416" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000430-festool-204308-selfclean-filter-bags.png?raw=true</x:v>
+      </x:c>
       <x:c r="M416" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N416" t="str"/>
       <x:c r="O416" t="str"/>
@@ -21023,9 +21033,11 @@
       <x:c r="K417" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L417" t="str"/>
+      <x:c r="L417" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000431-festool-205653-d225-p40-granat-disc.png?raw=true</x:v>
+      </x:c>
       <x:c r="M417" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N417" t="str"/>
       <x:c r="O417" t="str"/>
@@ -21068,9 +21080,11 @@
       <x:c r="K418" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L418" t="str"/>
+      <x:c r="L418" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000432-festool-497117-80x133-p40-granat-sheet.png?raw=true</x:v>
+      </x:c>
       <x:c r="M418" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N418" t="str"/>
       <x:c r="O418" t="str"/>
@@ -21113,9 +21127,11 @@
       <x:c r="K419" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L419" t="str"/>
+      <x:c r="L419" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000433-festool-497165-d125-p40-granat-disc.png?raw=true</x:v>
+      </x:c>
       <x:c r="M419" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N419" t="str"/>
       <x:c r="O419" t="str"/>
@@ -21158,9 +21174,11 @@
       <x:c r="K420" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L420" t="str"/>
+      <x:c r="L420" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000434-festool-497363-d90-p40-granat-disc.png?raw=true</x:v>
+      </x:c>
       <x:c r="M420" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N420" t="str"/>
       <x:c r="O420" t="str"/>
@@ -21203,9 +21221,11 @@
       <x:c r="K421" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L421" t="str"/>
+      <x:c r="L421" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000435-festool-497390-v93-p40-granat-sheet.png?raw=true</x:v>
+      </x:c>
       <x:c r="M421" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N421" t="str"/>
       <x:c r="O421" t="str"/>
@@ -21248,9 +21268,11 @@
       <x:c r="K422" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L422" t="str"/>
+      <x:c r="L422" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000436-festool-575160-d150-p40-granat-disc.png?raw=true</x:v>
+      </x:c>
       <x:c r="M422" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N422" t="str"/>
       <x:c r="O422" t="str"/>
@@ -21293,9 +21315,11 @@
       <x:c r="K423" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L423" t="str"/>
+      <x:c r="L423" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000437-festool-planex-lhs-225-eq-plus.png?raw=true</x:v>
+      </x:c>
       <x:c r="M423" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N423" t="str"/>
       <x:c r="O423" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 181-192
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R904a35e177304531"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R4842fbc96c2d413d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21362,9 +21362,11 @@
       <x:c r="K424" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L424" t="str"/>
+      <x:c r="L424" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000438-festool-ro-150-feq-plus-us.png?raw=true</x:v>
+      </x:c>
       <x:c r="M424" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N424" t="str"/>
       <x:c r="O424" t="str"/>
@@ -21407,9 +21409,11 @@
       <x:c r="K425" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L425" t="str"/>
+      <x:c r="L425" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000439-festool-ro-125-feq-plus-us.png?raw=true</x:v>
+      </x:c>
       <x:c r="M425" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N425" t="str"/>
       <x:c r="O425" t="str"/>
@@ -21452,9 +21456,11 @@
       <x:c r="K426" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L426" t="str"/>
+      <x:c r="L426" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000440-festool-rts-400-req-plus-us.png?raw=true</x:v>
+      </x:c>
       <x:c r="M426" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N426" t="str"/>
       <x:c r="O426" t="str"/>
@@ -21544,9 +21550,11 @@
       <x:c r="K428" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L428" t="str"/>
+      <x:c r="L428" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000442-festool-ro-90-dx-feq-plus-us.png?raw=true</x:v>
+      </x:c>
       <x:c r="M428" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N428" t="str"/>
       <x:c r="O428" t="str"/>
@@ -21589,9 +21597,11 @@
       <x:c r="K429" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L429" t="str"/>
+      <x:c r="L429" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000443-festool-ets-ec150-3-eq-plus-us.png?raw=true</x:v>
+      </x:c>
       <x:c r="M429" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N429" t="str"/>
       <x:c r="O429" t="str"/>
@@ -21634,9 +21644,11 @@
       <x:c r="K430" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L430" t="str"/>
+      <x:c r="L430" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000444-festool-ets-ec125-3-eq-plus-us.png?raw=true</x:v>
+      </x:c>
       <x:c r="M430" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N430" t="str"/>
       <x:c r="O430" t="str"/>
@@ -21679,9 +21691,11 @@
       <x:c r="K431" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L431" t="str"/>
+      <x:c r="L431" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000445-festool-rg-130-eci-plus-us.png?raw=true</x:v>
+      </x:c>
       <x:c r="M431" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N431" t="str"/>
       <x:c r="O431" t="str"/>
@@ -21724,9 +21738,11 @@
       <x:c r="K432" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L432" t="str"/>
+      <x:c r="L432" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000446-festool-dtsc-400-3-0-i-plus-us.png?raw=true</x:v>
+      </x:c>
       <x:c r="M432" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N432" t="str"/>
       <x:c r="O432" t="str"/>
@@ -21769,9 +21785,11 @@
       <x:c r="K433" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L433" t="str"/>
+      <x:c r="L433" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000447-festool-dts-400-req-plus-us.png?raw=true</x:v>
+      </x:c>
       <x:c r="M433" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N433" t="str"/>
       <x:c r="O433" t="str"/>
@@ -21814,9 +21832,11 @@
       <x:c r="K434" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L434" t="str"/>
+      <x:c r="L434" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000448-festool-577542-delta-p40-granat-sheet.png?raw=true</x:v>
+      </x:c>
       <x:c r="M434" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N434" t="str"/>
       <x:c r="O434" t="str"/>
@@ -21859,9 +21879,11 @@
       <x:c r="K435" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L435" t="str"/>
+      <x:c r="L435" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PC-000000449-festool-t18-plus-3-hpc-4-0-i-set-us.png?raw=true</x:v>
+      </x:c>
       <x:c r="M435" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N435" t="str"/>
       <x:c r="O435" t="str"/>
@@ -21904,9 +21926,11 @@
       <x:c r="K436" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L436" t="str"/>
+      <x:c r="L436" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000450-festool-tid-18-basic-us.png?raw=true</x:v>
+      </x:c>
       <x:c r="M436" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N436" t="str"/>
       <x:c r="O436" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 193-204
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R4842fbc96c2d413d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R18e4ea77b6ab498e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22020,9 +22020,11 @@
       <x:c r="K438" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L438" t="str"/>
+      <x:c r="L438" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000452-festool-ct-48-e-ac-hepa.png?raw=true</x:v>
+      </x:c>
       <x:c r="M438" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N438" t="str"/>
       <x:c r="O438" t="str"/>
@@ -22065,9 +22067,11 @@
       <x:c r="K439" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L439" t="str"/>
+      <x:c r="L439" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000453-festool-ct-15-hepa-us.png?raw=true</x:v>
+      </x:c>
       <x:c r="M439" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N439" t="str"/>
       <x:c r="O439" t="str"/>
@@ -22110,9 +22114,11 @@
       <x:c r="K440" t="str">
         <x:v>FESTOOL</x:v>
       </x:c>
-      <x:c r="L440" t="str"/>
+      <x:c r="L440" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FES-000000454-festool-ct-midi-i-hepa-us.png?raw=true</x:v>
+      </x:c>
       <x:c r="M440" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N440" t="str"/>
       <x:c r="O440" t="str"/>
@@ -22255,9 +22261,11 @@
       <x:c r="K443" t="str">
         <x:v>CANPRO</x:v>
       </x:c>
-      <x:c r="L443" t="str"/>
+      <x:c r="L443" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/R3-000000457-level360-sd100-5-100-grit-discs.png?raw=true</x:v>
+      </x:c>
       <x:c r="M443" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N443" t="str"/>
       <x:c r="O443" t="str"/>
@@ -22300,9 +22308,11 @@
       <x:c r="K444" t="str">
         <x:v>CANPRO</x:v>
       </x:c>
-      <x:c r="L444" t="str"/>
+      <x:c r="L444" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/R3-000000458-full-circle-flex-edge-2-replacement-pad.png?raw=true</x:v>
+      </x:c>
       <x:c r="M444" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N444" t="str"/>
       <x:c r="O444" t="str"/>
@@ -22345,9 +22355,11 @@
       <x:c r="K445" t="str">
         <x:v>GHI01</x:v>
       </x:c>
-      <x:c r="L445" t="str"/>
+      <x:c r="L445" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GI-000000459-black-jack-drive-kote-500.png?raw=true</x:v>
+      </x:c>
       <x:c r="M445" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N445" t="str"/>
       <x:c r="O445" t="str"/>
@@ -22390,9 +22402,11 @@
       <x:c r="K446" t="str">
         <x:v>CANPRO</x:v>
       </x:c>
-      <x:c r="L446" t="str"/>
+      <x:c r="L446" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GOR-000000460-gorilla-wood-glue-8oz.png?raw=true</x:v>
+      </x:c>
       <x:c r="M446" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N446" t="str"/>
       <x:c r="O446" t="str"/>
@@ -22576,9 +22590,11 @@
       <x:c r="K450" t="str">
         <x:v>CANPRO</x:v>
       </x:c>
-      <x:c r="L450" t="str"/>
+      <x:c r="L450" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GOR-000000464-gorilla-epoxy-clear.png?raw=true</x:v>
+      </x:c>
       <x:c r="M450" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N450" t="str"/>
       <x:c r="O450" t="str"/>
@@ -22621,9 +22637,11 @@
       <x:c r="K451" t="str">
         <x:v>GOE01</x:v>
       </x:c>
-      <x:c r="L451" t="str"/>
+      <x:c r="L451" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/EZ-000000465-ez-mix-70032-one-quart-cup.png?raw=true</x:v>
+      </x:c>
       <x:c r="M451" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N451" t="str"/>
       <x:c r="O451" t="str"/>
@@ -22719,9 +22737,11 @@
       <x:c r="K453" t="str">
         <x:v>GOE01</x:v>
       </x:c>
-      <x:c r="L453" t="str"/>
+      <x:c r="L453" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/NAT-000000467-nazionale-silver-leaf-500-sheet-pack.png?raw=true</x:v>
+      </x:c>
       <x:c r="M453" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N453" t="str"/>
       <x:c r="O453" t="str"/>
@@ -22764,9 +22784,11 @@
       <x:c r="K454" t="str">
         <x:v>GOE01</x:v>
       </x:c>
-      <x:c r="L454" t="str"/>
+      <x:c r="L454" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/NAT-000000468-nazionale-composition-gold-leaf-500-sheet-pack.png?raw=true</x:v>
+      </x:c>
       <x:c r="M454" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N454" t="str"/>
       <x:c r="O454" t="str"/>
@@ -22944,9 +22966,11 @@
       <x:c r="K458" t="str">
         <x:v>GOE01</x:v>
       </x:c>
-      <x:c r="L458" t="str"/>
+      <x:c r="L458" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GY-000000472-dux-water-based-gilding-size-8oz.png?raw=true</x:v>
+      </x:c>
       <x:c r="M458" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N458" t="str"/>
       <x:c r="O458" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 205-216
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R18e4ea77b6ab498e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R2e17acdba0184200"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23058,9 +23058,11 @@
       <x:c r="K460" t="str">
         <x:v>GRA01-S</x:v>
       </x:c>
-      <x:c r="L460" t="str"/>
+      <x:c r="L460" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GRA-000000474-graco-206994-tsl-throat-seal-liquid.png?raw=true</x:v>
+      </x:c>
       <x:c r="M460" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N460" t="str"/>
       <x:c r="O460" t="str"/>
@@ -23148,9 +23150,11 @@
       <x:c r="K462" t="str">
         <x:v>GRA01-S</x:v>
       </x:c>
-      <x:c r="L462" t="str"/>
+      <x:c r="L462" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GRA-000000476-graco-ultra-quickshot-20b473.png?raw=true</x:v>
+      </x:c>
       <x:c r="M462" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N462" t="str"/>
       <x:c r="O462" t="str"/>
@@ -23193,9 +23197,11 @@
       <x:c r="K463" t="str">
         <x:v>GRA01-S</x:v>
       </x:c>
-      <x:c r="L463" t="str"/>
+      <x:c r="L463" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GRA-000000477-graco-ll5315-linelazer-rac-5-switchtip.png?raw=true</x:v>
+      </x:c>
       <x:c r="M463" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N463" t="str"/>
       <x:c r="O463" t="str"/>
@@ -23283,9 +23289,11 @@
       <x:c r="K465" t="str">
         <x:v>GRA01-S</x:v>
       </x:c>
-      <x:c r="L465" t="str"/>
+      <x:c r="L465" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GRA-000000479-graco-finishpro-gx19-17f924.png?raw=true</x:v>
+      </x:c>
       <x:c r="M465" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N465" t="str"/>
       <x:c r="O465" t="str"/>
@@ -23328,9 +23336,11 @@
       <x:c r="K466" t="str">
         <x:v>GRA01-S</x:v>
       </x:c>
-      <x:c r="L466" t="str"/>
+      <x:c r="L466" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GRA-000000480-graco-fflp108-fine-finish-switchtip.png?raw=true</x:v>
+      </x:c>
       <x:c r="M466" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N466" t="str"/>
       <x:c r="O466" t="str"/>
@@ -23418,9 +23428,11 @@
       <x:c r="K468" t="str">
         <x:v>GRA01-S</x:v>
       </x:c>
-      <x:c r="L468" t="str"/>
+      <x:c r="L468" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GRA-000000482-graco-contractor-powershot-xt-18h301.png?raw=true</x:v>
+      </x:c>
       <x:c r="M468" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N468" t="str"/>
       <x:c r="O468" t="str"/>
@@ -23870,9 +23882,11 @@
       <x:c r="K478" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L478" t="str"/>
+      <x:c r="L478" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/JBW-000000492-jb-weld-superweld-instant-adhesive.png?raw=true</x:v>
+      </x:c>
       <x:c r="M478" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N478" t="str"/>
       <x:c r="O478" t="str"/>
@@ -23915,9 +23929,11 @@
       <x:c r="K479" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L479" t="str"/>
+      <x:c r="L479" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/JBW-000000493-jb-weld-original-cold-weld-8265s.png?raw=true</x:v>
+      </x:c>
       <x:c r="M479" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N479" t="str"/>
       <x:c r="O479" t="str"/>
@@ -23960,9 +23976,11 @@
       <x:c r="K480" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L480" t="str"/>
+      <x:c r="L480" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/JBW-000000494-jb-weld-minuteweld-syringe-50101.png?raw=true</x:v>
+      </x:c>
       <x:c r="M480" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N480" t="str"/>
       <x:c r="O480" t="str"/>
@@ -24232,9 +24250,11 @@
       <x:c r="K486" t="str">
         <x:v>DIVERS</x:v>
       </x:c>
-      <x:c r="L486" t="str"/>
+      <x:c r="L486" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/KRY-000000500-krylon-fusion-satin-black-k02732007.png?raw=true</x:v>
+      </x:c>
       <x:c r="M486" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N486" t="str"/>
       <x:c r="O486" t="str"/>
@@ -24277,9 +24297,11 @@
       <x:c r="K487" t="str">
         <x:v>DIVERS</x:v>
       </x:c>
-      <x:c r="L487" t="str"/>
+      <x:c r="L487" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/KRY-000000501-krylon-fusion-metallic-gold-k02770007.png?raw=true</x:v>
+      </x:c>
       <x:c r="M487" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N487" t="str"/>
       <x:c r="O487" t="str"/>
@@ -24322,9 +24344,11 @@
       <x:c r="K488" t="str">
         <x:v>DIVERS</x:v>
       </x:c>
-      <x:c r="L488" t="str"/>
+      <x:c r="L488" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/KRY-000000502-krylon-fusion-gloss-black-k02702007.png?raw=true</x:v>
+      </x:c>
       <x:c r="M488" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N488" t="str"/>
       <x:c r="O488" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 217-228
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R2e17acdba0184200"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R28660eac4f894ecc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -24391,9 +24391,11 @@
       <x:c r="K489" t="str">
         <x:v>DIVERS</x:v>
       </x:c>
-      <x:c r="L489" t="str"/>
+      <x:c r="L489" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/KRY-000000503-krylon-fusion-flat-black-k02728007.png?raw=true</x:v>
+      </x:c>
       <x:c r="M489" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N489" t="str"/>
       <x:c r="O489" t="str"/>
@@ -24759,9 +24761,11 @@
       <x:c r="K497" t="str">
         <x:v>DOVER</x:v>
       </x:c>
-      <x:c r="L497" t="str"/>
+      <x:c r="L497" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PC-000000511-pc-woody-6oz.png?raw=true</x:v>
+      </x:c>
       <x:c r="M497" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N497" t="str"/>
       <x:c r="O497" t="str"/>
@@ -24804,9 +24808,11 @@
       <x:c r="K498" t="str">
         <x:v>DOVER</x:v>
       </x:c>
-      <x:c r="L498" t="str"/>
+      <x:c r="L498" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PC-000000512-pc-clear-1oz.png?raw=true</x:v>
+      </x:c>
       <x:c r="M498" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N498" t="str"/>
       <x:c r="O498" t="str"/>
@@ -24849,9 +24855,11 @@
       <x:c r="K499" t="str">
         <x:v>DOVER</x:v>
       </x:c>
-      <x:c r="L499" t="str"/>
+      <x:c r="L499" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PC-000000513-pc-petrifier-8oz.png?raw=true</x:v>
+      </x:c>
       <x:c r="M499" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N499" t="str"/>
       <x:c r="O499" t="str"/>
@@ -24894,9 +24902,11 @@
       <x:c r="K500" t="str">
         <x:v>DOVER</x:v>
       </x:c>
-      <x:c r="L500" t="str"/>
+      <x:c r="L500" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PC-000000514-pc-lumber-1oz.png?raw=true</x:v>
+      </x:c>
       <x:c r="M500" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N500" t="str"/>
       <x:c r="O500" t="str"/>
@@ -25078,9 +25088,11 @@
       <x:c r="K504" t="str">
         <x:v>MEODED</x:v>
       </x:c>
-      <x:c r="L504" t="str"/>
+      <x:c r="L504" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MEO-000000518-meoded-stain-shield-quart.png?raw=true</x:v>
+      </x:c>
       <x:c r="M504" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N504" t="str"/>
       <x:c r="O504" t="str"/>
@@ -25313,9 +25325,11 @@
       <x:c r="K509" t="str">
         <x:v>MEODED</x:v>
       </x:c>
-      <x:c r="L509" t="str"/>
+      <x:c r="L509" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MEO-000000523-meoded-moroccan-clay.png?raw=true</x:v>
+      </x:c>
       <x:c r="M509" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N509" t="str"/>
       <x:c r="O509" t="str"/>
@@ -25452,9 +25466,11 @@
       <x:c r="K512" t="str">
         <x:v>MEODED</x:v>
       </x:c>
-      <x:c r="L512" t="str"/>
+      <x:c r="L512" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MEO-000000526-meoded-box-brush.png?raw=true</x:v>
+      </x:c>
       <x:c r="M512" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N512" t="str"/>
       <x:c r="O512" t="str"/>
@@ -25497,9 +25513,11 @@
       <x:c r="K513" t="str">
         <x:v>MEODED</x:v>
       </x:c>
-      <x:c r="L513" t="str"/>
+      <x:c r="L513" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MEO-000000527-meoded-hydrowax.png?raw=true</x:v>
+      </x:c>
       <x:c r="M513" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N513" t="str"/>
       <x:c r="O513" t="str"/>
@@ -26094,9 +26112,11 @@
       <x:c r="K526" t="str">
         <x:v>DIVERS</x:v>
       </x:c>
-      <x:c r="L526" t="str"/>
+      <x:c r="L526" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MIN-000000540-minwax-tung-oil-finish-1qt.png?raw=true</x:v>
+      </x:c>
       <x:c r="M526" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N526" t="str"/>
       <x:c r="O526" t="str"/>
@@ -26184,9 +26204,11 @@
       <x:c r="K528" t="str">
         <x:v>DIVERS</x:v>
       </x:c>
-      <x:c r="L528" t="str"/>
+      <x:c r="L528" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MIN-000000542-minwax-stainable-wood-filler-16oz.png?raw=true</x:v>
+      </x:c>
       <x:c r="M528" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N528" t="str"/>
       <x:c r="O528" t="str"/>
@@ -26366,9 +26388,11 @@
       <x:c r="K532" t="str">
         <x:v>DIVERS</x:v>
       </x:c>
-      <x:c r="L532" t="str"/>
+      <x:c r="L532" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MIN-000000546-minwax-pre-stain-wood-conditioner-1qt.png?raw=true</x:v>
+      </x:c>
       <x:c r="M532" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N532" t="str"/>
       <x:c r="O532" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 229-240
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R28660eac4f894ecc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R8281570c347e4f31"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26435,9 +26435,11 @@
       <x:c r="K533" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L533" t="str"/>
+      <x:c r="L533" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MM-000000547-modern-masters-flash-gold-me164-6oz.png?raw=true</x:v>
+      </x:c>
       <x:c r="M533" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N533" t="str"/>
       <x:c r="O533" t="str"/>
@@ -26488,9 +26490,11 @@
       <x:c r="K534" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L534" t="str"/>
+      <x:c r="L534" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MM-000000548-modern-masters-masterclear-supreme-satin-gallon.png?raw=true</x:v>
+      </x:c>
       <x:c r="M534" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N534" t="str"/>
       <x:c r="O534" t="str"/>
@@ -26533,9 +26537,11 @@
       <x:c r="K535" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L535" t="str"/>
+      <x:c r="L535" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DYN-000000549-ptc-pro-tint-medium-yellow-74303.png?raw=true</x:v>
+      </x:c>
       <x:c r="M535" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N535" t="str"/>
       <x:c r="O535" t="str"/>
@@ -26578,9 +26584,11 @@
       <x:c r="K536" t="str">
         <x:v>TOO01</x:v>
       </x:c>
-      <x:c r="L536" t="str"/>
+      <x:c r="L536" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/KS-000000550-klenks-815201-white-epoxy-enamel-1l.png?raw=true</x:v>
+      </x:c>
       <x:c r="M536" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N536" t="str"/>
       <x:c r="O536" t="str"/>
@@ -26623,9 +26631,11 @@
       <x:c r="K537" t="str">
         <x:v>YHD01</x:v>
       </x:c>
-      <x:c r="L537" t="str"/>
+      <x:c r="L537" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/HOM-000000551-homax-4092-orange-peel-spray-texture-20oz.png?raw=true</x:v>
+      </x:c>
       <x:c r="M537" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N537" t="str"/>
       <x:c r="O537" t="str"/>
@@ -26668,9 +26678,11 @@
       <x:c r="K538" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L538" t="str"/>
+      <x:c r="L538" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/HOM-000000552-homax-4575-pro-popcorn-ceiling-texture.png?raw=true</x:v>
+      </x:c>
       <x:c r="M538" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N538" t="str"/>
       <x:c r="O538" t="str"/>
@@ -26713,9 +26725,11 @@
       <x:c r="K539" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L539" t="str"/>
+      <x:c r="L539" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GO-000000553-goof-off-ultimate-remover-fg653-16oz.png?raw=true</x:v>
+      </x:c>
       <x:c r="M539" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N539" t="str"/>
       <x:c r="O539" t="str"/>
@@ -26758,9 +26772,11 @@
       <x:c r="K540" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L540" t="str"/>
+      <x:c r="L540" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GO-000000554-goof-off-2-low-odor-remover-6oz.png?raw=true</x:v>
+      </x:c>
       <x:c r="M540" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N540" t="str"/>
       <x:c r="O540" t="str"/>
@@ -26803,9 +26819,11 @@
       <x:c r="K541" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L541" t="str"/>
+      <x:c r="L541" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GO-000000555-goof-off-fg654-professional-strength-16oz.png?raw=true</x:v>
+      </x:c>
       <x:c r="M541" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N541" t="str"/>
       <x:c r="O541" t="str"/>
@@ -26848,9 +26866,11 @@
       <x:c r="K542" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L542" t="str"/>
+      <x:c r="L542" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DYN-000000556-dynamic-chomp-cleaner-degreaser-946ml.png?raw=true</x:v>
+      </x:c>
       <x:c r="M542" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N542" t="str"/>
       <x:c r="O542" t="str"/>
@@ -26893,9 +26913,11 @@
       <x:c r="K543" t="str">
         <x:v>YHD01</x:v>
       </x:c>
-      <x:c r="L543" t="str"/>
+      <x:c r="L543" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CI-000000557-circa-1850-wallpaper-prep-coat-1l.png?raw=true</x:v>
+      </x:c>
       <x:c r="M543" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N543" t="str"/>
       <x:c r="O543" t="str"/>
@@ -26938,9 +26960,11 @@
       <x:c r="K544" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L544" t="str"/>
+      <x:c r="L544" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GG-000000558-goo-gone-gg66-all-purpose-cleaner-24oz.png?raw=true</x:v>
+      </x:c>
       <x:c r="M544" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N544" t="str"/>
       <x:c r="O544" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 241-252
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R8281570c347e4f31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R8aafb6f13b344072"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -27007,9 +27007,11 @@
       <x:c r="K545" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L545" t="str"/>
+      <x:c r="L545" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DYN-000000559-dynamic-kz00sl96-super-lid-with-spout.png?raw=true</x:v>
+      </x:c>
       <x:c r="M545" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N545" t="str"/>
       <x:c r="O545" t="str"/>
@@ -27052,9 +27054,11 @@
       <x:c r="K546" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L546" t="str"/>
+      <x:c r="L546" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DYN-000000560-dynamic-az002882-staining-pad.png?raw=true</x:v>
+      </x:c>
       <x:c r="M546" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N546" t="str"/>
       <x:c r="O546" t="str"/>
@@ -27097,9 +27101,11 @@
       <x:c r="K547" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L547" t="str"/>
+      <x:c r="L547" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ST-000000561-spring-tools-32r12-combo-nail-set.png?raw=true</x:v>
+      </x:c>
       <x:c r="M547" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N547" t="str"/>
       <x:c r="O547" t="str"/>
@@ -27189,9 +27195,11 @@
       <x:c r="K549" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L549" t="str"/>
+      <x:c r="L549" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RHO-000000563-rhodes-american-grade-1-steel-wool-12-pack.png?raw=true</x:v>
+      </x:c>
       <x:c r="M549" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N549" t="str"/>
       <x:c r="O549" t="str"/>
@@ -27234,9 +27242,11 @@
       <x:c r="K550" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L550" t="str"/>
+      <x:c r="L550" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DYN-000000564-dynamic-dyna-patch-pro-860ml.png?raw=true</x:v>
+      </x:c>
       <x:c r="M550" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N550" t="str"/>
       <x:c r="O550" t="str"/>
@@ -27326,9 +27336,11 @@
       <x:c r="K552" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L552" t="str"/>
+      <x:c r="L552" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PRE-000000566-preval-0268-power-unit.png?raw=true</x:v>
+      </x:c>
       <x:c r="M552" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N552" t="str"/>
       <x:c r="O552" t="str"/>
@@ -27371,9 +27383,11 @@
       <x:c r="K553" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L553" t="str"/>
+      <x:c r="L553" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PIC-000000567-proform-pic1-picasso-oval-angled-brush.png?raw=true</x:v>
+      </x:c>
       <x:c r="M553" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N553" t="str"/>
       <x:c r="O553" t="str"/>
@@ -27416,9 +27430,11 @@
       <x:c r="K554" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L554" t="str"/>
+      <x:c r="L554" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GB-000000568-dynamic-glue-buster-adhesive-remover-3-78l.png?raw=true</x:v>
+      </x:c>
       <x:c r="M554" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N554" t="str"/>
       <x:c r="O554" t="str"/>
@@ -27461,9 +27477,11 @@
       <x:c r="K555" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L555" t="str"/>
+      <x:c r="L555" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DYN-000000569-dynamic-11174-brush-roller-spinner-cleaner.png?raw=true</x:v>
+      </x:c>
       <x:c r="M555" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N555" t="str"/>
       <x:c r="O555" t="str"/>
@@ -27506,9 +27524,11 @@
       <x:c r="K556" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L556" t="str"/>
+      <x:c r="L556" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CC-000000570-crocodile-cloth-original.png?raw=true</x:v>
+      </x:c>
       <x:c r="M556" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N556" t="str"/>
       <x:c r="O556" t="str"/>
@@ -27596,9 +27616,11 @@
       <x:c r="K558" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L558" t="str"/>
+      <x:c r="L558" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DYN-000000572-1000-plus-stain-remover-909ml.png?raw=true</x:v>
+      </x:c>
       <x:c r="M558" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N558" t="str"/>
       <x:c r="O558" t="str"/>
@@ -27641,9 +27663,11 @@
       <x:c r="K559" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L559" t="str"/>
+      <x:c r="L559" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/REC-000000573-recochem-solvable-boiled-linseed-oil.png?raw=true</x:v>
+      </x:c>
       <x:c r="M559" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N559" t="str"/>
       <x:c r="O559" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 253-264
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R8aafb6f13b344072"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Ra0d5a748525d41d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -27710,9 +27710,11 @@
       <x:c r="K560" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L560" t="str"/>
+      <x:c r="L560" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PEN-000000574-penofin-red-label-sable-gallon.png?raw=true</x:v>
+      </x:c>
       <x:c r="M560" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N560" t="str"/>
       <x:c r="O560" t="str"/>
@@ -27755,9 +27757,11 @@
       <x:c r="K561" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L561" t="str"/>
+      <x:c r="L561" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PEN-000000575-penofin-tsf-hardwood-satin-finish.png?raw=true</x:v>
+      </x:c>
       <x:c r="M561" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N561" t="str"/>
       <x:c r="O561" t="str"/>
@@ -27800,9 +27804,11 @@
       <x:c r="K562" t="str">
         <x:v>YHD01</x:v>
       </x:c>
-      <x:c r="L562" t="str"/>
+      <x:c r="L562" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PEN-000000576-penofin-exterior-hardwood-formula-quart.png?raw=true</x:v>
+      </x:c>
       <x:c r="M562" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N562" t="str"/>
       <x:c r="O562" t="str"/>
@@ -27900,9 +27906,11 @@
       <x:c r="K564" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L564" t="str"/>
+      <x:c r="L564" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DYN-000000578-monkey-rung-spin-pro-mini.png?raw=true</x:v>
+      </x:c>
       <x:c r="M564" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N564" t="str"/>
       <x:c r="O564" t="str"/>
@@ -27945,9 +27953,11 @@
       <x:c r="K565" t="str">
         <x:v>SAINT-G</x:v>
       </x:c>
-      <x:c r="L565" t="str"/>
+      <x:c r="L565" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/NOR-000000579-norton-wallsand-pad-150-grit.png?raw=true</x:v>
+      </x:c>
       <x:c r="M565" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N565" t="str"/>
       <x:c r="O565" t="str"/>
@@ -27990,9 +28000,11 @@
       <x:c r="K566" t="str">
         <x:v>SAINT-G</x:v>
       </x:c>
-      <x:c r="L566" t="str"/>
+      <x:c r="L566" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/NOR-000000580-norton-3x-sandpaper-180-grit.png?raw=true</x:v>
+      </x:c>
       <x:c r="M566" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N566" t="str"/>
       <x:c r="O566" t="str"/>
@@ -28035,9 +28047,11 @@
       <x:c r="K567" t="str">
         <x:v>SAINT-G</x:v>
       </x:c>
-      <x:c r="L567" t="str"/>
+      <x:c r="L567" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/NOR-000000581-norton-3x-sandpaper-100-grit.png?raw=true</x:v>
+      </x:c>
       <x:c r="M567" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N567" t="str"/>
       <x:c r="O567" t="str"/>
@@ -28088,9 +28102,11 @@
       <x:c r="K568" t="str">
         <x:v>SAINT-G</x:v>
       </x:c>
-      <x:c r="L568" t="str"/>
+      <x:c r="L568" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/NOR-000000582-norton-12x18-red-buffing-pad.png?raw=true</x:v>
+      </x:c>
       <x:c r="M568" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N568" t="str"/>
       <x:c r="O568" t="str"/>
@@ -28133,9 +28149,11 @@
       <x:c r="K569" t="str">
         <x:v>SAINT-G</x:v>
       </x:c>
-      <x:c r="L569" t="str"/>
+      <x:c r="L569" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/NOR-000000583-norton-12x18-60-grit-adhesive-sheets.png?raw=true</x:v>
+      </x:c>
       <x:c r="M569" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N569" t="str"/>
       <x:c r="O569" t="str"/>
@@ -28178,9 +28196,11 @@
       <x:c r="K570" t="str">
         <x:v>NOUR</x:v>
       </x:c>
-      <x:c r="L570" t="str"/>
+      <x:c r="L570" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/NO-000000584-nour-32-100nlw-limewash-brush.png?raw=true</x:v>
+      </x:c>
       <x:c r="M570" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N570" t="str"/>
       <x:c r="O570" t="str"/>
@@ -28223,9 +28243,11 @@
       <x:c r="K571" t="str">
         <x:v>NOUR</x:v>
       </x:c>
-      <x:c r="L571" t="str"/>
+      <x:c r="L571" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/NO-000000585-nour-polylamb-roller-refill.png?raw=true</x:v>
+      </x:c>
       <x:c r="M571" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N571" t="str"/>
       <x:c r="O571" t="str"/>
@@ -28268,9 +28290,11 @@
       <x:c r="K572" t="str">
         <x:v>NOUR</x:v>
       </x:c>
-      <x:c r="L572" t="str"/>
+      <x:c r="L572" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AP-000000586-allpro-silver-series-2-5-polyester-brush.png?raw=true</x:v>
+      </x:c>
       <x:c r="M572" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N572" t="str"/>
       <x:c r="O572" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 265-276
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Ra0d5a748525d41d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R36d8006b6bce4a4d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -28337,9 +28337,11 @@
       <x:c r="K573" t="str">
         <x:v>NOUR</x:v>
       </x:c>
-      <x:c r="L573" t="str"/>
+      <x:c r="L573" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AP-000000587-allpro-microfiber-roller-9x5-8.png?raw=true</x:v>
+      </x:c>
       <x:c r="M573" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N573" t="str"/>
       <x:c r="O573" t="str"/>
@@ -28429,9 +28431,11 @@
       <x:c r="K575" t="str">
         <x:v>OLF01</x:v>
       </x:c>
-      <x:c r="L575" t="str"/>
+      <x:c r="L575" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/OLF-000000589-olfa-abb50b-black-9mm-blades.png?raw=true</x:v>
+      </x:c>
       <x:c r="M575" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N575" t="str"/>
       <x:c r="O575" t="str"/>
@@ -28576,9 +28580,11 @@
       <x:c r="K578" t="str">
         <x:v>OLF01</x:v>
       </x:c>
-      <x:c r="L578" t="str"/>
+      <x:c r="L578" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/OLF-000000592-olfa-lbb50b-black-18mm-blades.png?raw=true</x:v>
+      </x:c>
       <x:c r="M578" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N578" t="str"/>
       <x:c r="O578" t="str"/>
@@ -28676,9 +28682,11 @@
       <x:c r="K580" t="str">
         <x:v>PPG</x:v>
       </x:c>
-      <x:c r="L580" t="str"/>
+      <x:c r="L580" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/OLY-000000594-olympic-rescue-it.png?raw=true</x:v>
+      </x:c>
       <x:c r="M580" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N580" t="str"/>
       <x:c r="O580" t="str"/>
@@ -28721,9 +28729,11 @@
       <x:c r="K581" t="str">
         <x:v>PPG</x:v>
       </x:c>
-      <x:c r="L581" t="str"/>
+      <x:c r="L581" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/OLY-000000595-olympic-maximum-semi-transparent-neutral.png?raw=true</x:v>
+      </x:c>
       <x:c r="M581" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N581" t="str"/>
       <x:c r="O581" t="str"/>
@@ -28766,9 +28776,11 @@
       <x:c r="K582" t="str">
         <x:v>OMC</x:v>
       </x:c>
-      <x:c r="L582" t="str"/>
+      <x:c r="L582" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/OMC-000000596-painters-plastic.png?raw=true</x:v>
+      </x:c>
       <x:c r="M582" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N582" t="str"/>
       <x:c r="O582" t="str"/>
@@ -28811,9 +28823,11 @@
       <x:c r="K583" t="str">
         <x:v>OMC</x:v>
       </x:c>
-      <x:c r="L583" t="str"/>
+      <x:c r="L583" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/OMC-000000597-fiberglass-drywall-tape.png?raw=true</x:v>
+      </x:c>
       <x:c r="M583" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N583" t="str"/>
       <x:c r="O583" t="str"/>
@@ -28856,9 +28870,11 @@
       <x:c r="K584" t="str">
         <x:v>OMC</x:v>
       </x:c>
-      <x:c r="L584" t="str"/>
+      <x:c r="L584" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/OMC-000000598-drywall-paper-tape.png?raw=true</x:v>
+      </x:c>
       <x:c r="M584" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N584" t="str"/>
       <x:c r="O584" t="str"/>
@@ -28901,9 +28917,11 @@
       <x:c r="K585" t="str">
         <x:v>OMC</x:v>
       </x:c>
-      <x:c r="L585" t="str"/>
+      <x:c r="L585" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/OMC-000000599-drywall-corner-tape.png?raw=true</x:v>
+      </x:c>
       <x:c r="M585" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N585" t="str"/>
       <x:c r="O585" t="str"/>
@@ -28946,9 +28964,11 @@
       <x:c r="K586" t="str">
         <x:v>OMC</x:v>
       </x:c>
-      <x:c r="L586" t="str"/>
+      <x:c r="L586" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/OMC-000000600-pre-taped-plastic-drop-cloth.png?raw=true</x:v>
+      </x:c>
       <x:c r="M586" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N586" t="str"/>
       <x:c r="O586" t="str"/>
@@ -28999,9 +29019,11 @@
       <x:c r="K587" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L587" t="str"/>
+      <x:c r="L587" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PI-000000601-trim-roller-3x5mm.png?raw=true</x:v>
+      </x:c>
       <x:c r="M587" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N587" t="str"/>
       <x:c r="O587" t="str"/>
@@ -29044,9 +29066,11 @@
       <x:c r="K588" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L588" t="str"/>
+      <x:c r="L588" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PI-000000602-pintar-slit-foam-refill.png?raw=true</x:v>
+      </x:c>
       <x:c r="M588" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N588" t="str"/>
       <x:c r="O588" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 277-288
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R36d8006b6bce4a4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R49f4aea9d7f543bf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -239,7 +239,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
-        <x:v>﻿Type</x:v>
+        <x:v>Type</x:v>
       </x:c>
       <x:c r="B1" t="str">
         <x:v>Name</x:v>
@@ -22161,9 +22161,11 @@
       <x:c r="K441" t="str">
         <x:v>FLA01-S</x:v>
       </x:c>
-      <x:c r="L441" t="str"/>
+      <x:c r="L441" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FC-000000455-flame-control-finish-coat.png?raw=true</x:v>
+      </x:c>
       <x:c r="M441" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N441" t="str">
         <x:v>Finishes</x:v>
@@ -22692,9 +22694,11 @@
       <x:c r="K452" t="str">
         <x:v>GOE01</x:v>
       </x:c>
-      <x:c r="L452" t="str"/>
+      <x:c r="L452" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GY-000000466-slik-bottle-fisheye-eliminator.png?raw=true</x:v>
+      </x:c>
       <x:c r="M452" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N452" t="str"/>
       <x:c r="O452" t="str"/>
@@ -22831,9 +22835,11 @@
       <x:c r="K455" t="str">
         <x:v>GOE01</x:v>
       </x:c>
-      <x:c r="L455" t="str"/>
+      <x:c r="L455" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GY-000000469-goudey-ngr-stain-red.png?raw=true</x:v>
+      </x:c>
       <x:c r="M455" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N455" t="str"/>
       <x:c r="O455" t="str"/>
@@ -22876,9 +22882,11 @@
       <x:c r="K456" t="str">
         <x:v>GOE01</x:v>
       </x:c>
-      <x:c r="L456" t="str"/>
+      <x:c r="L456" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GY-000000470-goudey-natural-paste-wood-filler.png?raw=true</x:v>
+      </x:c>
       <x:c r="M456" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N456" t="str"/>
       <x:c r="O456" t="str"/>
@@ -22921,9 +22929,11 @@
       <x:c r="K457" t="str">
         <x:v>GOE01</x:v>
       </x:c>
-      <x:c r="L457" t="str"/>
+      <x:c r="L457" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GY-000000471-goudey-acetone.png?raw=true</x:v>
+      </x:c>
       <x:c r="M457" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N457" t="str"/>
       <x:c r="O457" t="str"/>
@@ -23013,9 +23023,11 @@
       <x:c r="K459" t="str">
         <x:v>GRA01-S</x:v>
       </x:c>
-      <x:c r="L459" t="str"/>
+      <x:c r="L459" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GRA-000000473-graco-tip-hd.png?raw=true</x:v>
+      </x:c>
       <x:c r="M459" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N459" t="str"/>
       <x:c r="O459" t="str"/>
@@ -23105,9 +23117,11 @@
       <x:c r="K461" t="str">
         <x:v>GRA01-S</x:v>
       </x:c>
-      <x:c r="L461" t="str"/>
+      <x:c r="L461" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GRA-000000475-graco-rac-10-tip.png?raw=true</x:v>
+      </x:c>
       <x:c r="M461" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N461" t="str"/>
       <x:c r="O461" t="str"/>
@@ -23244,9 +23258,11 @@
       <x:c r="K464" t="str">
         <x:v>GRA01-S</x:v>
       </x:c>
-      <x:c r="L464" t="str"/>
+      <x:c r="L464" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GRA-000000478-graco-flat-tip.png?raw=true</x:v>
+      </x:c>
       <x:c r="M464" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N464" t="str"/>
       <x:c r="O464" t="str"/>
@@ -23383,9 +23399,11 @@
       <x:c r="K467" t="str">
         <x:v>GRA01-S</x:v>
       </x:c>
-      <x:c r="L467" t="str"/>
+      <x:c r="L467" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GRA-000000481-graco-filter.png?raw=true</x:v>
+      </x:c>
       <x:c r="M467" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N467" t="str"/>
       <x:c r="O467" t="str"/>
@@ -23475,9 +23493,11 @@
       <x:c r="K469" t="str">
         <x:v>GRA01-S</x:v>
       </x:c>
-      <x:c r="L469" t="str"/>
+      <x:c r="L469" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GRA-000000483-graco-extension.png?raw=true</x:v>
+      </x:c>
       <x:c r="M469" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N469" t="str"/>
       <x:c r="O469" t="str"/>
@@ -23520,9 +23540,11 @@
       <x:c r="K470" t="str">
         <x:v>GRIME</x:v>
       </x:c>
-      <x:c r="L470" t="str"/>
+      <x:c r="L470" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GE-000000484-purple-max-cleaner-degreaser.png?raw=true</x:v>
+      </x:c>
       <x:c r="M470" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N470" t="str"/>
       <x:c r="O470" t="str"/>
@@ -23565,9 +23587,11 @@
       <x:c r="K471" t="str">
         <x:v>GRIME</x:v>
       </x:c>
-      <x:c r="L471" t="str"/>
+      <x:c r="L471" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GE-000000485-power-maxx-hand-cleaner.png?raw=true</x:v>
+      </x:c>
       <x:c r="M471" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N471" t="str"/>
       <x:c r="O471" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 289-300
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R49f4aea9d7f543bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rbdd84e3c13314196"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23634,9 +23634,11 @@
       <x:c r="K472" t="str">
         <x:v>GRIME</x:v>
       </x:c>
-      <x:c r="L472" t="str"/>
+      <x:c r="L472" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GE-000000485-power-maxx-hand-cleaner.png?raw=true</x:v>
+      </x:c>
       <x:c r="M472" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N472" t="str"/>
       <x:c r="O472" t="str"/>
@@ -23679,9 +23681,11 @@
       <x:c r="K473" t="str">
         <x:v>GRIME</x:v>
       </x:c>
-      <x:c r="L473" t="str"/>
+      <x:c r="L473" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/GE-000000487-grime-eater-orange-hand-cleaner.png?raw=true</x:v>
+      </x:c>
       <x:c r="M473" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N473" t="str"/>
       <x:c r="O473" t="str"/>
@@ -23771,9 +23775,11 @@
       <x:c r="K475" t="str">
         <x:v>CANPRO</x:v>
       </x:c>
-      <x:c r="L475" t="str"/>
+      <x:c r="L475" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/HPP-000000489-handy-pail-liners.png?raw=true</x:v>
+      </x:c>
       <x:c r="M475" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N475" t="str"/>
       <x:c r="O475" t="str"/>
@@ -23816,9 +23822,11 @@
       <x:c r="K476" t="str">
         <x:v>HOLLAND</x:v>
       </x:c>
-      <x:c r="L476" t="str"/>
+      <x:c r="L476" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/HOL-000000490-shoppro-cordless-led-tripod-worklight.png?raw=true</x:v>
+      </x:c>
       <x:c r="M476" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N476" t="str"/>
       <x:c r="O476" t="str"/>
@@ -23861,9 +23869,11 @@
       <x:c r="K477" t="str">
         <x:v>HOLLAND</x:v>
       </x:c>
-      <x:c r="L477" t="str"/>
+      <x:c r="L477" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/HOL-000000491-shoppro-360-cannon-work-light.png?raw=true</x:v>
+      </x:c>
       <x:c r="M477" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N477" t="str"/>
       <x:c r="O477" t="str"/>
@@ -24047,9 +24057,11 @@
       <x:c r="K481" t="str">
         <x:v>CANPRO</x:v>
       </x:c>
-      <x:c r="L481" t="str"/>
+      <x:c r="L481" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/JEN-000000495-jen-2-inch-foam-brush.png?raw=true</x:v>
+      </x:c>
       <x:c r="M481" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N481" t="str"/>
       <x:c r="O481" t="str"/>
@@ -24092,9 +24104,11 @@
       <x:c r="K482" t="str">
         <x:v>EAE01</x:v>
       </x:c>
-      <x:c r="L482" t="str"/>
+      <x:c r="L482" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/KLI-000000496-wet-sanding-paper-1500-grit.png?raw=true</x:v>
+      </x:c>
       <x:c r="M482" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N482" t="str"/>
       <x:c r="O482" t="str"/>
@@ -24137,9 +24151,11 @@
       <x:c r="K483" t="str">
         <x:v>EAE01</x:v>
       </x:c>
-      <x:c r="L483" t="str"/>
+      <x:c r="L483" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/KLI-000000497-498-red-sandpaper-roll-100-grit.png?raw=true</x:v>
+      </x:c>
       <x:c r="M483" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N483" t="str"/>
       <x:c r="O483" t="str"/>
@@ -24182,9 +24198,11 @@
       <x:c r="K484" t="str">
         <x:v>EAE01</x:v>
       </x:c>
-      <x:c r="L484" t="str"/>
+      <x:c r="L484" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/KLI-000000497-498-red-sandpaper-roll-100-grit.png?raw=true</x:v>
+      </x:c>
       <x:c r="M484" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N484" t="str"/>
       <x:c r="O484" t="str"/>
@@ -24462,9 +24480,11 @@
       <x:c r="K490" t="str">
         <x:v>ABSOLUT</x:v>
       </x:c>
-      <x:c r="L490" t="str"/>
+      <x:c r="L490" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/LNL-000000504-last-n-last-satin-spar-varnish.png?raw=true</x:v>
+      </x:c>
       <x:c r="M490" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N490" t="str"/>
       <x:c r="O490" t="str"/>
@@ -24507,9 +24527,11 @@
       <x:c r="K491" t="str">
         <x:v>ABSOLUT</x:v>
       </x:c>
-      <x:c r="L491" t="str"/>
+      <x:c r="L491" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/LNL-000000505-last-n-last-gloss-urethane-350-voc.png?raw=true</x:v>
+      </x:c>
       <x:c r="M491" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N491" t="str"/>
       <x:c r="O491" t="str"/>
@@ -24552,9 +24574,11 @@
       <x:c r="K492" t="str">
         <x:v>ABSOLUT</x:v>
       </x:c>
-      <x:c r="L492" t="str"/>
+      <x:c r="L492" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/LNL-000000506-absco-polyurethane-satin.png?raw=true</x:v>
+      </x:c>
       <x:c r="M492" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N492" t="str"/>
       <x:c r="O492" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 301-312
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rbdd84e3c13314196"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Ra485cd50b6be441a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -24621,9 +24621,11 @@
       <x:c r="K493" t="str">
         <x:v>LEAKTITE</x:v>
       </x:c>
-      <x:c r="L493" t="str"/>
+      <x:c r="L493" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/LEA-000000507-leaktite-multi-purpose-mixing-pail.png?raw=true</x:v>
+      </x:c>
       <x:c r="M493" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N493" t="str"/>
       <x:c r="O493" t="str"/>
@@ -24674,9 +24676,11 @@
       <x:c r="K494" t="str">
         <x:v>LEM01</x:v>
       </x:c>
-      <x:c r="L494" t="str"/>
+      <x:c r="L494" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/LEM-000000508-lemmer-pot-liner.png?raw=true</x:v>
+      </x:c>
       <x:c r="M494" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N494" t="str"/>
       <x:c r="O494" t="str"/>
@@ -24719,9 +24723,11 @@
       <x:c r="K495" t="str">
         <x:v>LEM01</x:v>
       </x:c>
-      <x:c r="L495" t="str"/>
+      <x:c r="L495" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/LEM-000000509-lemmer-a910g-gravity-gun-conventional.png?raw=true</x:v>
+      </x:c>
       <x:c r="M495" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N495" t="str"/>
       <x:c r="O495" t="str"/>
@@ -24764,9 +24770,11 @@
       <x:c r="K496" t="str">
         <x:v>LEM01</x:v>
       </x:c>
-      <x:c r="L496" t="str"/>
+      <x:c r="L496" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/LEM-000000510-lemmer-pressure-pot-gun-hose-complete.png?raw=true</x:v>
+      </x:c>
       <x:c r="M496" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N496" t="str"/>
       <x:c r="O496" t="str"/>
@@ -24997,9 +25005,11 @@
       <x:c r="K501" t="str">
         <x:v>KILZ</x:v>
       </x:c>
-      <x:c r="L501" t="str"/>
+      <x:c r="L501" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/KIL-000000515-kilz-low-odor-spray-primer.png?raw=true</x:v>
+      </x:c>
       <x:c r="M501" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N501" t="str"/>
       <x:c r="O501" t="str"/>
@@ -25183,9 +25193,11 @@
       <x:c r="K505" t="str">
         <x:v>MEODED</x:v>
       </x:c>
-      <x:c r="L505" t="str"/>
+      <x:c r="L505" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MEO-000000519-meoded-plasterseal-plus.png?raw=true</x:v>
+      </x:c>
       <x:c r="M505" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N505" t="str"/>
       <x:c r="O505" t="str"/>
@@ -25228,9 +25240,11 @@
       <x:c r="K506" t="str">
         <x:v>MEODED</x:v>
       </x:c>
-      <x:c r="L506" t="str"/>
+      <x:c r="L506" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MEO-000000520-meoded-plasterguard-satin.png?raw=true</x:v>
+      </x:c>
       <x:c r="M506" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N506" t="str">
         <x:v>Finishes</x:v>
@@ -25281,9 +25295,11 @@
       <x:c r="K507" t="str">
         <x:v>MEODED</x:v>
       </x:c>
-      <x:c r="L507" t="str"/>
+      <x:c r="L507" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MEO-000000521-meoded-pearlas-velvet-white.png?raw=true</x:v>
+      </x:c>
       <x:c r="M507" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N507" t="str"/>
       <x:c r="O507" t="str"/>
@@ -25655,9 +25671,11 @@
       <x:c r="K515" t="str">
         <x:v>MEODED</x:v>
       </x:c>
-      <x:c r="L515" t="str"/>
+      <x:c r="L515" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MEO-000000529-meoded-crystal-brush-white-base.png?raw=true</x:v>
+      </x:c>
       <x:c r="M515" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N515" t="str"/>
       <x:c r="O515" t="str"/>
@@ -25700,9 +25718,11 @@
       <x:c r="K516" t="str">
         <x:v>MEODED</x:v>
       </x:c>
-      <x:c r="L516" t="str"/>
+      <x:c r="L516" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MEO-000000530-meoded-cristallo-clear-matte.png?raw=true</x:v>
+      </x:c>
       <x:c r="M516" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N516" t="str"/>
       <x:c r="O516" t="str"/>
@@ -25745,9 +25765,11 @@
       <x:c r="K517" t="str">
         <x:v>MEODED</x:v>
       </x:c>
-      <x:c r="L517" t="str"/>
+      <x:c r="L517" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MEO-000000531-meoded-concretta-fs-white.png?raw=true</x:v>
+      </x:c>
       <x:c r="M517" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N517" t="str"/>
       <x:c r="O517" t="str"/>
@@ -25790,9 +25812,11 @@
       <x:c r="K518" t="str">
         <x:v>YHD01</x:v>
       </x:c>
-      <x:c r="L518" t="str"/>
+      <x:c r="L518" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ME-000000532-messmers-uv-plus-natural.png?raw=true</x:v>
+      </x:c>
       <x:c r="M518" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N518" t="str"/>
       <x:c r="O518" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 313-324
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Ra485cd50b6be441a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rb096ed8b1ce0420b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25859,9 +25859,11 @@
       <x:c r="K519" t="str">
         <x:v>METAL</x:v>
       </x:c>
-      <x:c r="L519" t="str"/>
+      <x:c r="L519" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MET-000000533-metaltech-aluminum-scaffold.png?raw=true</x:v>
+      </x:c>
       <x:c r="M519" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N519" t="str"/>
       <x:c r="O519" t="str"/>
@@ -25904,9 +25906,11 @@
       <x:c r="K520" t="str">
         <x:v>METAL</x:v>
       </x:c>
-      <x:c r="L520" t="str"/>
+      <x:c r="L520" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MET-000000534-metaltech-yellow-baker-scaffold.png?raw=true</x:v>
+      </x:c>
       <x:c r="M520" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N520" t="str"/>
       <x:c r="O520" t="str"/>
@@ -25949,9 +25953,11 @@
       <x:c r="K521" t="str">
         <x:v>METAL</x:v>
       </x:c>
-      <x:c r="L521" t="str"/>
+      <x:c r="L521" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MET-000000535-metaltech-portable-work-platform.png?raw=true</x:v>
+      </x:c>
       <x:c r="M521" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N521" t="str"/>
       <x:c r="O521" t="str"/>
@@ -25994,9 +26000,11 @@
       <x:c r="K522" t="str">
         <x:v>METAL</x:v>
       </x:c>
-      <x:c r="L522" t="str"/>
+      <x:c r="L522" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MET-000000536-metaltech-aluminum-step-ladder.png?raw=true</x:v>
+      </x:c>
       <x:c r="M522" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N522" t="str"/>
       <x:c r="O522" t="str"/>
@@ -26039,9 +26047,11 @@
       <x:c r="K523" t="str">
         <x:v>DIVERS</x:v>
       </x:c>
-      <x:c r="L523" t="str"/>
+      <x:c r="L523" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MIN-000000537-minwax-wood-putty-910-golden-oak.png?raw=true</x:v>
+      </x:c>
       <x:c r="M523" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N523" t="str"/>
       <x:c r="O523" t="str"/>
@@ -26084,9 +26094,11 @@
       <x:c r="K524" t="str">
         <x:v>DIVERS</x:v>
       </x:c>
-      <x:c r="L524" t="str"/>
+      <x:c r="L524" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MIN-000000538-minwax-wood-filler.png?raw=true</x:v>
+      </x:c>
       <x:c r="M524" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N524" t="str"/>
       <x:c r="O524" t="str"/>
@@ -26231,9 +26243,11 @@
       <x:c r="K527" t="str">
         <x:v>DIVERS</x:v>
       </x:c>
-      <x:c r="L527" t="str"/>
+      <x:c r="L527" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MIN-000000541-minwax-teak-oil.png?raw=true</x:v>
+      </x:c>
       <x:c r="M527" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N527" t="str"/>
       <x:c r="O527" t="str"/>
@@ -26323,9 +26337,11 @@
       <x:c r="K529" t="str">
         <x:v>DIVERS</x:v>
       </x:c>
-      <x:c r="L529" t="str"/>
+      <x:c r="L529" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MIN-000000543-minwax-paste-wax.png?raw=true</x:v>
+      </x:c>
       <x:c r="M529" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N529" t="str"/>
       <x:c r="O529" t="str"/>
@@ -26415,9 +26431,11 @@
       <x:c r="K531" t="str">
         <x:v>DIVERS</x:v>
       </x:c>
-      <x:c r="L531" t="str"/>
+      <x:c r="L531" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/MIN-000000545-minwax-antique-oil-finish.png?raw=true</x:v>
+      </x:c>
       <x:c r="M531" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N531" t="str"/>
       <x:c r="O531" t="str"/>
@@ -27643,9 +27661,11 @@
       <x:c r="K557" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L557" t="str"/>
+      <x:c r="L557" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/DYN-000000571-dynamic-measuring-bucket.png?raw=true</x:v>
+      </x:c>
       <x:c r="M557" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N557" t="str"/>
       <x:c r="O557" t="str"/>
@@ -29185,9 +29205,11 @@
       <x:c r="K589" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L589" t="str"/>
+      <x:c r="L589" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PI-000000603-pre-caulking-filler-rope.png?raw=true</x:v>
+      </x:c>
       <x:c r="M589" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N589" t="str"/>
       <x:c r="O589" t="str"/>
@@ -29230,9 +29252,11 @@
       <x:c r="K590" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L590" t="str"/>
+      <x:c r="L590" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PI-000000604-pipe-roller.png?raw=true</x:v>
+      </x:c>
       <x:c r="M590" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N590" t="str"/>
       <x:c r="O590" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 325-336
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rb096ed8b1ce0420b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R6e1ab7fda41949f7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -29299,9 +29299,11 @@
       <x:c r="K591" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L591" t="str"/>
+      <x:c r="L591" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PI-000000605-pintar-lint-free-roller-refill.png?raw=true</x:v>
+      </x:c>
       <x:c r="M591" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N591" t="str"/>
       <x:c r="O591" t="str"/>
@@ -29352,9 +29354,11 @@
       <x:c r="K592" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L592" t="str"/>
+      <x:c r="L592" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PI-000000606-pintar-lambskin-block-applicator.png?raw=true</x:v>
+      </x:c>
       <x:c r="M592" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N592" t="str"/>
       <x:c r="O592" t="str"/>
@@ -29397,9 +29401,11 @@
       <x:c r="K593" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L593" t="str"/>
+      <x:c r="L593" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PI-000000607-water-wiz-pad-with-block.png?raw=true</x:v>
+      </x:c>
       <x:c r="M593" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N593" t="str"/>
       <x:c r="O593" t="str"/>
@@ -29442,9 +29448,11 @@
       <x:c r="K594" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L594" t="str"/>
+      <x:c r="L594" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PI-000000608-microfiber-pad-with-block.png?raw=true</x:v>
+      </x:c>
       <x:c r="M594" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N594" t="str"/>
       <x:c r="O594" t="str"/>
@@ -29487,9 +29495,11 @@
       <x:c r="K595" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L595" t="str"/>
+      <x:c r="L595" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/OLY-000000609-olympian-bristlex-stain-brush-4in.png?raw=true</x:v>
+      </x:c>
       <x:c r="M595" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N595" t="str"/>
       <x:c r="O595" t="str"/>
@@ -29532,9 +29542,11 @@
       <x:c r="K596" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L596" t="str"/>
+      <x:c r="L596" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/LEX-000000610-lexel-clear-squeeze-tube.png?raw=true</x:v>
+      </x:c>
       <x:c r="M596" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N596" t="str"/>
       <x:c r="O596" t="str"/>
@@ -29577,9 +29589,11 @@
       <x:c r="K597" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L597" t="str"/>
+      <x:c r="L597" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/LEX-000000611-lexel-clear-sealant.png?raw=true</x:v>
+      </x:c>
       <x:c r="M597" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N597" t="str"/>
       <x:c r="O597" t="str"/>
@@ -29622,9 +29636,11 @@
       <x:c r="K598" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L598" t="str"/>
+      <x:c r="L598" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PI-000000612-pintar-heavy-duty-18in-roller-frame.png?raw=true</x:v>
+      </x:c>
       <x:c r="M598" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N598" t="str"/>
       <x:c r="O598" t="str"/>
@@ -29667,9 +29683,11 @@
       <x:c r="K599" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L599" t="str"/>
+      <x:c r="L599" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PI-000000613-pintar-4l-jumbo-metal-tray.png?raw=true</x:v>
+      </x:c>
       <x:c r="M599" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N599" t="str"/>
       <x:c r="O599" t="str"/>
@@ -29712,9 +29730,11 @@
       <x:c r="K600" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L600" t="str"/>
+      <x:c r="L600" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CAN-000000614-canpro-microfiber-roller-refill.png?raw=true</x:v>
+      </x:c>
       <x:c r="M600" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N600" t="str"/>
       <x:c r="O600" t="str"/>
@@ -29757,9 +29777,11 @@
       <x:c r="K601" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L601" t="str"/>
+      <x:c r="L601" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ALL-000000615-allway-contour-scraper-six-blades.png?raw=true</x:v>
+      </x:c>
       <x:c r="M601" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N601" t="str"/>
       <x:c r="O601" t="str"/>
@@ -29802,9 +29824,11 @@
       <x:c r="K602" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L602" t="str"/>
+      <x:c r="L602" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ALL-000000616-allway-five-gallon-pour-spout.png?raw=true</x:v>
+      </x:c>
       <x:c r="M602" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N602" t="str"/>
       <x:c r="O602" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 337-348
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R6e1ab7fda41949f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rc7447ab7c31a4ebf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -29871,9 +29871,11 @@
       <x:c r="K603" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L603" t="str"/>
+      <x:c r="L603" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AP-000000617-allpro-washi-tape.png?raw=true</x:v>
+      </x:c>
       <x:c r="M603" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N603" t="str"/>
       <x:c r="O603" t="str"/>
@@ -29916,9 +29918,11 @@
       <x:c r="K604" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L604" t="str"/>
+      <x:c r="L604" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AP-000000618-allpro-microfiber-roller-refill-15mm.png?raw=true</x:v>
+      </x:c>
       <x:c r="M604" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N604" t="str"/>
       <x:c r="O604" t="str"/>
@@ -29961,9 +29965,11 @@
       <x:c r="K605" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L605" t="str"/>
+      <x:c r="L605" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PI-000000619-pintar-foam-roller-refill-9-5in.png?raw=true</x:v>
+      </x:c>
       <x:c r="M605" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N605" t="str"/>
       <x:c r="O605" t="str"/>
@@ -30006,9 +30012,11 @@
       <x:c r="K606" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L606" t="str"/>
+      <x:c r="L606" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PI-000000620-pintar-mini-cage-roller-frame.png?raw=true</x:v>
+      </x:c>
       <x:c r="M606" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N606" t="str"/>
       <x:c r="O606" t="str"/>
@@ -30059,9 +30067,11 @@
       <x:c r="K607" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L607" t="str"/>
+      <x:c r="L607" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PI-000000605-pintar-lint-free-roller-refill.png?raw=true</x:v>
+      </x:c>
       <x:c r="M607" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N607" t="str"/>
       <x:c r="O607" t="str"/>
@@ -30112,9 +30122,11 @@
       <x:c r="K608" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L608" t="str"/>
+      <x:c r="L608" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PI-000000622-pintar-stain-paint-brush-4in.png?raw=true</x:v>
+      </x:c>
       <x:c r="M608" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N608" t="str"/>
       <x:c r="O608" t="str"/>
@@ -30157,9 +30169,11 @@
       <x:c r="K609" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L609" t="str"/>
+      <x:c r="L609" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PI-000000623-pintar-stain-brush-3in.png?raw=true</x:v>
+      </x:c>
       <x:c r="M609" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N609" t="str"/>
       <x:c r="O609" t="str"/>
@@ -30202,9 +30216,11 @@
       <x:c r="K610" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L610" t="str"/>
+      <x:c r="L610" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PI-000000613-pintar-4l-jumbo-metal-tray.png?raw=true</x:v>
+      </x:c>
       <x:c r="M610" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N610" t="str"/>
       <x:c r="O610" t="str"/>
@@ -30247,9 +30263,11 @@
       <x:c r="K611" t="str">
         <x:v>PIN02-S</x:v>
       </x:c>
-      <x:c r="L611" t="str"/>
+      <x:c r="L611" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PI-000000625-jumbo-roller-refill.png?raw=true</x:v>
+      </x:c>
       <x:c r="M611" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N611" t="str"/>
       <x:c r="O611" t="str"/>
@@ -30292,9 +30310,11 @@
       <x:c r="K612" t="str">
         <x:v>POL02</x:v>
       </x:c>
-      <x:c r="L612" t="str"/>
+      <x:c r="L612" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/POL-000000628-polytarp-lightweight-plastic-500sqft.png?raw=true</x:v>
+      </x:c>
       <x:c r="M612" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N612" t="str"/>
       <x:c r="O612" t="str"/>
@@ -30337,9 +30357,11 @@
       <x:c r="K613" t="str">
         <x:v>POL02</x:v>
       </x:c>
-      <x:c r="L613" t="str"/>
+      <x:c r="L613" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/POL-000000627-polytarp-plastic-economy-1500sqft.png?raw=true</x:v>
+      </x:c>
       <x:c r="M613" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N613" t="str"/>
       <x:c r="O613" t="str"/>
@@ -30382,9 +30404,11 @@
       <x:c r="K614" t="str">
         <x:v>POL02</x:v>
       </x:c>
-      <x:c r="L614" t="str"/>
+      <x:c r="L614" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/POL-000000628-polytarp-lightweight-plastic-500sqft.png?raw=true</x:v>
+      </x:c>
       <x:c r="M614" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N614" t="str"/>
       <x:c r="O614" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 349-360
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rc7447ab7c31a4ebf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R96707c167b324900"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -30498,9 +30498,11 @@
       <x:c r="K616" t="str">
         <x:v>CANPRO</x:v>
       </x:c>
-      <x:c r="L616" t="str"/>
+      <x:c r="L616" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PRO-000000630-prodec-mini-roller-frame.png?raw=true</x:v>
+      </x:c>
       <x:c r="M616" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N616" t="str"/>
       <x:c r="O616" t="str"/>
@@ -30543,9 +30545,11 @@
       <x:c r="K617" t="str">
         <x:v>CANPRO</x:v>
       </x:c>
-      <x:c r="L617" t="str"/>
+      <x:c r="L617" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PRO-000000631-prodec-ice-fusion-cutting-in-brush-2-5in.png?raw=true</x:v>
+      </x:c>
       <x:c r="M617" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N617" t="str"/>
       <x:c r="O617" t="str"/>
@@ -30588,9 +30592,11 @@
       <x:c r="K618" t="str">
         <x:v>CANPRO</x:v>
       </x:c>
-      <x:c r="L618" t="str"/>
+      <x:c r="L618" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PRO-000000632-prodec-ice-fusion-angle-oval-brush.png?raw=true</x:v>
+      </x:c>
       <x:c r="M618" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N618" t="str"/>
       <x:c r="O618" t="str"/>
@@ -30680,9 +30686,11 @@
       <x:c r="K620" t="str">
         <x:v>CANPRO</x:v>
       </x:c>
-      <x:c r="L620" t="str"/>
+      <x:c r="L620" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PRO-000000634-prodec-saber-extension-pole.png?raw=true</x:v>
+      </x:c>
       <x:c r="M620" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N620" t="str"/>
       <x:c r="O620" t="str"/>
@@ -30725,9 +30733,11 @@
       <x:c r="K621" t="str">
         <x:v>PROTEK</x:v>
       </x:c>
-      <x:c r="L621" t="str"/>
+      <x:c r="L621" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PRO-000000635-waterbased-varnish-zero-gloss.png?raw=true</x:v>
+      </x:c>
       <x:c r="M621" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N621" t="str"/>
       <x:c r="O621" t="str"/>
@@ -30770,9 +30780,11 @@
       <x:c r="K622" t="str">
         <x:v>PROTEK</x:v>
       </x:c>
-      <x:c r="L622" t="str"/>
+      <x:c r="L622" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TEX-000000636-textureline-flat-wax.png?raw=true</x:v>
+      </x:c>
       <x:c r="M622" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N622" t="str"/>
       <x:c r="O622" t="str"/>
@@ -30815,9 +30827,11 @@
       <x:c r="K623" t="str">
         <x:v>PROTEK</x:v>
       </x:c>
-      <x:c r="L623" t="str"/>
+      <x:c r="L623" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TEX-000000637-textureline-venetian-pastel-basecoat.png?raw=true</x:v>
+      </x:c>
       <x:c r="M623" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N623" t="str"/>
       <x:c r="O623" t="str"/>
@@ -30860,9 +30874,11 @@
       <x:c r="K624" t="str">
         <x:v>PROTEK</x:v>
       </x:c>
-      <x:c r="L624" t="str"/>
+      <x:c r="L624" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TEX-000000638-textureline-metaltech-base.png?raw=true</x:v>
+      </x:c>
       <x:c r="M624" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N624" t="str"/>
       <x:c r="O624" t="str"/>
@@ -30905,9 +30921,11 @@
       <x:c r="K625" t="str">
         <x:v>PROTEK</x:v>
       </x:c>
-      <x:c r="L625" t="str"/>
+      <x:c r="L625" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TEX-000000638-textureline-metaltech-base.png?raw=true</x:v>
+      </x:c>
       <x:c r="M625" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N625" t="str"/>
       <x:c r="O625" t="str"/>
@@ -30950,9 +30968,11 @@
       <x:c r="K626" t="str">
         <x:v>PROTEK</x:v>
       </x:c>
-      <x:c r="L626" t="str"/>
+      <x:c r="L626" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TEX-000000638-textureline-metaltech-base.png?raw=true</x:v>
+      </x:c>
       <x:c r="M626" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N626" t="str"/>
       <x:c r="O626" t="str"/>
@@ -30995,9 +31015,11 @@
       <x:c r="K627" t="str">
         <x:v>PROTEK</x:v>
       </x:c>
-      <x:c r="L627" t="str"/>
+      <x:c r="L627" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TEX-000000641-textureline-marmorino-classic.png?raw=true</x:v>
+      </x:c>
       <x:c r="M627" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N627" t="str"/>
       <x:c r="O627" t="str"/>
@@ -31040,9 +31062,11 @@
       <x:c r="K628" t="str">
         <x:v>PROTEK</x:v>
       </x:c>
-      <x:c r="L628" t="str"/>
+      <x:c r="L628" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TEX-000000642-textureline-carolina-sandstone.png?raw=true</x:v>
+      </x:c>
       <x:c r="M628" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N628" t="str"/>
       <x:c r="O628" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 361-372
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R96707c167b324900"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rface0c2ca3ce40aa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -31109,9 +31109,11 @@
       <x:c r="K629" t="str">
         <x:v>PROTEK</x:v>
       </x:c>
-      <x:c r="L629" t="str"/>
+      <x:c r="L629" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TEX-000000643-textureline-burnishing-wax.png?raw=true</x:v>
+      </x:c>
       <x:c r="M629" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N629" t="str"/>
       <x:c r="O629" t="str"/>
@@ -31154,9 +31156,11 @@
       <x:c r="K630" t="str">
         <x:v>PROTEK</x:v>
       </x:c>
-      <x:c r="L630" t="str"/>
+      <x:c r="L630" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TEX-000000637-textureline-venetian-pastel-basecoat.png?raw=true</x:v>
+      </x:c>
       <x:c r="M630" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N630" t="str"/>
       <x:c r="O630" t="str"/>
@@ -31199,9 +31203,11 @@
       <x:c r="K631" t="str">
         <x:v>PROTEK</x:v>
       </x:c>
-      <x:c r="L631" t="str"/>
+      <x:c r="L631" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PRO-000000645-sheffield-red-hot-aluminum.png?raw=true</x:v>
+      </x:c>
       <x:c r="M631" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N631" t="str"/>
       <x:c r="O631" t="str"/>
@@ -31244,9 +31250,11 @@
       <x:c r="K632" t="str">
         <x:v>PROTEK</x:v>
       </x:c>
-      <x:c r="L632" t="str"/>
+      <x:c r="L632" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TEX-000000641-textureline-marmorino-classic.png?raw=true</x:v>
+      </x:c>
       <x:c r="M632" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N632" t="str"/>
       <x:c r="O632" t="str"/>
@@ -31289,9 +31297,11 @@
       <x:c r="K633" t="str">
         <x:v>PROTEK</x:v>
       </x:c>
-      <x:c r="L633" t="str"/>
+      <x:c r="L633" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PRO-000000647-stucco-veneziano-scraper.png?raw=true</x:v>
+      </x:c>
       <x:c r="M633" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N633" t="str"/>
       <x:c r="O633" t="str"/>
@@ -31334,9 +31344,11 @@
       <x:c r="K634" t="str">
         <x:v>PROTEK</x:v>
       </x:c>
-      <x:c r="L634" t="str"/>
+      <x:c r="L634" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PRO-000000648-come-bianko-trowel.png?raw=true</x:v>
+      </x:c>
       <x:c r="M634" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N634" t="str"/>
       <x:c r="O634" t="str"/>
@@ -31379,9 +31391,11 @@
       <x:c r="K635" t="str">
         <x:v>PROTEK</x:v>
       </x:c>
-      <x:c r="L635" t="str"/>
+      <x:c r="L635" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PRO-000000649-come-310lu-trowel.png?raw=true</x:v>
+      </x:c>
       <x:c r="M635" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N635" t="str"/>
       <x:c r="O635" t="str"/>
@@ -31424,9 +31438,11 @@
       <x:c r="K636" t="str">
         <x:v>PROTEK</x:v>
       </x:c>
-      <x:c r="L636" t="str"/>
+      <x:c r="L636" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PC-000000650-stucco-antico-applicators.png?raw=true</x:v>
+      </x:c>
       <x:c r="M636" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N636" t="str"/>
       <x:c r="O636" t="str"/>
@@ -31469,9 +31485,11 @@
       <x:c r="K637" t="str">
         <x:v>PROTEK</x:v>
       </x:c>
-      <x:c r="L637" t="str"/>
+      <x:c r="L637" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PRO-000000651-come-310li-trowel.png?raw=true</x:v>
+      </x:c>
       <x:c r="M637" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N637" t="str"/>
       <x:c r="O637" t="str"/>
@@ -31514,9 +31532,11 @@
       <x:c r="K638" t="str">
         <x:v>DEVIL</x:v>
       </x:c>
-      <x:c r="L638" t="str"/>
+      <x:c r="L638" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RD-000000652-create-a-color-standard-caulk-mixer.png?raw=true</x:v>
+      </x:c>
       <x:c r="M638" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N638" t="str"/>
       <x:c r="O638" t="str"/>
@@ -31559,9 +31579,11 @@
       <x:c r="K639" t="str">
         <x:v>DEVIL</x:v>
       </x:c>
-      <x:c r="L639" t="str"/>
+      <x:c r="L639" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RD-000000653-create-a-color-pro-caulk-mixer.png?raw=true</x:v>
+      </x:c>
       <x:c r="M639" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N639" t="str"/>
       <x:c r="O639" t="str"/>
@@ -31604,9 +31626,11 @@
       <x:c r="K640" t="str">
         <x:v>ROMAN-S</x:v>
       </x:c>
-      <x:c r="L640" t="str"/>
+      <x:c r="L640" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ROM-000000654-roman-pro-880-ultra-clear-gallon.png?raw=true</x:v>
+      </x:c>
       <x:c r="M640" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N640" t="str"/>
       <x:c r="O640" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 373-384
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rface0c2ca3ce40aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rbe8d023d4bc94f46"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -31673,9 +31673,11 @@
       <x:c r="K641" t="str">
         <x:v>ROMAN-S</x:v>
       </x:c>
-      <x:c r="L641" t="str"/>
+      <x:c r="L641" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ROM-000000655-roman-pro-999-rx35-primer.png?raw=true</x:v>
+      </x:c>
       <x:c r="M641" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N641" t="str"/>
       <x:c r="O641" t="str"/>
@@ -31718,9 +31720,11 @@
       <x:c r="K642" t="str">
         <x:v>ROMAN-S</x:v>
       </x:c>
-      <x:c r="L642" t="str"/>
+      <x:c r="L642" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ROM-000000656-roman-pro-977-ultra-prime.png?raw=true</x:v>
+      </x:c>
       <x:c r="M642" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N642" t="str"/>
       <x:c r="O642" t="str"/>
@@ -31763,9 +31767,11 @@
       <x:c r="K643" t="str">
         <x:v>ROMAN-S</x:v>
       </x:c>
-      <x:c r="L643" t="str"/>
+      <x:c r="L643" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ROM-000000657-roman-780-heavy-duty-strippable-clear.png?raw=true</x:v>
+      </x:c>
       <x:c r="M643" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N643" t="str"/>
       <x:c r="O643" t="str"/>
@@ -31808,9 +31814,11 @@
       <x:c r="K644" t="str">
         <x:v>ROMAN-S</x:v>
       </x:c>
-      <x:c r="L644" t="str"/>
+      <x:c r="L644" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ROM-000000658-roman-pro-555-extreme-tack.png?raw=true</x:v>
+      </x:c>
       <x:c r="M644" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N644" t="str"/>
       <x:c r="O644" t="str"/>
@@ -31853,9 +31861,11 @@
       <x:c r="K645" t="str">
         <x:v>ROS01-S</x:v>
       </x:c>
-      <x:c r="L645" t="str"/>
+      <x:c r="L645" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ROS-000000659-rosco-projection-screen-paint.png?raw=true</x:v>
+      </x:c>
       <x:c r="M645" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N645" t="str"/>
       <x:c r="O645" t="str"/>
@@ -31898,9 +31908,11 @@
       <x:c r="K646" t="str">
         <x:v>ROS01-S</x:v>
       </x:c>
-      <x:c r="L646" t="str"/>
+      <x:c r="L646" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ROS-000000660-rosco-chroma-key-green.png?raw=true</x:v>
+      </x:c>
       <x:c r="M646" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N646" t="str"/>
       <x:c r="O646" t="str"/>
@@ -31943,9 +31955,11 @@
       <x:c r="K647" t="str">
         <x:v>ROS01-S</x:v>
       </x:c>
-      <x:c r="L647" t="str"/>
+      <x:c r="L647" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ROS-000000661-rosco-chroma-key-blue.png?raw=true</x:v>
+      </x:c>
       <x:c r="M647" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N647" t="str"/>
       <x:c r="O647" t="str"/>
@@ -32035,9 +32049,11 @@
       <x:c r="K649" t="str">
         <x:v>ROS01-S</x:v>
       </x:c>
-      <x:c r="L649" t="str"/>
+      <x:c r="L649" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ROS-000000663-rosco-tv-black.png?raw=true</x:v>
+      </x:c>
       <x:c r="M649" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N649" t="str"/>
       <x:c r="O649" t="str"/>
@@ -32080,9 +32096,11 @@
       <x:c r="K650" t="str">
         <x:v>ROS01-S</x:v>
       </x:c>
-      <x:c r="L650" t="str"/>
+      <x:c r="L650" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ROS-000000664-roscoflamex-pa.png?raw=true</x:v>
+      </x:c>
       <x:c r="M650" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N650" t="str"/>
       <x:c r="O650" t="str"/>
@@ -32125,9 +32143,11 @@
       <x:c r="K651" t="str">
         <x:v>RBS01</x:v>
       </x:c>
-      <x:c r="L651" t="str"/>
+      <x:c r="L651" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CS-000000665-cgc-sheetrock-90.png?raw=true</x:v>
+      </x:c>
       <x:c r="M651" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N651" t="str"/>
       <x:c r="O651" t="str"/>
@@ -32170,9 +32190,11 @@
       <x:c r="K652" t="str">
         <x:v>RBS01</x:v>
       </x:c>
-      <x:c r="L652" t="str"/>
+      <x:c r="L652" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CS-000000666-cgc-all-purpose-joint-compound-12l.png?raw=true</x:v>
+      </x:c>
       <x:c r="M652" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N652" t="str"/>
       <x:c r="O652" t="str"/>
@@ -32223,9 +32245,11 @@
       <x:c r="K653" t="str">
         <x:v>RBS01</x:v>
       </x:c>
-      <x:c r="L653" t="str"/>
+      <x:c r="L653" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CS-000000667-cgc-dust-control-compound-12l.png?raw=true</x:v>
+      </x:c>
       <x:c r="M653" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N653" t="str"/>
       <x:c r="O653" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 385-396
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rbe8d023d4bc94f46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R4f9b16d6ad3647ec"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -239,7 +239,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
-        <x:v>Type</x:v>
+        <x:v>﻿Type</x:v>
       </x:c>
       <x:c r="B1" t="str">
         <x:v>Name</x:v>
@@ -32292,9 +32292,11 @@
       <x:c r="K654" t="str">
         <x:v>RBS01</x:v>
       </x:c>
-      <x:c r="L654" t="str"/>
+      <x:c r="L654" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CS-000000668-cgc-dust-control-compound-17l.png?raw=true</x:v>
+      </x:c>
       <x:c r="M654" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N654" t="str"/>
       <x:c r="O654" t="str"/>
@@ -32337,9 +32339,11 @@
       <x:c r="K655" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L655" t="str"/>
+      <x:c r="L655" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SK-000000669-seal-krete-clear-seal-satin.png?raw=true</x:v>
+      </x:c>
       <x:c r="M655" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N655" t="str"/>
       <x:c r="O655" t="str"/>
@@ -32429,9 +32433,11 @@
       <x:c r="K657" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L657" t="str"/>
+      <x:c r="L657" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RO-000000671-rust-oleum-self-etching-primer.png?raw=true</x:v>
+      </x:c>
       <x:c r="M657" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N657" t="str"/>
       <x:c r="O657" t="str"/>
@@ -32474,9 +32480,11 @@
       <x:c r="K658" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L658" t="str"/>
+      <x:c r="L658" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RO-000000672-rust-oleum-mirror-effect-silver.png?raw=true</x:v>
+      </x:c>
       <x:c r="M658" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N658" t="str"/>
       <x:c r="O658" t="str"/>
@@ -32519,9 +32527,11 @@
       <x:c r="K659" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L659" t="str"/>
+      <x:c r="L659" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RO-000000673-rust-oleum-metallic-gold.png?raw=true</x:v>
+      </x:c>
       <x:c r="M659" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N659" t="str"/>
       <x:c r="O659" t="str"/>
@@ -32564,9 +32574,11 @@
       <x:c r="K660" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L660" t="str"/>
+      <x:c r="L660" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RO-000000674-rust-oleum-leakseal-clear.png?raw=true</x:v>
+      </x:c>
       <x:c r="M660" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N660" t="str"/>
       <x:c r="O660" t="str"/>
@@ -32609,9 +32621,11 @@
       <x:c r="K661" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L661" t="str"/>
+      <x:c r="L661" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RO-000000675-rust-oleum-leakseal-black.png?raw=true</x:v>
+      </x:c>
       <x:c r="M661" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N661" t="str"/>
       <x:c r="O661" t="str"/>
@@ -32654,9 +32668,11 @@
       <x:c r="K662" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L662" t="str"/>
+      <x:c r="L662" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RO-000000676-rust-oleum-appliance-epoxy-gloss-white.png?raw=true</x:v>
+      </x:c>
       <x:c r="M662" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N662" t="str"/>
       <x:c r="O662" t="str"/>
@@ -32699,9 +32715,11 @@
       <x:c r="K663" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L663" t="str"/>
+      <x:c r="L663" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RO-000000677-rust-oleum-painters-touch-latex-black.png?raw=true</x:v>
+      </x:c>
       <x:c r="M663" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N663" t="str">
         <x:v>Finishes</x:v>
@@ -32752,9 +32770,11 @@
       <x:c r="K664" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L664" t="str"/>
+      <x:c r="L664" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TR-000000678-tremclad-rust-primer-red-oxide.png?raw=true</x:v>
+      </x:c>
       <x:c r="M664" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N664" t="str"/>
       <x:c r="O664" t="str"/>
@@ -32797,9 +32817,11 @@
       <x:c r="K665" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L665" t="str"/>
+      <x:c r="L665" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TR-000000679-tremclad-rust-paint-gloss-white.png?raw=true</x:v>
+      </x:c>
       <x:c r="M665" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N665" t="str"/>
       <x:c r="O665" t="str"/>
@@ -32842,9 +32864,11 @@
       <x:c r="K666" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L666" t="str"/>
+      <x:c r="L666" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/KK-000000680-krud-kutter-original-946ml.png?raw=true</x:v>
+      </x:c>
       <x:c r="M666" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N666" t="str"/>
       <x:c r="O666" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 397-408
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R4f9b16d6ad3647ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R9237b1ad464a482e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -32911,9 +32911,11 @@
       <x:c r="K667" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L667" t="str"/>
+      <x:c r="L667" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/KK-000000681-krud-kutter-oil-grabber.png?raw=true</x:v>
+      </x:c>
       <x:c r="M667" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N667" t="str"/>
       <x:c r="O667" t="str"/>
@@ -32956,9 +32958,11 @@
       <x:c r="K668" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L668" t="str"/>
+      <x:c r="L668" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CON-000000682-concrobium-mold-control-spray.png?raw=true</x:v>
+      </x:c>
       <x:c r="M668" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N668" t="str"/>
       <x:c r="O668" t="str"/>
@@ -33001,9 +33005,11 @@
       <x:c r="K669" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L669" t="str"/>
+      <x:c r="L669" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/RS-000000683-ready-seal-exterior-stain-natural.png?raw=true</x:v>
+      </x:c>
       <x:c r="M669" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N669" t="str"/>
       <x:c r="O669" t="str"/>
@@ -33046,9 +33052,11 @@
       <x:c r="K670" t="str">
         <x:v>SAMAN</x:v>
       </x:c>
-      <x:c r="L670" t="str"/>
+      <x:c r="L670" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SA-000000684-saman-water-based-clear-finish.png?raw=true</x:v>
+      </x:c>
       <x:c r="M670" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N670" t="str"/>
       <x:c r="O670" t="str"/>
@@ -33091,9 +33099,11 @@
       <x:c r="K671" t="str">
         <x:v>SAMAN</x:v>
       </x:c>
-      <x:c r="L671" t="str"/>
+      <x:c r="L671" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SA-000000685-saman-water-based-wood-floor-stain.png?raw=true</x:v>
+      </x:c>
       <x:c r="M671" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N671" t="str"/>
       <x:c r="O671" t="str"/>
@@ -33136,9 +33146,11 @@
       <x:c r="K672" t="str">
         <x:v>SAMAN</x:v>
       </x:c>
-      <x:c r="L672" t="str"/>
+      <x:c r="L672" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SA-000000686-saman-water-based-clear-glaze.png?raw=true</x:v>
+      </x:c>
       <x:c r="M672" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N672" t="str"/>
       <x:c r="O672" t="str"/>
@@ -33181,9 +33193,11 @@
       <x:c r="K673" t="str">
         <x:v>SAMAN</x:v>
       </x:c>
-      <x:c r="L673" t="str"/>
+      <x:c r="L673" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SA-000000687-saman-tung-oil-natural.png?raw=true</x:v>
+      </x:c>
       <x:c r="M673" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N673" t="str"/>
       <x:c r="O673" t="str"/>
@@ -33226,9 +33240,11 @@
       <x:c r="K674" t="str">
         <x:v>SAMAN</x:v>
       </x:c>
-      <x:c r="L674" t="str"/>
+      <x:c r="L674" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SA-000000688-saman-tabletop-epoxy.png?raw=true</x:v>
+      </x:c>
       <x:c r="M674" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N674" t="str"/>
       <x:c r="O674" t="str"/>
@@ -33271,9 +33287,11 @@
       <x:c r="K675" t="str">
         <x:v>SAMAN</x:v>
       </x:c>
-      <x:c r="L675" t="str"/>
+      <x:c r="L675" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SA-000000689-saman-retarder-gallon.png?raw=true</x:v>
+      </x:c>
       <x:c r="M675" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N675" t="str"/>
       <x:c r="O675" t="str"/>
@@ -33316,9 +33334,11 @@
       <x:c r="K676" t="str">
         <x:v>SAMAN</x:v>
       </x:c>
-      <x:c r="L676" t="str"/>
+      <x:c r="L676" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SA-000000690-saman-casting-epoxy-1-5l.png?raw=true</x:v>
+      </x:c>
       <x:c r="M676" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N676" t="str"/>
       <x:c r="O676" t="str"/>
@@ -33361,9 +33381,11 @@
       <x:c r="K677" t="str">
         <x:v>SAMAN</x:v>
       </x:c>
-      <x:c r="L677" t="str"/>
+      <x:c r="L677" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SA-000000691-saman-beeswax-wood-finish.png?raw=true</x:v>
+      </x:c>
       <x:c r="M677" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N677" t="str"/>
       <x:c r="O677" t="str"/>
@@ -33406,9 +33428,11 @@
       <x:c r="K678" t="str">
         <x:v>SAMAN</x:v>
       </x:c>
-      <x:c r="L678" t="str"/>
+      <x:c r="L678" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/CAN-000000692-canpro-tsp-eco-spray.png?raw=true</x:v>
+      </x:c>
       <x:c r="M678" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N678" t="str"/>
       <x:c r="O678" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 409-420
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R9237b1ad464a482e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rabac06a255ca4b34"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -33475,9 +33475,11 @@
       <x:c r="K679" t="str">
         <x:v>TRITON-</x:v>
       </x:c>
-      <x:c r="L679" t="str"/>
+      <x:c r="L679" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SK-000000693-seal-king-strip-all.png?raw=true</x:v>
+      </x:c>
       <x:c r="M679" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N679" t="str"/>
       <x:c r="O679" t="str"/>
@@ -33520,9 +33522,11 @@
       <x:c r="K680" t="str">
         <x:v>TRITON-</x:v>
       </x:c>
-      <x:c r="L680" t="str"/>
+      <x:c r="L680" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SK-000000694-seal-king-seal-grip.png?raw=true</x:v>
+      </x:c>
       <x:c r="M680" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N680" t="str"/>
       <x:c r="O680" t="str"/>
@@ -33565,9 +33569,11 @@
       <x:c r="K681" t="str">
         <x:v>TRITON-</x:v>
       </x:c>
-      <x:c r="L681" t="str"/>
+      <x:c r="L681" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SK-000000695-seal-king-rust-remover.png?raw=true</x:v>
+      </x:c>
       <x:c r="M681" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N681" t="str"/>
       <x:c r="O681" t="str"/>
@@ -33657,9 +33663,11 @@
       <x:c r="K683" t="str">
         <x:v>TRITON-</x:v>
       </x:c>
-      <x:c r="L683" t="str"/>
+      <x:c r="L683" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SK-000000697-seal-king-oil-off.png?raw=true</x:v>
+      </x:c>
       <x:c r="M683" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N683" t="str"/>
       <x:c r="O683" t="str"/>
@@ -33702,9 +33710,11 @@
       <x:c r="K684" t="str">
         <x:v>TRITON-</x:v>
       </x:c>
-      <x:c r="L684" t="str"/>
+      <x:c r="L684" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SK-000000698-seal-king-natural-stone-sealer-natural-look.png?raw=true</x:v>
+      </x:c>
       <x:c r="M684" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N684" t="str"/>
       <x:c r="O684" t="str"/>
@@ -33747,9 +33757,11 @@
       <x:c r="K685" t="str">
         <x:v>TRITON-</x:v>
       </x:c>
-      <x:c r="L685" t="str"/>
+      <x:c r="L685" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SK-000000699-seal-king-natural-stone-sealer-colour-enhancer.png?raw=true</x:v>
+      </x:c>
       <x:c r="M685" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N685" t="str"/>
       <x:c r="O685" t="str"/>
@@ -33792,9 +33804,11 @@
       <x:c r="K686" t="str">
         <x:v>TRITON-</x:v>
       </x:c>
-      <x:c r="L686" t="str"/>
+      <x:c r="L686" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SK-000000700-seal-king-grease-release.png?raw=true</x:v>
+      </x:c>
       <x:c r="M686" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N686" t="str"/>
       <x:c r="O686" t="str"/>
@@ -33837,9 +33851,11 @@
       <x:c r="K687" t="str">
         <x:v>TRITON-</x:v>
       </x:c>
-      <x:c r="L687" t="str"/>
+      <x:c r="L687" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SK-000000701-seal-king-efflorescence-cleaner.png?raw=true</x:v>
+      </x:c>
       <x:c r="M687" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N687" t="str"/>
       <x:c r="O687" t="str"/>
@@ -33882,9 +33898,11 @@
       <x:c r="K688" t="str">
         <x:v>TRITON-</x:v>
       </x:c>
-      <x:c r="L688" t="str"/>
+      <x:c r="L688" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SK-000000702-seal-king-easy-strip.png?raw=true</x:v>
+      </x:c>
       <x:c r="M688" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N688" t="str"/>
       <x:c r="O688" t="str"/>
@@ -33974,9 +33992,11 @@
       <x:c r="K690" t="str">
         <x:v>CANPRO</x:v>
       </x:c>
-      <x:c r="L690" t="str"/>
+      <x:c r="L690" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AP-000000704-allpro-spray-fire-engine-red.png?raw=true</x:v>
+      </x:c>
       <x:c r="M690" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N690" t="str"/>
       <x:c r="O690" t="str"/>
@@ -34066,9 +34086,11 @@
       <x:c r="K692" t="str">
         <x:v>SHURTAP</x:v>
       </x:c>
-      <x:c r="L692" t="str"/>
+      <x:c r="L692" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FT-000000706-frogtape-delicate-surface-1-5in.png?raw=true</x:v>
+      </x:c>
       <x:c r="M692" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N692" t="str"/>
       <x:c r="O692" t="str"/>
@@ -34111,9 +34133,11 @@
       <x:c r="K693" t="str">
         <x:v>SHURTAP</x:v>
       </x:c>
-      <x:c r="L693" t="str"/>
+      <x:c r="L693" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FT-000000707-frogtape-advanced-1-5in.png?raw=true</x:v>
+      </x:c>
       <x:c r="M693" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N693" t="str"/>
       <x:c r="O693" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 421-432
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rabac06a255ca4b34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R63ed23c67707441b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -34180,9 +34180,11 @@
       <x:c r="K694" t="str">
         <x:v>SHURTAP</x:v>
       </x:c>
-      <x:c r="L694" t="str"/>
+      <x:c r="L694" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FT-000000708-frogtape-multi-surface.png?raw=true</x:v>
+      </x:c>
       <x:c r="M694" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N694" t="str"/>
       <x:c r="O694" t="str"/>
@@ -34225,9 +34227,11 @@
       <x:c r="K695" t="str">
         <x:v>SHURTAP</x:v>
       </x:c>
-      <x:c r="L695" t="str"/>
+      <x:c r="L695" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FT-000000709-shurtape-green-masking-tape.png?raw=true</x:v>
+      </x:c>
       <x:c r="M695" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N695" t="str"/>
       <x:c r="O695" t="str"/>
@@ -34270,9 +34274,11 @@
       <x:c r="K696" t="str">
         <x:v>SIA</x:v>
       </x:c>
-      <x:c r="L696" t="str"/>
+      <x:c r="L696" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SIA-000000710-siafast-8-hole-100-grit.png?raw=true</x:v>
+      </x:c>
       <x:c r="M696" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N696" t="str"/>
       <x:c r="O696" t="str"/>
@@ -34315,9 +34321,11 @@
       <x:c r="K697" t="str">
         <x:v>SIA</x:v>
       </x:c>
-      <x:c r="L697" t="str"/>
+      <x:c r="L697" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SIA-000000711-siasoft-roll-100-grit.png?raw=true</x:v>
+      </x:c>
       <x:c r="M697" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N697" t="str"/>
       <x:c r="O697" t="str"/>
@@ -34360,9 +34368,11 @@
       <x:c r="K698" t="str">
         <x:v>PAR03-S</x:v>
       </x:c>
-      <x:c r="L698" t="str"/>
+      <x:c r="L698" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SIK-000000712-sikkens-srd-005-natural-oak.png?raw=true</x:v>
+      </x:c>
       <x:c r="M698" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N698" t="str"/>
       <x:c r="O698" t="str"/>
@@ -34405,9 +34415,11 @@
       <x:c r="K699" t="str">
         <x:v>PAR03-S</x:v>
       </x:c>
-      <x:c r="L699" t="str"/>
+      <x:c r="L699" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SIK-000000713-sikkens-cetol-dek-cedar-077.png?raw=true</x:v>
+      </x:c>
       <x:c r="M699" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N699" t="str"/>
       <x:c r="O699" t="str"/>
@@ -34450,9 +34462,11 @@
       <x:c r="K700" t="str">
         <x:v>PAR03-S</x:v>
       </x:c>
-      <x:c r="L700" t="str"/>
+      <x:c r="L700" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SIK-000000714-cetol-door-window-satin-colorless.png?raw=true</x:v>
+      </x:c>
       <x:c r="M700" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N700" t="str"/>
       <x:c r="O700" t="str"/>
@@ -34495,9 +34509,11 @@
       <x:c r="K701" t="str">
         <x:v>PAR03-S</x:v>
       </x:c>
-      <x:c r="L701" t="str"/>
+      <x:c r="L701" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SIK-000000715-cetol-23-005-natural-oak.png?raw=true</x:v>
+      </x:c>
       <x:c r="M701" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N701" t="str"/>
       <x:c r="O701" t="str"/>
@@ -34540,9 +34556,11 @@
       <x:c r="K702" t="str">
         <x:v>PAR03-S</x:v>
       </x:c>
-      <x:c r="L702" t="str"/>
+      <x:c r="L702" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SIK-000000716-cetol-1-005-natural-oak.png?raw=true</x:v>
+      </x:c>
       <x:c r="M702" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N702" t="str"/>
       <x:c r="O702" t="str"/>
@@ -34585,9 +34603,11 @@
       <x:c r="K703" t="str">
         <x:v>CANPRO</x:v>
       </x:c>
-      <x:c r="L703" t="str"/>
+      <x:c r="L703" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SIM-000000717-smark-dry-erase-clear-200sqft.png?raw=true</x:v>
+      </x:c>
       <x:c r="M703" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N703" t="str"/>
       <x:c r="O703" t="str"/>
@@ -34630,9 +34650,11 @@
       <x:c r="K704" t="str">
         <x:v>UFS01</x:v>
       </x:c>
-      <x:c r="L704" t="str"/>
+      <x:c r="L704" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SIO-000000718-sioux-orbital-sander-velcro.png?raw=true</x:v>
+      </x:c>
       <x:c r="M704" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N704" t="str"/>
       <x:c r="O704" t="str"/>
@@ -34675,9 +34697,11 @@
       <x:c r="K705" t="str">
         <x:v>UFS01</x:v>
       </x:c>
-      <x:c r="L705" t="str"/>
+      <x:c r="L705" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SIO-000000719-sioux-orbital-sander.png?raw=true</x:v>
+      </x:c>
       <x:c r="M705" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N705" t="str"/>
       <x:c r="O705" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 433-444
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R63ed23c67707441b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R4ced5cdbc75f44bd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -34744,9 +34744,11 @@
       <x:c r="K706" t="str">
         <x:v>SUN01-S</x:v>
       </x:c>
-      <x:c r="L706" t="str"/>
+      <x:c r="L706" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SUN-000000720-sunshield-c-tone.png?raw=true</x:v>
+      </x:c>
       <x:c r="M706" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N706" t="str"/>
       <x:c r="O706" t="str"/>
@@ -34789,9 +34791,11 @@
       <x:c r="K707" t="str">
         <x:v>SUN01-S</x:v>
       </x:c>
-      <x:c r="L707" t="str"/>
+      <x:c r="L707" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SUN-000000721-sunshield-clear.png?raw=true</x:v>
+      </x:c>
       <x:c r="M707" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N707" t="str"/>
       <x:c r="O707" t="str"/>
@@ -34834,9 +34838,11 @@
       <x:c r="K708" t="str">
         <x:v>SIMMS</x:v>
       </x:c>
-      <x:c r="L708" t="str"/>
+      <x:c r="L708" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/SIM-000000722-simms-tray-arm.png?raw=true</x:v>
+      </x:c>
       <x:c r="M708" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N708" t="str"/>
       <x:c r="O708" t="str"/>
@@ -34879,9 +34885,11 @@
       <x:c r="K709" t="str">
         <x:v>GOLDLEAF</x:v>
       </x:c>
-      <x:c r="L709" t="str"/>
+      <x:c r="L709" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TGL-000000723-gold-leaf-box-10000.png?raw=true</x:v>
+      </x:c>
       <x:c r="M709" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N709" t="str"/>
       <x:c r="O709" t="str"/>
@@ -34924,9 +34932,11 @@
       <x:c r="K710" t="str">
         <x:v>TIT01-S</x:v>
       </x:c>
-      <x:c r="L710" t="str"/>
+      <x:c r="L710" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TIT-000000724-wagner-furno-heat-gun.png?raw=true</x:v>
+      </x:c>
       <x:c r="M710" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N710" t="str"/>
       <x:c r="O710" t="str"/>
@@ -35063,9 +35073,11 @@
       <x:c r="K713" t="str">
         <x:v>TIT01-S</x:v>
       </x:c>
-      <x:c r="L713" t="str"/>
+      <x:c r="L713" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TIT-000000727-titan-rx80-2-finger.png?raw=true</x:v>
+      </x:c>
       <x:c r="M713" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N713" t="str"/>
       <x:c r="O713" t="str"/>
@@ -35108,9 +35120,11 @@
       <x:c r="K714" t="str">
         <x:v>TIT01-S</x:v>
       </x:c>
-      <x:c r="L714" t="str"/>
+      <x:c r="L714" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TIT-000000728-titan-piston-lube-quart.png?raw=true</x:v>
+      </x:c>
       <x:c r="M714" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N714" t="str"/>
       <x:c r="O714" t="str"/>
@@ -35153,9 +35167,11 @@
       <x:c r="K715" t="str">
         <x:v>TIT01-S</x:v>
       </x:c>
-      <x:c r="L715" t="str"/>
+      <x:c r="L715" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TIT-000000729-titan-piston-lube.png?raw=true</x:v>
+      </x:c>
       <x:c r="M715" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N715" t="str"/>
       <x:c r="O715" t="str"/>
@@ -35292,9 +35308,11 @@
       <x:c r="K718" t="str">
         <x:v>TIT01-S</x:v>
       </x:c>
-      <x:c r="L718" t="str"/>
+      <x:c r="L718" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TIT-000000732-titan-hea-tips.png?raw=true</x:v>
+      </x:c>
       <x:c r="M718" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N718" t="str"/>
       <x:c r="O718" t="str"/>
@@ -35431,9 +35449,11 @@
       <x:c r="K721" t="str">
         <x:v>TIT01-S</x:v>
       </x:c>
-      <x:c r="L721" t="str"/>
+      <x:c r="L721" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TIT-000000735-titan-airless-hose.png?raw=true</x:v>
+      </x:c>
       <x:c r="M721" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N721" t="str"/>
       <x:c r="O721" t="str"/>
@@ -35476,9 +35496,11 @@
       <x:c r="K722" t="str">
         <x:v>TIT01-S</x:v>
       </x:c>
-      <x:c r="L722" t="str"/>
+      <x:c r="L722" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TIT-000000736-titan-hose.png?raw=true</x:v>
+      </x:c>
       <x:c r="M722" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N722" t="str"/>
       <x:c r="O722" t="str"/>
@@ -35568,9 +35590,11 @@
       <x:c r="K724" t="str">
         <x:v>TIT01-S</x:v>
       </x:c>
-      <x:c r="L724" t="str"/>
+      <x:c r="L724" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TIT-000000738-titan-capspray-106.png?raw=true</x:v>
+      </x:c>
       <x:c r="M724" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N724" t="str"/>
       <x:c r="O724" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 445-456
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R4ced5cdbc75f44bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R0e915e7d37384050"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -35637,9 +35637,11 @@
       <x:c r="K725" t="str">
         <x:v>TOO01</x:v>
       </x:c>
-      <x:c r="L725" t="str"/>
+      <x:c r="L725" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TOO-000000739-durapro-premium-contact-cement.png?raw=true</x:v>
+      </x:c>
       <x:c r="M725" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N725" t="str"/>
       <x:c r="O725" t="str"/>
@@ -35682,9 +35684,11 @@
       <x:c r="K726" t="str">
         <x:v>TOO01</x:v>
       </x:c>
-      <x:c r="L726" t="str"/>
+      <x:c r="L726" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/PC-000000740-wire-brush-set.png?raw=true</x:v>
+      </x:c>
       <x:c r="M726" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N726" t="str"/>
       <x:c r="O726" t="str"/>
@@ -35735,9 +35739,11 @@
       <x:c r="K727" t="str">
         <x:v>TOO01</x:v>
       </x:c>
-      <x:c r="L727" t="str"/>
+      <x:c r="L727" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TOO-000000741-twx-neoprene-knee-pads.png?raw=true</x:v>
+      </x:c>
       <x:c r="M727" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N727" t="str"/>
       <x:c r="O727" t="str"/>
@@ -35780,9 +35786,11 @@
       <x:c r="K728" t="str">
         <x:v>TOO01</x:v>
       </x:c>
-      <x:c r="L728" t="str"/>
+      <x:c r="L728" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TOO-000000742-toolway-foam-knee-pads.png?raw=true</x:v>
+      </x:c>
       <x:c r="M728" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N728" t="str"/>
       <x:c r="O728" t="str"/>
@@ -35825,9 +35833,11 @@
       <x:c r="K729" t="str">
         <x:v>TOO01</x:v>
       </x:c>
-      <x:c r="L729" t="str"/>
+      <x:c r="L729" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TOO-000000743-polyfilla-prep.png?raw=true</x:v>
+      </x:c>
       <x:c r="M729" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N729" t="str"/>
       <x:c r="O729" t="str"/>
@@ -35870,9 +35880,11 @@
       <x:c r="K730" t="str">
         <x:v>TOO01</x:v>
       </x:c>
-      <x:c r="L730" t="str"/>
+      <x:c r="L730" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TOO-000000744-plastic-mud-pan.png?raw=true</x:v>
+      </x:c>
       <x:c r="M730" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N730" t="str"/>
       <x:c r="O730" t="str"/>
@@ -35915,9 +35927,11 @@
       <x:c r="K731" t="str">
         <x:v>TOO01</x:v>
       </x:c>
-      <x:c r="L731" t="str"/>
+      <x:c r="L731" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TOO-000000745-pl-premium-construction-adhesive.png?raw=true</x:v>
+      </x:c>
       <x:c r="M731" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N731" t="str"/>
       <x:c r="O731" t="str"/>
@@ -35960,9 +35974,11 @@
       <x:c r="K732" t="str">
         <x:v>TOO01</x:v>
       </x:c>
-      <x:c r="L732" t="str"/>
+      <x:c r="L732" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TOO-000000746-muriatic-acid.png?raw=true</x:v>
+      </x:c>
       <x:c r="M732" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N732" t="str"/>
       <x:c r="O732" t="str"/>
@@ -36005,9 +36021,11 @@
       <x:c r="K733" t="str">
         <x:v>TOO01</x:v>
       </x:c>
-      <x:c r="L733" t="str"/>
+      <x:c r="L733" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TOO-000000747-measuring-wheel.png?raw=true</x:v>
+      </x:c>
       <x:c r="M733" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N733" t="str"/>
       <x:c r="O733" t="str"/>
@@ -36050,9 +36068,11 @@
       <x:c r="K734" t="str">
         <x:v>TOO01</x:v>
       </x:c>
-      <x:c r="L734" t="str"/>
+      <x:c r="L734" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TOO-000000748-instant-polyfilla-tube.png?raw=true</x:v>
+      </x:c>
       <x:c r="M734" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N734" t="str"/>
       <x:c r="O734" t="str"/>
@@ -36095,9 +36115,11 @@
       <x:c r="K735" t="str">
         <x:v>TOO01</x:v>
       </x:c>
-      <x:c r="L735" t="str"/>
+      <x:c r="L735" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TOO-000000749-heavy-duty-angled-broom.png?raw=true</x:v>
+      </x:c>
       <x:c r="M735" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N735" t="str"/>
       <x:c r="O735" t="str"/>
@@ -36140,9 +36162,11 @@
       <x:c r="K736" t="str">
         <x:v>TOO01</x:v>
       </x:c>
-      <x:c r="L736" t="str"/>
+      <x:c r="L736" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TOO-000000750-black-garbage-bags-15pk-3mil.png?raw=true</x:v>
+      </x:c>
       <x:c r="M736" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N736" t="str"/>
       <x:c r="O736" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 457-468
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R0e915e7d37384050"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R49f987b1b2924fb6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -36209,9 +36209,11 @@
       <x:c r="K737" t="str">
         <x:v>TOO01</x:v>
       </x:c>
-      <x:c r="L737" t="str"/>
+      <x:c r="L737" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TOO-000000751-extension-cord-15m-int-ext.png?raw=true</x:v>
+      </x:c>
       <x:c r="M737" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N737" t="str"/>
       <x:c r="O737" t="str"/>
@@ -36254,9 +36256,11 @@
       <x:c r="K738" t="str">
         <x:v>TOWER</x:v>
       </x:c>
-      <x:c r="L738" t="str"/>
+      <x:c r="L738" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AP-000000752-allpro-pro-stretch-caulking-white.png?raw=true</x:v>
+      </x:c>
       <x:c r="M738" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N738" t="str"/>
       <x:c r="O738" t="str"/>
@@ -36346,9 +36350,11 @@
       <x:c r="K740" t="str">
         <x:v>TRIMACO</x:v>
       </x:c>
-      <x:c r="L740" t="str"/>
+      <x:c r="L740" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TRI-000000754-protective-film-for-carpets.png?raw=true</x:v>
+      </x:c>
       <x:c r="M740" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N740" t="str"/>
       <x:c r="O740" t="str"/>
@@ -36391,9 +36397,11 @@
       <x:c r="K741" t="str">
         <x:v>TRIMACO</x:v>
       </x:c>
-      <x:c r="L741" t="str"/>
+      <x:c r="L741" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TRI-000000755-trimaco-90-day-floorsmart-tape.png?raw=true</x:v>
+      </x:c>
       <x:c r="M741" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N741" t="str"/>
       <x:c r="O741" t="str"/>
@@ -36436,9 +36444,11 @@
       <x:c r="K742" t="str">
         <x:v>TRIMACO</x:v>
       </x:c>
-      <x:c r="L742" t="str"/>
+      <x:c r="L742" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TRI-000000756-stay-put-canvas-plus-runner.png?raw=true</x:v>
+      </x:c>
       <x:c r="M742" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N742" t="str"/>
       <x:c r="O742" t="str"/>
@@ -36481,9 +36491,11 @@
       <x:c r="K743" t="str">
         <x:v>TRIMACO</x:v>
       </x:c>
-      <x:c r="L743" t="str"/>
+      <x:c r="L743" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TRI-000000757-protective-film-hard-surfaces.png?raw=true</x:v>
+      </x:c>
       <x:c r="M743" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N743" t="str"/>
       <x:c r="O743" t="str"/>
@@ -36526,9 +36538,11 @@
       <x:c r="K744" t="str">
         <x:v>TRIMACO</x:v>
       </x:c>
-      <x:c r="L744" t="str"/>
+      <x:c r="L744" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TRI-000000758-gallon-nylon-strainer.png?raw=true</x:v>
+      </x:c>
       <x:c r="M744" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N744" t="str"/>
       <x:c r="O744" t="str"/>
@@ -36571,9 +36585,11 @@
       <x:c r="K745" t="str">
         <x:v>TRIMACO</x:v>
       </x:c>
-      <x:c r="L745" t="str"/>
+      <x:c r="L745" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TRI-000000759-floorshell-seam-tape.png?raw=true</x:v>
+      </x:c>
       <x:c r="M745" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N745" t="str"/>
       <x:c r="O745" t="str"/>
@@ -36616,9 +36632,11 @@
       <x:c r="K746" t="str">
         <x:v>TRIMACO</x:v>
       </x:c>
-      <x:c r="L746" t="str"/>
+      <x:c r="L746" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TRI-000000760-easy-mask-tape-n-drape.png?raw=true</x:v>
+      </x:c>
       <x:c r="M746" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N746" t="str"/>
       <x:c r="O746" t="str"/>
@@ -36661,9 +36679,11 @@
       <x:c r="K747" t="str">
         <x:v>TRIMACO</x:v>
       </x:c>
-      <x:c r="L747" t="str"/>
+      <x:c r="L747" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AP-000000761-cone-strainer-allpro.png?raw=true</x:v>
+      </x:c>
       <x:c r="M747" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N747" t="str"/>
       <x:c r="O747" t="str"/>
@@ -36706,9 +36726,11 @@
       <x:c r="K748" t="str">
         <x:v>TRIMACO</x:v>
       </x:c>
-      <x:c r="L748" t="str"/>
+      <x:c r="L748" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TRI-000000762-cone-strainer.png?raw=true</x:v>
+      </x:c>
       <x:c r="M748" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N748" t="str"/>
       <x:c r="O748" t="str"/>
@@ -36751,9 +36773,11 @@
       <x:c r="K749" t="str">
         <x:v>TRIMACO</x:v>
       </x:c>
-      <x:c r="L749" t="str"/>
+      <x:c r="L749" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TRI-000000763-caution-wet-paint.png?raw=true</x:v>
+      </x:c>
       <x:c r="M749" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N749" t="str"/>
       <x:c r="O749" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 469-480
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R49f987b1b2924fb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rac21760342f84b35"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -36820,9 +36820,11 @@
       <x:c r="K750" t="str">
         <x:v>TRIMACO</x:v>
       </x:c>
-      <x:c r="L750" t="str"/>
+      <x:c r="L750" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AP-000000764-allpro-tack-cloth.png?raw=true</x:v>
+      </x:c>
       <x:c r="M750" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N750" t="str"/>
       <x:c r="O750" t="str"/>
@@ -36865,9 +36867,11 @@
       <x:c r="K751" t="str">
         <x:v>TRIMACO</x:v>
       </x:c>
-      <x:c r="L751" t="str"/>
+      <x:c r="L751" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AP-000000765-allpro-spray-sock.png?raw=true</x:v>
+      </x:c>
       <x:c r="M751" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N751" t="str"/>
       <x:c r="O751" t="str"/>
@@ -36910,9 +36914,11 @@
       <x:c r="K752" t="str">
         <x:v>TRIMACO</x:v>
       </x:c>
-      <x:c r="L752" t="str"/>
+      <x:c r="L752" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AP-000000766-allpro-gallon-nylon-strainer.png?raw=true</x:v>
+      </x:c>
       <x:c r="M752" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N752" t="str"/>
       <x:c r="O752" t="str"/>
@@ -36955,9 +36961,11 @@
       <x:c r="K753" t="str">
         <x:v>TRIMACO</x:v>
       </x:c>
-      <x:c r="L753" t="str"/>
+      <x:c r="L753" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/AP-000000767-allpro-5-gallon-nylon-paint-strainer-25pk.png?raw=true</x:v>
+      </x:c>
       <x:c r="M753" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N753" t="str"/>
       <x:c r="O753" t="str"/>
@@ -37000,9 +37008,11 @@
       <x:c r="K754" t="str">
         <x:v>TRIMACO</x:v>
       </x:c>
-      <x:c r="L754" t="str"/>
+      <x:c r="L754" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TRI-000000768-nylon-strainers.png?raw=true</x:v>
+      </x:c>
       <x:c r="M754" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N754" t="str"/>
       <x:c r="O754" t="str"/>
@@ -37045,9 +37055,11 @@
       <x:c r="K755" t="str">
         <x:v>TRIMACO</x:v>
       </x:c>
-      <x:c r="L755" t="str"/>
+      <x:c r="L755" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TRI-000000769-trimaco-12-inch-masking-paper.png?raw=true</x:v>
+      </x:c>
       <x:c r="M755" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N755" t="str"/>
       <x:c r="O755" t="str"/>
@@ -37090,9 +37102,11 @@
       <x:c r="K756" t="str">
         <x:v>TRITECH</x:v>
       </x:c>
-      <x:c r="L756" t="str"/>
+      <x:c r="L756" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TRI-000000770-tritech-t93r-ultra-finish-tip-408.png?raw=true</x:v>
+      </x:c>
       <x:c r="M756" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N756" t="str"/>
       <x:c r="O756" t="str"/>
@@ -37135,9 +37149,11 @@
       <x:c r="K757" t="str">
         <x:v>TRITECH</x:v>
       </x:c>
-      <x:c r="L757" t="str"/>
+      <x:c r="L757" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TRI-000000771-tritech-t93r-contractor-tip-415.png?raw=true</x:v>
+      </x:c>
       <x:c r="M757" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N757" t="str"/>
       <x:c r="O757" t="str"/>
@@ -37180,9 +37196,11 @@
       <x:c r="K758" t="str">
         <x:v>TRITECH</x:v>
       </x:c>
-      <x:c r="L758" t="str"/>
+      <x:c r="L758" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TRI-000000772-tritech-t9-hi-cart-110v.png?raw=true</x:v>
+      </x:c>
       <x:c r="M758" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N758" t="str"/>
       <x:c r="O758" t="str"/>
@@ -37225,9 +37243,11 @@
       <x:c r="K759" t="str">
         <x:v>TRITECH</x:v>
       </x:c>
-      <x:c r="L759" t="str"/>
+      <x:c r="L759" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/TRI-000000773-tritech-t4-110v-stand.png?raw=true</x:v>
+      </x:c>
       <x:c r="M759" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N759" t="str"/>
       <x:c r="O759" t="str"/>
@@ -37270,9 +37290,11 @@
       <x:c r="K760" t="str">
         <x:v>VCI01</x:v>
       </x:c>
-      <x:c r="L760" t="str"/>
+      <x:c r="L760" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/VC-000000774-satin-finish-cleaner-stainless-steel.png?raw=true</x:v>
+      </x:c>
       <x:c r="M760" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N760" t="str"/>
       <x:c r="O760" t="str"/>
@@ -37315,9 +37337,11 @@
       <x:c r="K761" t="str">
         <x:v>VCI01</x:v>
       </x:c>
-      <x:c r="L761" t="str"/>
+      <x:c r="L761" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/VC-000000775-grease-buster-concentrate-cleaner.png?raw=true</x:v>
+      </x:c>
       <x:c r="M761" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N761" t="str"/>
       <x:c r="O761" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 481-492
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rac21760342f84b35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R9925ea1318964550"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -37384,9 +37384,11 @@
       <x:c r="K762" t="str">
         <x:v>VCI01</x:v>
       </x:c>
-      <x:c r="L762" t="str"/>
+      <x:c r="L762" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/VC-000000776-crete-clean-concrete-etching-clean.png?raw=true</x:v>
+      </x:c>
       <x:c r="M762" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N762" t="str"/>
       <x:c r="O762" t="str"/>
@@ -37429,9 +37431,11 @@
       <x:c r="K763" t="str">
         <x:v>VCI01</x:v>
       </x:c>
-      <x:c r="L763" t="str"/>
+      <x:c r="L763" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/VC-000000777-acoustical-tile-restorer.png?raw=true</x:v>
+      </x:c>
       <x:c r="M763" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N763" t="str"/>
       <x:c r="O763" t="str"/>
@@ -37474,9 +37478,11 @@
       <x:c r="K764" t="str">
         <x:v>VIC</x:v>
       </x:c>
-      <x:c r="L764" t="str"/>
+      <x:c r="L764" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/VS-000000778-green-rubber-gloves-sol-vex-large.png?raw=true</x:v>
+      </x:c>
       <x:c r="M764" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N764" t="str"/>
       <x:c r="O764" t="str"/>
@@ -37519,9 +37525,11 @@
       <x:c r="K765" t="str">
         <x:v>VIC</x:v>
       </x:c>
-      <x:c r="L765" t="str"/>
+      <x:c r="L765" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/VS-000000779-foot-slip-covers-5-pairs.png?raw=true</x:v>
+      </x:c>
       <x:c r="M765" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N765" t="str"/>
       <x:c r="O765" t="str"/>
@@ -37564,9 +37572,11 @@
       <x:c r="K766" t="str">
         <x:v>VIC</x:v>
       </x:c>
-      <x:c r="L766" t="str"/>
+      <x:c r="L766" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/VS-000000780-blackshield-black-nitrile-medium.png?raw=true</x:v>
+      </x:c>
       <x:c r="M766" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N766" t="str"/>
       <x:c r="O766" t="str"/>
@@ -37609,9 +37619,11 @@
       <x:c r="K767" t="str">
         <x:v>VIC</x:v>
       </x:c>
-      <x:c r="L767" t="str"/>
+      <x:c r="L767" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/VS-000000781-black-nitrile-8-mil-gloves-large-50-box.png?raw=true</x:v>
+      </x:c>
       <x:c r="M767" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N767" t="str"/>
       <x:c r="O767" t="str"/>
@@ -37654,9 +37666,11 @@
       <x:c r="K768" t="str">
         <x:v>WALLS</x:v>
       </x:c>
-      <x:c r="L768" t="str"/>
+      <x:c r="L768" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/REN-000000782-renner-exterior-uv-water-based-varnish-matte.png?raw=true</x:v>
+      </x:c>
       <x:c r="M768" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N768" t="str"/>
       <x:c r="O768" t="str"/>
@@ -37699,9 +37713,11 @@
       <x:c r="K769" t="str">
         <x:v>CANPRO</x:v>
       </x:c>
-      <x:c r="L769" t="str"/>
+      <x:c r="L769" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/WAR-000000783-warner-adjustable-spray-shield.png?raw=true</x:v>
+      </x:c>
       <x:c r="M769" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N769" t="str"/>
       <x:c r="O769" t="str"/>
@@ -37744,9 +37760,11 @@
       <x:c r="K770" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L770" t="str"/>
+      <x:c r="L770" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/WAT-000000784-watco-danish-oil-dark-walnut.png?raw=true</x:v>
+      </x:c>
       <x:c r="M770" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N770" t="str"/>
       <x:c r="O770" t="str"/>
@@ -37789,9 +37807,11 @@
       <x:c r="K771" t="str">
         <x:v>WIPECO</x:v>
       </x:c>
-      <x:c r="L771" t="str"/>
+      <x:c r="L771" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/WIP-000000785-workeze-coverall-large.png?raw=true</x:v>
+      </x:c>
       <x:c r="M771" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N771" t="str"/>
       <x:c r="O771" t="str"/>
@@ -37834,9 +37854,11 @@
       <x:c r="K772" t="str">
         <x:v>WIPECO</x:v>
       </x:c>
-      <x:c r="L772" t="str"/>
+      <x:c r="L772" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/WIP-000000786-wipeco-painters-glove-large.png?raw=true</x:v>
+      </x:c>
       <x:c r="M772" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N772" t="str"/>
       <x:c r="O772" t="str"/>
@@ -37879,9 +37901,11 @@
       <x:c r="K773" t="str">
         <x:v>WIPECO</x:v>
       </x:c>
-      <x:c r="L773" t="str"/>
+      <x:c r="L773" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/WIP-000000787-stainpro-stain-pad.png?raw=true</x:v>
+      </x:c>
       <x:c r="M773" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N773" t="str"/>
       <x:c r="O773" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 493-504
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R9925ea1318964550"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rc98a42b1a3424941"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -37948,9 +37948,11 @@
       <x:c r="K774" t="str">
         <x:v>WIPECO</x:v>
       </x:c>
-      <x:c r="L774" t="str"/>
+      <x:c r="L774" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/WIP-000000788-stainpro-leak-proof-drop-cloth.png?raw=true</x:v>
+      </x:c>
       <x:c r="M774" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N774" t="str"/>
       <x:c r="O774" t="str"/>
@@ -37993,9 +37995,11 @@
       <x:c r="K775" t="str">
         <x:v>WOOSTER</x:v>
       </x:c>
-      <x:c r="L775" t="str"/>
+      <x:c r="L775" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/WBC-000000789-wooster-super-fab-roller-cover-4-5-x-3-8-2pk.png?raw=true</x:v>
+      </x:c>
       <x:c r="M775" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N775" t="str"/>
       <x:c r="O775" t="str"/>
@@ -38132,9 +38136,11 @@
       <x:c r="K778" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L778" t="str"/>
+      <x:c r="L778" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/WBC-000000792-wooster-sherlock-roller-frame-9-5.png?raw=true</x:v>
+      </x:c>
       <x:c r="M778" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N778" t="str"/>
       <x:c r="O778" t="str"/>
@@ -38177,9 +38183,11 @@
       <x:c r="K779" t="str">
         <x:v>WOOSTER</x:v>
       </x:c>
-      <x:c r="L779" t="str"/>
+      <x:c r="L779" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/WBC-000000793-wooster-pro-doo-z-roller-cover-6-5-x-3-8-2pk.png?raw=true</x:v>
+      </x:c>
       <x:c r="M779" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N779" t="str"/>
       <x:c r="O779" t="str"/>
@@ -38222,9 +38230,11 @@
       <x:c r="K780" t="str">
         <x:v>WOOSTER</x:v>
       </x:c>
-      <x:c r="L780" t="str"/>
+      <x:c r="L780" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/WBC-000000794-wooster-mohair-blend-roller-cover-14-x-1-4.png?raw=true</x:v>
+      </x:c>
       <x:c r="M780" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Images for Review</x:v>
       </x:c>
       <x:c r="N780" t="str"/>
       <x:c r="O780" t="str"/>
@@ -38267,9 +38277,11 @@
       <x:c r="K781" t="str">
         <x:v>WOOSTER</x:v>
       </x:c>
-      <x:c r="L781" t="str"/>
+      <x:c r="L781" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/WBC-000000795-wooster-jumbo-koter-big-green-flocked-foam-roller.png?raw=true</x:v>
+      </x:c>
       <x:c r="M781" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N781" t="str"/>
       <x:c r="O781" t="str"/>
@@ -38312,9 +38324,11 @@
       <x:c r="K782" t="str">
         <x:v>MUM01</x:v>
       </x:c>
-      <x:c r="L782" t="str"/>
+      <x:c r="L782" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/WBC-000000796-wooster-jumbo-koter-14-inch-roller-frame.png?raw=true</x:v>
+      </x:c>
       <x:c r="M782" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N782" t="str"/>
       <x:c r="O782" t="str"/>
@@ -38357,9 +38371,11 @@
       <x:c r="K783" t="str">
         <x:v>WOOSTER</x:v>
       </x:c>
-      <x:c r="L783" t="str"/>
+      <x:c r="L783" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/WBC-000000797-wooster-jumbo-koter-microfiber-4-5-x-3-8-2pk.png?raw=true</x:v>
+      </x:c>
       <x:c r="M783" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N783" t="str"/>
       <x:c r="O783" t="str"/>
@@ -38449,9 +38465,11 @@
       <x:c r="K785" t="str">
         <x:v>WOOSTER</x:v>
       </x:c>
-      <x:c r="L785" t="str"/>
+      <x:c r="L785" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/WBC-000000799-wooster-wide-boy-5-gallon-bucket.png?raw=true</x:v>
+      </x:c>
       <x:c r="M785" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N785" t="str"/>
       <x:c r="O785" t="str"/>
@@ -38494,9 +38512,11 @@
       <x:c r="K786" t="str">
         <x:v>WOOSTER</x:v>
       </x:c>
-      <x:c r="L786" t="str"/>
+      <x:c r="L786" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/WO-000000800-wooster-sherlock-extension-pole-4-8-ft.png?raw=true</x:v>
+      </x:c>
       <x:c r="M786" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N786" t="str"/>
       <x:c r="O786" t="str"/>
@@ -38586,9 +38606,11 @@
       <x:c r="K788" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L788" t="str"/>
+      <x:c r="L788" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/XIM-000000802-xim-uma-acrylic-primer.png?raw=true</x:v>
+      </x:c>
       <x:c r="M788" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N788" t="str"/>
       <x:c r="O788" t="str"/>
@@ -38631,9 +38653,11 @@
       <x:c r="K789" t="str">
         <x:v>YHD01</x:v>
       </x:c>
-      <x:c r="L789" t="str"/>
+      <x:c r="L789" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/HOW-000000803-howard-restor-a-finish-walnut.png?raw=true</x:v>
+      </x:c>
       <x:c r="M789" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N789" t="str"/>
       <x:c r="O789" t="str"/>

</xml_diff>

<commit_message>
Add reviewed product images 505-512
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_working.xlsx
+++ b/products_categories_descriptions_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rc98a42b1a3424941"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R156bd360883e421d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -38700,9 +38700,11 @@
       <x:c r="K790" t="str">
         <x:v>YHD01</x:v>
       </x:c>
-      <x:c r="L790" t="str"/>
+      <x:c r="L790" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/FLO-000000804-floetrol-gallon-flood.png?raw=true</x:v>
+      </x:c>
       <x:c r="M790" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N790" t="str"/>
       <x:c r="O790" t="str"/>
@@ -38745,9 +38747,11 @@
       <x:c r="K791" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L791" t="str"/>
+      <x:c r="L791" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ZI-000000805-zinsser-odor-killing-primer.png?raw=true</x:v>
+      </x:c>
       <x:c r="M791" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N791" t="str"/>
       <x:c r="O791" t="str"/>
@@ -38900,9 +38904,11 @@
       <x:c r="K794" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L794" t="str"/>
+      <x:c r="L794" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ZI-000000808-zinsser-watertite-hydraulic-cement.png?raw=true</x:v>
+      </x:c>
       <x:c r="M794" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N794" t="str"/>
       <x:c r="O794" t="str"/>
@@ -38945,9 +38951,11 @@
       <x:c r="K795" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L795" t="str"/>
+      <x:c r="L795" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ZI-000000809-zinsser-shieldz-universal-wallcovering-primer.png?raw=true</x:v>
+      </x:c>
       <x:c r="M795" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N795" t="str"/>
       <x:c r="O795" t="str"/>
@@ -38990,9 +38998,11 @@
       <x:c r="K796" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L796" t="str"/>
+      <x:c r="L796" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ZI-000000810-zinsser-peel-stop-plus-high-build-binding-primer.png?raw=true</x:v>
+      </x:c>
       <x:c r="M796" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N796" t="str"/>
       <x:c r="O796" t="str"/>
@@ -39035,9 +39045,11 @@
       <x:c r="K797" t="str">
         <x:v>FLE01-S</x:v>
       </x:c>
-      <x:c r="L797" t="str"/>
+      <x:c r="L797" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ZI-000000811-zinsser-dif-wallpaper-stripper-gel.png?raw=true</x:v>
+      </x:c>
       <x:c r="M797" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N797" t="str"/>
       <x:c r="O797" t="str"/>
@@ -39080,9 +39092,11 @@
       <x:c r="K798" t="str">
         <x:v>ZIPWALL</x:v>
       </x:c>
-      <x:c r="L798" t="str"/>
+      <x:c r="L798" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ZIP-000000812-zipwall-zippole10.png?raw=true</x:v>
+      </x:c>
       <x:c r="M798" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N798" t="str"/>
       <x:c r="O798" t="str"/>
@@ -39125,9 +39139,11 @@
       <x:c r="K799" t="str">
         <x:v>ZIPWALL</x:v>
       </x:c>
-      <x:c r="L799" t="str"/>
+      <x:c r="L799" t="str">
+        <x:v>https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/review-images/ZIP-000000813-zipwall-heavy-duty-zipper-package-front.png?raw=true</x:v>
+      </x:c>
       <x:c r="M799" t="str">
-        <x:v>No Qualifying Image</x:v>
+        <x:v>Image Added</x:v>
       </x:c>
       <x:c r="N799" t="str"/>
       <x:c r="O799" t="str"/>

</xml_diff>